<commit_message>
093 Week 2/3 data update
</commit_message>
<xml_diff>
--- a/data/SUMMER_GOLF_2026.xlsx
+++ b/data/SUMMER_GOLF_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="79">
   <si>
     <t>SUMMER GOLF 2026 - THURSDAY SINGLES</t>
   </si>
@@ -237,6 +237,9 @@
   </si>
   <si>
     <t>WILL VINE</t>
+  </si>
+  <si>
+    <t>JOHN ANTCLIFFE/PAUL HANCOX</t>
   </si>
   <si>
     <t>SUNDAY</t>
@@ -929,7 +932,9 @@
       <c r="C5" s="13">
         <v>29.0</v>
       </c>
-      <c r="D5" s="14"/>
+      <c r="D5" s="14">
+        <v>30.0</v>
+      </c>
       <c r="E5" s="13"/>
       <c r="F5" s="14"/>
       <c r="G5" s="13"/>
@@ -954,7 +959,7 @@
       <c r="Z5" s="17"/>
       <c r="AA5" s="15">
         <f t="shared" ref="AA5:AA19" si="1">sum(C5:Z5)</f>
-        <v>29</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -964,7 +969,9 @@
       <c r="C6" s="13">
         <v>34.0</v>
       </c>
-      <c r="D6" s="14"/>
+      <c r="D6" s="14">
+        <v>33.0</v>
+      </c>
       <c r="E6" s="13"/>
       <c r="F6" s="14"/>
       <c r="G6" s="13"/>
@@ -989,7 +996,7 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>34</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7">
@@ -997,7 +1004,9 @@
         <v>32</v>
       </c>
       <c r="C7" s="13"/>
-      <c r="D7" s="14"/>
+      <c r="D7" s="14">
+        <v>28.0</v>
+      </c>
       <c r="E7" s="13"/>
       <c r="F7" s="14"/>
       <c r="G7" s="13"/>
@@ -1022,7 +1031,7 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -1032,7 +1041,9 @@
       <c r="C8" s="13">
         <v>36.0</v>
       </c>
-      <c r="D8" s="14"/>
+      <c r="D8" s="14">
+        <v>34.0</v>
+      </c>
       <c r="E8" s="13"/>
       <c r="F8" s="14"/>
       <c r="G8" s="13"/>
@@ -1057,7 +1068,7 @@
       <c r="Z8" s="19"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>36</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9">
@@ -1067,7 +1078,9 @@
       <c r="C9" s="13">
         <v>30.0</v>
       </c>
-      <c r="D9" s="14"/>
+      <c r="D9" s="14">
+        <v>34.0</v>
+      </c>
       <c r="E9" s="13"/>
       <c r="F9" s="14"/>
       <c r="G9" s="13"/>
@@ -1092,7 +1105,7 @@
       <c r="Z9" s="17"/>
       <c r="AA9" s="15">
         <f t="shared" si="1"/>
-        <v>30</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10">
@@ -1102,7 +1115,9 @@
       <c r="C10" s="13">
         <v>32.0</v>
       </c>
-      <c r="D10" s="14"/>
+      <c r="D10" s="14">
+        <v>34.0</v>
+      </c>
       <c r="E10" s="13"/>
       <c r="F10" s="15"/>
       <c r="G10" s="13"/>
@@ -1127,7 +1142,7 @@
       <c r="Z10" s="17"/>
       <c r="AA10" s="15">
         <f t="shared" si="1"/>
-        <v>32</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11">
@@ -1137,7 +1152,9 @@
       <c r="C11" s="13">
         <v>39.0</v>
       </c>
-      <c r="D11" s="14"/>
+      <c r="D11" s="14">
+        <v>30.0</v>
+      </c>
       <c r="E11" s="13"/>
       <c r="F11" s="14"/>
       <c r="G11" s="13"/>
@@ -1162,7 +1179,7 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>39</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12">
@@ -1205,7 +1222,9 @@
       <c r="C13" s="13">
         <v>28.0</v>
       </c>
-      <c r="D13" s="14"/>
+      <c r="D13" s="14">
+        <v>29.0</v>
+      </c>
       <c r="E13" s="13"/>
       <c r="F13" s="14"/>
       <c r="G13" s="13"/>
@@ -1230,7 +1249,7 @@
       <c r="Z13" s="17"/>
       <c r="AA13" s="15">
         <f t="shared" si="1"/>
-        <v>28</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14">
@@ -1240,7 +1259,9 @@
       <c r="C14" s="13">
         <v>30.0</v>
       </c>
-      <c r="D14" s="14"/>
+      <c r="D14" s="14">
+        <v>31.0</v>
+      </c>
       <c r="E14" s="16"/>
       <c r="F14" s="14"/>
       <c r="G14" s="13"/>
@@ -1265,7 +1286,7 @@
       <c r="Z14" s="17"/>
       <c r="AA14" s="15">
         <f t="shared" si="1"/>
-        <v>30</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15">
@@ -1273,7 +1294,9 @@
         <v>40</v>
       </c>
       <c r="C15" s="13"/>
-      <c r="D15" s="14"/>
+      <c r="D15" s="14">
+        <v>28.0</v>
+      </c>
       <c r="E15" s="13"/>
       <c r="F15" s="14"/>
       <c r="G15" s="13"/>
@@ -1298,7 +1321,7 @@
       <c r="Z15" s="17"/>
       <c r="AA15" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16">
@@ -1374,7 +1397,9 @@
       <c r="C18" s="17">
         <v>23.0</v>
       </c>
-      <c r="D18" s="14"/>
+      <c r="D18" s="14">
+        <v>21.0</v>
+      </c>
       <c r="E18" s="13"/>
       <c r="F18" s="14"/>
       <c r="G18" s="13"/>
@@ -1399,7 +1424,7 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>23</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19">
@@ -1468,7 +1493,9 @@
       <c r="C21" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="24"/>
+      <c r="D21" s="24" t="s">
+        <v>34</v>
+      </c>
       <c r="E21" s="24"/>
       <c r="F21" s="24"/>
       <c r="G21" s="24"/>
@@ -1500,7 +1527,9 @@
       <c r="C22" s="27">
         <v>39.0</v>
       </c>
-      <c r="D22" s="27"/>
+      <c r="D22" s="27">
+        <v>34.0</v>
+      </c>
       <c r="E22" s="27"/>
       <c r="F22" s="27"/>
       <c r="G22" s="27"/>
@@ -1707,7 +1736,9 @@
         <v>28.0</v>
       </c>
       <c r="D6" s="14"/>
-      <c r="E6" s="13"/>
+      <c r="E6" s="13">
+        <v>31.0</v>
+      </c>
       <c r="F6" s="14"/>
       <c r="G6" s="13"/>
       <c r="H6" s="14"/>
@@ -1731,7 +1762,7 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>28</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
@@ -1744,7 +1775,9 @@
       <c r="D7" s="14">
         <v>28.0</v>
       </c>
-      <c r="E7" s="13"/>
+      <c r="E7" s="13">
+        <v>30.0</v>
+      </c>
       <c r="F7" s="14"/>
       <c r="G7" s="13"/>
       <c r="H7" s="14"/>
@@ -1768,7 +1801,7 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>52</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8">
@@ -1781,7 +1814,9 @@
       <c r="D8" s="14">
         <v>24.0</v>
       </c>
-      <c r="E8" s="13"/>
+      <c r="E8" s="13">
+        <v>26.0</v>
+      </c>
       <c r="F8" s="14"/>
       <c r="G8" s="13"/>
       <c r="H8" s="14"/>
@@ -1805,7 +1840,7 @@
       <c r="Z8" s="17"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9">
@@ -1816,7 +1851,9 @@
         <v>24.0</v>
       </c>
       <c r="D9" s="14"/>
-      <c r="E9" s="13"/>
+      <c r="E9" s="13">
+        <v>29.0</v>
+      </c>
       <c r="F9" s="14"/>
       <c r="G9" s="13"/>
       <c r="H9" s="14"/>
@@ -1840,7 +1877,7 @@
       <c r="Z9" s="17"/>
       <c r="AA9" s="15">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10">
@@ -1884,7 +1921,9 @@
       <c r="D11" s="14">
         <v>33.0</v>
       </c>
-      <c r="E11" s="13"/>
+      <c r="E11" s="13">
+        <v>34.0</v>
+      </c>
       <c r="F11" s="14"/>
       <c r="G11" s="13"/>
       <c r="H11" s="15"/>
@@ -1908,7 +1947,7 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>33</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12">
@@ -2061,7 +2100,9 @@
       <c r="D16" s="14">
         <v>27.0</v>
       </c>
-      <c r="E16" s="13"/>
+      <c r="E16" s="13">
+        <v>37.0</v>
+      </c>
       <c r="F16" s="14"/>
       <c r="G16" s="13"/>
       <c r="H16" s="14"/>
@@ -2085,7 +2126,7 @@
       <c r="Z16" s="17"/>
       <c r="AA16" s="15">
         <f t="shared" si="1"/>
-        <v>27</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17">
@@ -2098,7 +2139,9 @@
       <c r="D17" s="14">
         <v>19.0</v>
       </c>
-      <c r="E17" s="13"/>
+      <c r="E17" s="13">
+        <v>26.0</v>
+      </c>
       <c r="F17" s="14"/>
       <c r="G17" s="13"/>
       <c r="H17" s="14"/>
@@ -2122,7 +2165,7 @@
       <c r="Z17" s="17"/>
       <c r="AA17" s="15">
         <f t="shared" si="1"/>
-        <v>39</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18">
@@ -2133,7 +2176,9 @@
         <v>32.0</v>
       </c>
       <c r="D18" s="14"/>
-      <c r="E18" s="13"/>
+      <c r="E18" s="13">
+        <v>32.0</v>
+      </c>
       <c r="F18" s="14"/>
       <c r="G18" s="13"/>
       <c r="H18" s="14"/>
@@ -2157,7 +2202,7 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>32</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19">
@@ -2170,7 +2215,9 @@
       <c r="D19" s="14">
         <v>30.0</v>
       </c>
-      <c r="E19" s="13"/>
+      <c r="E19" s="13">
+        <v>26.0</v>
+      </c>
       <c r="F19" s="14"/>
       <c r="G19" s="13"/>
       <c r="H19" s="14"/>
@@ -2194,7 +2241,7 @@
       <c r="Z19" s="17"/>
       <c r="AA19" s="15">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20">
@@ -2205,7 +2252,9 @@
         <v>28.0</v>
       </c>
       <c r="D20" s="14"/>
-      <c r="E20" s="13"/>
+      <c r="E20" s="13">
+        <v>30.0</v>
+      </c>
       <c r="F20" s="15"/>
       <c r="G20" s="13"/>
       <c r="H20" s="14"/>
@@ -2229,7 +2278,7 @@
       <c r="Z20" s="17"/>
       <c r="AA20" s="15">
         <f t="shared" si="1"/>
-        <v>28</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21">
@@ -2275,7 +2324,9 @@
       <c r="D22" s="14">
         <v>39.0</v>
       </c>
-      <c r="E22" s="13"/>
+      <c r="E22" s="13">
+        <v>27.0</v>
+      </c>
       <c r="F22" s="15"/>
       <c r="G22" s="13"/>
       <c r="H22" s="14"/>
@@ -2299,7 +2350,7 @@
       <c r="Z22" s="17"/>
       <c r="AA22" s="15">
         <f t="shared" si="1"/>
-        <v>59</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23">
@@ -2308,7 +2359,9 @@
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="14"/>
-      <c r="E23" s="13"/>
+      <c r="E23" s="13">
+        <v>34.0</v>
+      </c>
       <c r="F23" s="15"/>
       <c r="G23" s="13"/>
       <c r="H23" s="14"/>
@@ -2332,7 +2385,7 @@
       <c r="Z23" s="17"/>
       <c r="AA23" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24">
@@ -2380,7 +2433,9 @@
       <c r="D25" s="14">
         <v>25.0</v>
       </c>
-      <c r="E25" s="13"/>
+      <c r="E25" s="13">
+        <v>33.0</v>
+      </c>
       <c r="F25" s="15"/>
       <c r="G25" s="13"/>
       <c r="H25" s="14"/>
@@ -2404,7 +2459,7 @@
       <c r="Z25" s="17"/>
       <c r="AA25" s="15">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>93</v>
       </c>
     </row>
     <row r="26">
@@ -2415,7 +2470,9 @@
         <v>19.0</v>
       </c>
       <c r="D26" s="14"/>
-      <c r="E26" s="13"/>
+      <c r="E26" s="13">
+        <v>29.0</v>
+      </c>
       <c r="F26" s="15"/>
       <c r="G26" s="13"/>
       <c r="H26" s="14"/>
@@ -2439,7 +2496,7 @@
       <c r="Z26" s="17"/>
       <c r="AA26" s="15">
         <f t="shared" si="1"/>
-        <v>19</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" ht="9.0" customHeight="1">
@@ -2478,7 +2535,9 @@
       <c r="D28" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E28" s="24"/>
+      <c r="E28" s="24" t="s">
+        <v>34</v>
+      </c>
       <c r="F28" s="24"/>
       <c r="G28" s="24"/>
       <c r="H28" s="24"/>
@@ -2512,7 +2571,9 @@
       <c r="D29" s="27">
         <v>39.0</v>
       </c>
-      <c r="E29" s="27"/>
+      <c r="E29" s="27">
+        <v>37.0</v>
+      </c>
       <c r="F29" s="27"/>
       <c r="G29" s="27"/>
       <c r="H29" s="27"/>
@@ -2569,10 +2630,10 @@
         <v>43</v>
       </c>
       <c r="B2" s="33">
+        <v>15.0</v>
+      </c>
+      <c r="C2" s="34">
         <v>14.0</v>
-      </c>
-      <c r="C2" s="34">
-        <v>13.0</v>
       </c>
     </row>
     <row r="3">
@@ -2591,10 +2652,10 @@
         <v>64</v>
       </c>
       <c r="B4" s="33">
+        <v>9.0</v>
+      </c>
+      <c r="C4" s="34">
         <v>8.0</v>
-      </c>
-      <c r="C4" s="34">
-        <v>7.0</v>
       </c>
     </row>
     <row r="5">
@@ -2624,7 +2685,7 @@
         <v>33</v>
       </c>
       <c r="B7" s="33">
-        <v>22.0</v>
+        <v>23.0</v>
       </c>
       <c r="C7" s="34">
         <v>21.0</v>
@@ -2638,7 +2699,7 @@
         <v>32.0</v>
       </c>
       <c r="C8" s="34">
-        <v>30.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="9">
@@ -2646,7 +2707,7 @@
         <v>56</v>
       </c>
       <c r="B9" s="33">
-        <v>9.0</v>
+        <v>10.0</v>
       </c>
       <c r="C9" s="34">
         <v>8.0</v>
@@ -2690,10 +2751,10 @@
         <v>50</v>
       </c>
       <c r="B13" s="33">
-        <v>11.0</v>
+        <v>12.0</v>
       </c>
       <c r="C13" s="34">
-        <v>11.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="14">
@@ -2734,10 +2795,10 @@
         <v>36</v>
       </c>
       <c r="B17" s="33">
-        <v>12.0</v>
+        <v>11.0</v>
       </c>
       <c r="C17" s="34">
-        <v>11.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="18">
@@ -2756,7 +2817,7 @@
         <v>39</v>
       </c>
       <c r="B19" s="33">
-        <v>30.0</v>
+        <v>31.0</v>
       </c>
       <c r="C19" s="34">
         <v>29.0</v>
@@ -2811,10 +2872,10 @@
         <v>61</v>
       </c>
       <c r="B24" s="33">
-        <v>26.0</v>
+        <v>27.0</v>
       </c>
       <c r="C24" s="34">
-        <v>26.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="25">
@@ -2822,7 +2883,7 @@
         <v>58</v>
       </c>
       <c r="B25" s="33">
-        <v>20.0</v>
+        <v>19.0</v>
       </c>
       <c r="C25" s="34">
         <v>18.0</v>
@@ -2866,10 +2927,10 @@
         <v>57</v>
       </c>
       <c r="B29" s="14">
-        <v>22.0</v>
+        <v>24.0</v>
       </c>
       <c r="C29" s="14">
-        <v>22.0</v>
+        <v>25.0</v>
       </c>
     </row>
     <row r="30">
@@ -6774,7 +6835,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="6.0"/>
-    <col customWidth="1" min="2" max="2" width="24.75"/>
+    <col customWidth="1" min="2" max="2" width="31.38"/>
     <col customWidth="1" min="3" max="3" width="23.75"/>
   </cols>
   <sheetData>
@@ -6807,13 +6868,17 @@
       <c r="B3" s="42" t="s">
         <v>73</v>
       </c>
-      <c r="C3" s="43"/>
+      <c r="C3" s="43" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="14">
         <v>3.0</v>
       </c>
-      <c r="B4" s="42"/>
+      <c r="B4" s="42" t="s">
+        <v>74</v>
+      </c>
       <c r="C4" s="43"/>
     </row>
     <row r="5">
@@ -11841,16 +11906,16 @@
         <v>69</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D1" s="44" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2">
@@ -11888,11 +11953,11 @@
       </c>
       <c r="D3" s="46" t="str">
         <f>'THURSDAY SINGLES'!D21</f>
-        <v/>
-      </c>
-      <c r="E3" s="45" t="str">
+        <v>KEN PEEL</v>
+      </c>
+      <c r="E3" s="45">
         <f>'THURSDAY SINGLES'!D22</f>
-        <v/>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -11901,11 +11966,11 @@
       </c>
       <c r="B4" s="45" t="str">
         <f>'SUNDAY SINGLES'!E28</f>
-        <v/>
-      </c>
-      <c r="C4" s="45" t="str">
+        <v>KEN PEEL</v>
+      </c>
+      <c r="C4" s="45">
         <f>'SUNDAY SINGLES'!E29</f>
-        <v/>
+        <v>37</v>
       </c>
       <c r="D4" s="46" t="str">
         <f>'THURSDAY SINGLES'!E21</f>

</xml_diff>

<commit_message>
094 Week 3/4 data update
</commit_message>
<xml_diff>
--- a/data/SUMMER_GOLF_2026.xlsx
+++ b/data/SUMMER_GOLF_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="80">
   <si>
     <t>SUMMER GOLF 2026 - THURSDAY SINGLES</t>
   </si>
@@ -240,6 +240,9 @@
   </si>
   <si>
     <t>JOHN ANTCLIFFE/PAUL HANCOX</t>
+  </si>
+  <si>
+    <t>MICK SKINNER/BAZ MASON</t>
   </si>
   <si>
     <t>SUNDAY</t>
@@ -972,7 +975,9 @@
       <c r="D6" s="14">
         <v>33.0</v>
       </c>
-      <c r="E6" s="13"/>
+      <c r="E6" s="13">
+        <v>26.0</v>
+      </c>
       <c r="F6" s="14"/>
       <c r="G6" s="13"/>
       <c r="H6" s="14"/>
@@ -996,7 +1001,7 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>67</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7">
@@ -1007,7 +1012,9 @@
       <c r="D7" s="14">
         <v>28.0</v>
       </c>
-      <c r="E7" s="13"/>
+      <c r="E7" s="13">
+        <v>32.0</v>
+      </c>
       <c r="F7" s="14"/>
       <c r="G7" s="13"/>
       <c r="H7" s="14"/>
@@ -1031,7 +1038,7 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>28</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
@@ -1044,7 +1051,9 @@
       <c r="D8" s="14">
         <v>34.0</v>
       </c>
-      <c r="E8" s="13"/>
+      <c r="E8" s="13">
+        <v>30.0</v>
+      </c>
       <c r="F8" s="14"/>
       <c r="G8" s="13"/>
       <c r="H8" s="14"/>
@@ -1068,7 +1077,7 @@
       <c r="Z8" s="19"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -1081,7 +1090,9 @@
       <c r="D9" s="14">
         <v>34.0</v>
       </c>
-      <c r="E9" s="13"/>
+      <c r="E9" s="13">
+        <v>20.0</v>
+      </c>
       <c r="F9" s="14"/>
       <c r="G9" s="13"/>
       <c r="H9" s="14"/>
@@ -1105,7 +1116,7 @@
       <c r="Z9" s="17"/>
       <c r="AA9" s="15">
         <f t="shared" si="1"/>
-        <v>64</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10">
@@ -1118,7 +1129,9 @@
       <c r="D10" s="14">
         <v>34.0</v>
       </c>
-      <c r="E10" s="13"/>
+      <c r="E10" s="13">
+        <v>25.0</v>
+      </c>
       <c r="F10" s="15"/>
       <c r="G10" s="13"/>
       <c r="H10" s="14"/>
@@ -1142,7 +1155,7 @@
       <c r="Z10" s="17"/>
       <c r="AA10" s="15">
         <f t="shared" si="1"/>
-        <v>66</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11">
@@ -1155,7 +1168,9 @@
       <c r="D11" s="14">
         <v>30.0</v>
       </c>
-      <c r="E11" s="13"/>
+      <c r="E11" s="13">
+        <v>31.0</v>
+      </c>
       <c r="F11" s="14"/>
       <c r="G11" s="13"/>
       <c r="H11" s="14"/>
@@ -1179,7 +1194,7 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>69</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -1188,7 +1203,9 @@
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="14"/>
-      <c r="E12" s="13"/>
+      <c r="E12" s="13">
+        <v>22.0</v>
+      </c>
       <c r="F12" s="14"/>
       <c r="G12" s="13"/>
       <c r="H12" s="14"/>
@@ -1212,7 +1229,7 @@
       <c r="Z12" s="17"/>
       <c r="AA12" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13">
@@ -1225,7 +1242,9 @@
       <c r="D13" s="14">
         <v>29.0</v>
       </c>
-      <c r="E13" s="13"/>
+      <c r="E13" s="13">
+        <v>25.0</v>
+      </c>
       <c r="F13" s="14"/>
       <c r="G13" s="13"/>
       <c r="H13" s="14"/>
@@ -1249,7 +1268,7 @@
       <c r="Z13" s="17"/>
       <c r="AA13" s="15">
         <f t="shared" si="1"/>
-        <v>57</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14">
@@ -1262,7 +1281,9 @@
       <c r="D14" s="14">
         <v>31.0</v>
       </c>
-      <c r="E14" s="16"/>
+      <c r="E14" s="13">
+        <v>28.0</v>
+      </c>
       <c r="F14" s="14"/>
       <c r="G14" s="13"/>
       <c r="H14" s="14"/>
@@ -1286,7 +1307,7 @@
       <c r="Z14" s="17"/>
       <c r="AA14" s="15">
         <f t="shared" si="1"/>
-        <v>61</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15">
@@ -1297,7 +1318,9 @@
       <c r="D15" s="14">
         <v>28.0</v>
       </c>
-      <c r="E15" s="13"/>
+      <c r="E15" s="13">
+        <v>33.0</v>
+      </c>
       <c r="F15" s="14"/>
       <c r="G15" s="13"/>
       <c r="H15" s="14"/>
@@ -1321,7 +1344,7 @@
       <c r="Z15" s="17"/>
       <c r="AA15" s="15">
         <f t="shared" si="1"/>
-        <v>28</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16">
@@ -1400,7 +1423,9 @@
       <c r="D18" s="14">
         <v>21.0</v>
       </c>
-      <c r="E18" s="13"/>
+      <c r="E18" s="13">
+        <v>22.0</v>
+      </c>
       <c r="F18" s="14"/>
       <c r="G18" s="13"/>
       <c r="H18" s="14"/>
@@ -1424,7 +1449,7 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>44</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19">
@@ -1496,7 +1521,9 @@
       <c r="D21" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="E21" s="24"/>
+      <c r="E21" s="24" t="s">
+        <v>40</v>
+      </c>
       <c r="F21" s="24"/>
       <c r="G21" s="24"/>
       <c r="H21" s="24"/>
@@ -1530,7 +1557,9 @@
       <c r="D22" s="27">
         <v>34.0</v>
       </c>
-      <c r="E22" s="27"/>
+      <c r="E22" s="27">
+        <v>33.0</v>
+      </c>
       <c r="F22" s="27"/>
       <c r="G22" s="27"/>
       <c r="H22" s="27"/>
@@ -1702,7 +1731,9 @@
       </c>
       <c r="D5" s="14"/>
       <c r="E5" s="13"/>
-      <c r="F5" s="14"/>
+      <c r="F5" s="14">
+        <v>30.0</v>
+      </c>
       <c r="G5" s="13"/>
       <c r="H5" s="15"/>
       <c r="I5" s="13"/>
@@ -1725,7 +1756,7 @@
       <c r="Z5" s="19"/>
       <c r="AA5" s="15">
         <f t="shared" ref="AA5:AA26" si="1">SUM(C5:Z5)</f>
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -1739,7 +1770,9 @@
       <c r="E6" s="13">
         <v>31.0</v>
       </c>
-      <c r="F6" s="14"/>
+      <c r="F6" s="14">
+        <v>36.0</v>
+      </c>
       <c r="G6" s="13"/>
       <c r="H6" s="14"/>
       <c r="I6" s="13"/>
@@ -1762,7 +1795,7 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>59</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7">
@@ -1778,7 +1811,9 @@
       <c r="E7" s="13">
         <v>30.0</v>
       </c>
-      <c r="F7" s="14"/>
+      <c r="F7" s="14">
+        <v>33.0</v>
+      </c>
       <c r="G7" s="13"/>
       <c r="H7" s="14"/>
       <c r="I7" s="13"/>
@@ -1801,7 +1836,7 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>82</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8">
@@ -1817,7 +1852,9 @@
       <c r="E8" s="13">
         <v>26.0</v>
       </c>
-      <c r="F8" s="14"/>
+      <c r="F8" s="14">
+        <v>34.0</v>
+      </c>
       <c r="G8" s="13"/>
       <c r="H8" s="14"/>
       <c r="I8" s="13"/>
@@ -1840,7 +1877,7 @@
       <c r="Z8" s="17"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>74</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9">
@@ -1854,7 +1891,9 @@
       <c r="E9" s="13">
         <v>29.0</v>
       </c>
-      <c r="F9" s="14"/>
+      <c r="F9" s="14">
+        <v>30.0</v>
+      </c>
       <c r="G9" s="13"/>
       <c r="H9" s="14"/>
       <c r="I9" s="16"/>
@@ -1877,7 +1916,7 @@
       <c r="Z9" s="17"/>
       <c r="AA9" s="15">
         <f t="shared" si="1"/>
-        <v>53</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10">
@@ -1924,7 +1963,9 @@
       <c r="E11" s="13">
         <v>34.0</v>
       </c>
-      <c r="F11" s="14"/>
+      <c r="F11" s="14">
+        <v>34.0</v>
+      </c>
       <c r="G11" s="13"/>
       <c r="H11" s="15"/>
       <c r="I11" s="16"/>
@@ -1947,7 +1988,7 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>67</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12">
@@ -2066,7 +2107,9 @@
         <v>34.0</v>
       </c>
       <c r="E15" s="13"/>
-      <c r="F15" s="14"/>
+      <c r="F15" s="14">
+        <v>27.0</v>
+      </c>
       <c r="G15" s="13"/>
       <c r="H15" s="14"/>
       <c r="I15" s="13"/>
@@ -2089,7 +2132,7 @@
       <c r="Z15" s="17"/>
       <c r="AA15" s="15">
         <f t="shared" si="1"/>
-        <v>57</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16">
@@ -2103,7 +2146,9 @@
       <c r="E16" s="13">
         <v>37.0</v>
       </c>
-      <c r="F16" s="14"/>
+      <c r="F16" s="14">
+        <v>31.0</v>
+      </c>
       <c r="G16" s="13"/>
       <c r="H16" s="14"/>
       <c r="I16" s="13"/>
@@ -2126,7 +2171,7 @@
       <c r="Z16" s="17"/>
       <c r="AA16" s="15">
         <f t="shared" si="1"/>
-        <v>64</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17">
@@ -2142,7 +2187,9 @@
       <c r="E17" s="13">
         <v>26.0</v>
       </c>
-      <c r="F17" s="14"/>
+      <c r="F17" s="14">
+        <v>22.0</v>
+      </c>
       <c r="G17" s="13"/>
       <c r="H17" s="14"/>
       <c r="I17" s="13"/>
@@ -2165,7 +2212,7 @@
       <c r="Z17" s="17"/>
       <c r="AA17" s="15">
         <f t="shared" si="1"/>
-        <v>65</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18">
@@ -2179,7 +2226,9 @@
       <c r="E18" s="13">
         <v>32.0</v>
       </c>
-      <c r="F18" s="14"/>
+      <c r="F18" s="14">
+        <v>33.0</v>
+      </c>
       <c r="G18" s="13"/>
       <c r="H18" s="14"/>
       <c r="I18" s="13"/>
@@ -2202,7 +2251,7 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>64</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19">
@@ -2255,7 +2304,9 @@
       <c r="E20" s="13">
         <v>30.0</v>
       </c>
-      <c r="F20" s="15"/>
+      <c r="F20" s="14">
+        <v>31.0</v>
+      </c>
       <c r="G20" s="13"/>
       <c r="H20" s="14"/>
       <c r="I20" s="13"/>
@@ -2278,7 +2329,7 @@
       <c r="Z20" s="17"/>
       <c r="AA20" s="15">
         <f t="shared" si="1"/>
-        <v>58</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21">
@@ -2288,7 +2339,9 @@
       <c r="C21" s="13"/>
       <c r="D21" s="14"/>
       <c r="E21" s="13"/>
-      <c r="F21" s="15"/>
+      <c r="F21" s="14">
+        <v>36.0</v>
+      </c>
       <c r="G21" s="13"/>
       <c r="H21" s="14"/>
       <c r="I21" s="13"/>
@@ -2311,7 +2364,7 @@
       <c r="Z21" s="17"/>
       <c r="AA21" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22">
@@ -2327,7 +2380,9 @@
       <c r="E22" s="13">
         <v>27.0</v>
       </c>
-      <c r="F22" s="15"/>
+      <c r="F22" s="14">
+        <v>32.0</v>
+      </c>
       <c r="G22" s="13"/>
       <c r="H22" s="14"/>
       <c r="I22" s="13"/>
@@ -2350,7 +2405,7 @@
       <c r="Z22" s="17"/>
       <c r="AA22" s="15">
         <f t="shared" si="1"/>
-        <v>86</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23">
@@ -2473,7 +2528,9 @@
       <c r="E26" s="13">
         <v>29.0</v>
       </c>
-      <c r="F26" s="15"/>
+      <c r="F26" s="14">
+        <v>31.0</v>
+      </c>
       <c r="G26" s="13"/>
       <c r="H26" s="14"/>
       <c r="I26" s="13"/>
@@ -2496,7 +2553,7 @@
       <c r="Z26" s="17"/>
       <c r="AA26" s="15">
         <f t="shared" si="1"/>
-        <v>48</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" ht="9.0" customHeight="1">
@@ -2538,7 +2595,9 @@
       <c r="E28" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="F28" s="24"/>
+      <c r="F28" s="24" t="s">
+        <v>40</v>
+      </c>
       <c r="G28" s="24"/>
       <c r="H28" s="24"/>
       <c r="I28" s="24"/>
@@ -2574,7 +2633,9 @@
       <c r="E29" s="27">
         <v>37.0</v>
       </c>
-      <c r="F29" s="27"/>
+      <c r="F29" s="27">
+        <v>36.0</v>
+      </c>
       <c r="G29" s="27"/>
       <c r="H29" s="27"/>
       <c r="I29" s="27"/>
@@ -2644,7 +2705,7 @@
         <v>12.0</v>
       </c>
       <c r="C3" s="34">
-        <v>10.0</v>
+        <v>11.0</v>
       </c>
     </row>
     <row r="4">
@@ -2674,10 +2735,10 @@
         <v>38</v>
       </c>
       <c r="B6" s="33">
+        <v>15.0</v>
+      </c>
+      <c r="C6" s="34">
         <v>14.0</v>
-      </c>
-      <c r="C6" s="34">
-        <v>13.0</v>
       </c>
     </row>
     <row r="7">
@@ -2696,7 +2757,7 @@
         <v>34</v>
       </c>
       <c r="B8" s="33">
-        <v>32.0</v>
+        <v>33.0</v>
       </c>
       <c r="C8" s="34">
         <v>31.0</v>
@@ -2795,10 +2856,10 @@
         <v>36</v>
       </c>
       <c r="B17" s="33">
+        <v>12.0</v>
+      </c>
+      <c r="C17" s="34">
         <v>11.0</v>
-      </c>
-      <c r="C17" s="34">
-        <v>10.0</v>
       </c>
     </row>
     <row r="18">
@@ -6879,13 +6940,17 @@
       <c r="B4" s="42" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="43"/>
+      <c r="C4" s="43" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="14">
         <v>4.0</v>
       </c>
-      <c r="B5" s="42"/>
+      <c r="B5" s="42" t="s">
+        <v>75</v>
+      </c>
       <c r="C5" s="43"/>
     </row>
     <row r="6">
@@ -11906,16 +11971,16 @@
         <v>69</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D1" s="44" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2">
@@ -11974,11 +12039,11 @@
       </c>
       <c r="D4" s="46" t="str">
         <f>'THURSDAY SINGLES'!E21</f>
-        <v/>
-      </c>
-      <c r="E4" s="45" t="str">
+        <v>SCOTT LEONARDE</v>
+      </c>
+      <c r="E4" s="45">
         <f>'THURSDAY SINGLES'!E22</f>
-        <v/>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
@@ -11987,11 +12052,11 @@
       </c>
       <c r="B5" s="45" t="str">
         <f>'SUNDAY SINGLES'!F28</f>
-        <v/>
-      </c>
-      <c r="C5" s="45" t="str">
+        <v>SCOTT LEONARDE</v>
+      </c>
+      <c r="C5" s="45">
         <f>'SUNDAY SINGLES'!F29</f>
-        <v/>
+        <v>36</v>
       </c>
       <c r="D5" s="46" t="str">
         <f>'THURSDAY SINGLES'!F21</f>

</xml_diff>

<commit_message>
095 Week 4/5 data update
</commit_message>
<xml_diff>
--- a/data/SUMMER_GOLF_2026.xlsx
+++ b/data/SUMMER_GOLF_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="85">
   <si>
     <t>SUMMER GOLF 2026 - THURSDAY SINGLES</t>
   </si>
@@ -155,6 +155,9 @@
     <t>WEEKLY WINNER</t>
   </si>
   <si>
+    <t>STEVE  FELLOWS</t>
+  </si>
+  <si>
     <t>WINNERS SCORE</t>
   </si>
   <si>
@@ -165,6 +168,15 @@
   </si>
   <si>
     <t>26/04/26</t>
+  </si>
+  <si>
+    <t>17/05/26</t>
+  </si>
+  <si>
+    <t>24/05/26</t>
+  </si>
+  <si>
+    <t>31/05/26</t>
   </si>
   <si>
     <t>TONI SHIRLEY</t>
@@ -203,13 +215,13 @@
     <t>HELEN RIGG</t>
   </si>
   <si>
+    <t>STEW TAYLOR</t>
+  </si>
+  <si>
     <t>WHITE TEES</t>
   </si>
   <si>
     <t>YELLOW TEES</t>
-  </si>
-  <si>
-    <t>STEW TAYLOR</t>
   </si>
   <si>
     <t>CHRIS HARVEY</t>
@@ -243,6 +255,9 @@
   </si>
   <si>
     <t>MICK SKINNER/BAZ MASON</t>
+  </si>
+  <si>
+    <t>PAUL DIXON/STEW TAYLOR</t>
   </si>
   <si>
     <t>SUNDAY</t>
@@ -939,7 +954,9 @@
         <v>30.0</v>
       </c>
       <c r="E5" s="13"/>
-      <c r="F5" s="14"/>
+      <c r="F5" s="14">
+        <v>25.0</v>
+      </c>
       <c r="G5" s="13"/>
       <c r="H5" s="14"/>
       <c r="I5" s="13"/>
@@ -962,7 +979,7 @@
       <c r="Z5" s="17"/>
       <c r="AA5" s="15">
         <f t="shared" ref="AA5:AA19" si="1">sum(C5:Z5)</f>
-        <v>59</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6">
@@ -978,7 +995,9 @@
       <c r="E6" s="13">
         <v>26.0</v>
       </c>
-      <c r="F6" s="14"/>
+      <c r="F6" s="14">
+        <v>23.0</v>
+      </c>
       <c r="G6" s="13"/>
       <c r="H6" s="14"/>
       <c r="I6" s="13"/>
@@ -1001,7 +1020,7 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>93</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7">
@@ -1015,7 +1034,9 @@
       <c r="E7" s="13">
         <v>32.0</v>
       </c>
-      <c r="F7" s="14"/>
+      <c r="F7" s="14">
+        <v>27.0</v>
+      </c>
       <c r="G7" s="13"/>
       <c r="H7" s="14"/>
       <c r="I7" s="13"/>
@@ -1038,7 +1059,7 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8">
@@ -1054,7 +1075,9 @@
       <c r="E8" s="13">
         <v>30.0</v>
       </c>
-      <c r="F8" s="14"/>
+      <c r="F8" s="14">
+        <v>29.0</v>
+      </c>
       <c r="G8" s="13"/>
       <c r="H8" s="14"/>
       <c r="I8" s="13"/>
@@ -1077,7 +1100,7 @@
       <c r="Z8" s="19"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9">
@@ -1093,7 +1116,9 @@
       <c r="E9" s="13">
         <v>20.0</v>
       </c>
-      <c r="F9" s="14"/>
+      <c r="F9" s="14">
+        <v>29.0</v>
+      </c>
       <c r="G9" s="13"/>
       <c r="H9" s="14"/>
       <c r="I9" s="13"/>
@@ -1116,7 +1141,7 @@
       <c r="Z9" s="17"/>
       <c r="AA9" s="15">
         <f t="shared" si="1"/>
-        <v>84</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10">
@@ -1171,7 +1196,9 @@
       <c r="E11" s="13">
         <v>31.0</v>
       </c>
-      <c r="F11" s="14"/>
+      <c r="F11" s="14">
+        <v>29.0</v>
+      </c>
       <c r="G11" s="13"/>
       <c r="H11" s="14"/>
       <c r="I11" s="13"/>
@@ -1194,7 +1221,7 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12">
@@ -1206,7 +1233,9 @@
       <c r="E12" s="13">
         <v>22.0</v>
       </c>
-      <c r="F12" s="14"/>
+      <c r="F12" s="14">
+        <v>32.0</v>
+      </c>
       <c r="G12" s="13"/>
       <c r="H12" s="14"/>
       <c r="I12" s="13"/>
@@ -1229,7 +1258,7 @@
       <c r="Z12" s="17"/>
       <c r="AA12" s="15">
         <f t="shared" si="1"/>
-        <v>22</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13">
@@ -1321,7 +1350,9 @@
       <c r="E15" s="13">
         <v>33.0</v>
       </c>
-      <c r="F15" s="14"/>
+      <c r="F15" s="14">
+        <v>21.0</v>
+      </c>
       <c r="G15" s="13"/>
       <c r="H15" s="14"/>
       <c r="I15" s="13"/>
@@ -1344,7 +1375,7 @@
       <c r="Z15" s="17"/>
       <c r="AA15" s="15">
         <f t="shared" si="1"/>
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16">
@@ -1426,7 +1457,9 @@
       <c r="E18" s="13">
         <v>22.0</v>
       </c>
-      <c r="F18" s="14"/>
+      <c r="F18" s="14">
+        <v>29.0</v>
+      </c>
       <c r="G18" s="13"/>
       <c r="H18" s="14"/>
       <c r="I18" s="13"/>
@@ -1449,7 +1482,7 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>66</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19">
@@ -1459,7 +1492,9 @@
       <c r="C19" s="17"/>
       <c r="D19" s="14"/>
       <c r="E19" s="13"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="14">
+        <v>27.0</v>
+      </c>
       <c r="G19" s="13"/>
       <c r="H19" s="14"/>
       <c r="I19" s="13"/>
@@ -1482,7 +1517,7 @@
       <c r="Z19" s="17"/>
       <c r="AA19" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" ht="9.0" customHeight="1">
@@ -1524,7 +1559,9 @@
       <c r="E21" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="F21" s="24"/>
+      <c r="F21" s="24" t="s">
+        <v>46</v>
+      </c>
       <c r="G21" s="24"/>
       <c r="H21" s="24"/>
       <c r="I21" s="24"/>
@@ -1549,7 +1586,7 @@
     </row>
     <row r="22">
       <c r="B22" s="26" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C22" s="27">
         <v>39.0</v>
@@ -1560,7 +1597,9 @@
       <c r="E22" s="27">
         <v>33.0</v>
       </c>
-      <c r="F22" s="27"/>
+      <c r="F22" s="27">
+        <v>35.0</v>
+      </c>
       <c r="G22" s="27"/>
       <c r="H22" s="27"/>
       <c r="I22" s="27"/>
@@ -1602,7 +1641,7 @@
   <sheetData>
     <row r="2" ht="24.0" customHeight="1">
       <c r="B2" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
@@ -1615,16 +1654,26 @@
         <v>46360.0</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
+        <v>50</v>
+      </c>
+      <c r="G3" s="3">
+        <v>46086.0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>46300.0</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="L3" s="4"/>
       <c r="M3" s="5"/>
       <c r="N3" s="4"/>
@@ -1724,7 +1773,7 @@
     </row>
     <row r="5">
       <c r="B5" s="12" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C5" s="13">
         <v>24.0</v>
@@ -1734,7 +1783,9 @@
       <c r="F5" s="14">
         <v>30.0</v>
       </c>
-      <c r="G5" s="13"/>
+      <c r="G5" s="13">
+        <v>26.0</v>
+      </c>
       <c r="H5" s="15"/>
       <c r="I5" s="13"/>
       <c r="J5" s="14"/>
@@ -1756,12 +1807,12 @@
       <c r="Z5" s="19"/>
       <c r="AA5" s="15">
         <f t="shared" ref="AA5:AA26" si="1">SUM(C5:Z5)</f>
-        <v>54</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="18" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C6" s="13">
         <v>28.0</v>
@@ -1773,7 +1824,9 @@
       <c r="F6" s="14">
         <v>36.0</v>
       </c>
-      <c r="G6" s="13"/>
+      <c r="G6" s="13">
+        <v>31.0</v>
+      </c>
       <c r="H6" s="14"/>
       <c r="I6" s="13"/>
       <c r="J6" s="14"/>
@@ -1795,7 +1848,7 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>95</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7">
@@ -1814,7 +1867,9 @@
       <c r="F7" s="14">
         <v>33.0</v>
       </c>
-      <c r="G7" s="13"/>
+      <c r="G7" s="13">
+        <v>30.0</v>
+      </c>
       <c r="H7" s="14"/>
       <c r="I7" s="13"/>
       <c r="J7" s="14"/>
@@ -1836,7 +1891,7 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8">
@@ -1882,7 +1937,7 @@
     </row>
     <row r="9">
       <c r="B9" s="18" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C9" s="13">
         <v>24.0</v>
@@ -1894,7 +1949,9 @@
       <c r="F9" s="14">
         <v>30.0</v>
       </c>
-      <c r="G9" s="13"/>
+      <c r="G9" s="13">
+        <v>29.0</v>
+      </c>
       <c r="H9" s="14"/>
       <c r="I9" s="16"/>
       <c r="J9" s="15"/>
@@ -1916,7 +1973,7 @@
       <c r="Z9" s="17"/>
       <c r="AA9" s="15">
         <f t="shared" si="1"/>
-        <v>83</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10">
@@ -1927,7 +1984,9 @@
       <c r="D10" s="14"/>
       <c r="E10" s="13"/>
       <c r="F10" s="14"/>
-      <c r="G10" s="13"/>
+      <c r="G10" s="13">
+        <v>25.0</v>
+      </c>
       <c r="H10" s="14"/>
       <c r="I10" s="13"/>
       <c r="J10" s="14"/>
@@ -1949,12 +2008,12 @@
       <c r="Z10" s="19"/>
       <c r="AA10" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="18" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="14">
@@ -1966,7 +2025,9 @@
       <c r="F11" s="14">
         <v>34.0</v>
       </c>
-      <c r="G11" s="13"/>
+      <c r="G11" s="13">
+        <v>23.0</v>
+      </c>
       <c r="H11" s="15"/>
       <c r="I11" s="16"/>
       <c r="J11" s="15"/>
@@ -1988,7 +2049,7 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>101</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12">
@@ -2036,7 +2097,9 @@
       </c>
       <c r="E13" s="13"/>
       <c r="F13" s="14"/>
-      <c r="G13" s="13"/>
+      <c r="G13" s="13">
+        <v>26.0</v>
+      </c>
       <c r="H13" s="14"/>
       <c r="I13" s="16"/>
       <c r="J13" s="14"/>
@@ -2058,12 +2121,12 @@
       <c r="Z13" s="17"/>
       <c r="AA13" s="15">
         <f t="shared" si="1"/>
-        <v>59</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="18" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C14" s="13">
         <v>28.0</v>
@@ -2071,7 +2134,9 @@
       <c r="D14" s="14"/>
       <c r="E14" s="13"/>
       <c r="F14" s="14"/>
-      <c r="G14" s="13"/>
+      <c r="G14" s="13">
+        <v>21.0</v>
+      </c>
       <c r="H14" s="14"/>
       <c r="I14" s="16"/>
       <c r="J14" s="14"/>
@@ -2093,7 +2158,7 @@
       <c r="Z14" s="17"/>
       <c r="AA14" s="15">
         <f t="shared" si="1"/>
-        <v>28</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15">
@@ -2110,7 +2175,9 @@
       <c r="F15" s="14">
         <v>27.0</v>
       </c>
-      <c r="G15" s="13"/>
+      <c r="G15" s="13">
+        <v>21.0</v>
+      </c>
       <c r="H15" s="14"/>
       <c r="I15" s="13"/>
       <c r="J15" s="15"/>
@@ -2132,7 +2199,7 @@
       <c r="Z15" s="17"/>
       <c r="AA15" s="15">
         <f t="shared" si="1"/>
-        <v>84</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16">
@@ -2149,7 +2216,9 @@
       <c r="F16" s="14">
         <v>31.0</v>
       </c>
-      <c r="G16" s="13"/>
+      <c r="G16" s="13">
+        <v>32.0</v>
+      </c>
       <c r="H16" s="14"/>
       <c r="I16" s="13"/>
       <c r="J16" s="15"/>
@@ -2171,7 +2240,7 @@
       <c r="Z16" s="17"/>
       <c r="AA16" s="15">
         <f t="shared" si="1"/>
-        <v>95</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17">
@@ -2190,7 +2259,9 @@
       <c r="F17" s="14">
         <v>22.0</v>
       </c>
-      <c r="G17" s="13"/>
+      <c r="G17" s="13">
+        <v>20.0</v>
+      </c>
       <c r="H17" s="14"/>
       <c r="I17" s="13"/>
       <c r="J17" s="14"/>
@@ -2212,12 +2283,12 @@
       <c r="Z17" s="17"/>
       <c r="AA17" s="15">
         <f t="shared" si="1"/>
-        <v>87</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="18" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C18" s="13">
         <v>32.0</v>
@@ -2229,7 +2300,9 @@
       <c r="F18" s="14">
         <v>33.0</v>
       </c>
-      <c r="G18" s="13"/>
+      <c r="G18" s="13">
+        <v>39.0</v>
+      </c>
       <c r="H18" s="14"/>
       <c r="I18" s="13"/>
       <c r="J18" s="14"/>
@@ -2251,12 +2324,12 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="18" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C19" s="13">
         <v>30.0</v>
@@ -2268,7 +2341,9 @@
         <v>26.0</v>
       </c>
       <c r="F19" s="14"/>
-      <c r="G19" s="13"/>
+      <c r="G19" s="13">
+        <v>36.0</v>
+      </c>
       <c r="H19" s="14"/>
       <c r="I19" s="13"/>
       <c r="J19" s="14"/>
@@ -2290,12 +2365,12 @@
       <c r="Z19" s="17"/>
       <c r="AA19" s="15">
         <f t="shared" si="1"/>
-        <v>86</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="18" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C20" s="13">
         <v>28.0</v>
@@ -2307,7 +2382,9 @@
       <c r="F20" s="14">
         <v>31.0</v>
       </c>
-      <c r="G20" s="13"/>
+      <c r="G20" s="13">
+        <v>33.0</v>
+      </c>
       <c r="H20" s="14"/>
       <c r="I20" s="13"/>
       <c r="J20" s="14"/>
@@ -2329,7 +2406,7 @@
       <c r="Z20" s="17"/>
       <c r="AA20" s="15">
         <f t="shared" si="1"/>
-        <v>89</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21">
@@ -2369,7 +2446,7 @@
     </row>
     <row r="22">
       <c r="B22" s="18" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C22" s="13">
         <v>20.0</v>
@@ -2383,7 +2460,9 @@
       <c r="F22" s="14">
         <v>32.0</v>
       </c>
-      <c r="G22" s="13"/>
+      <c r="G22" s="13">
+        <v>36.0</v>
+      </c>
       <c r="H22" s="14"/>
       <c r="I22" s="13"/>
       <c r="J22" s="14"/>
@@ -2405,7 +2484,7 @@
       <c r="Z22" s="17"/>
       <c r="AA22" s="15">
         <f t="shared" si="1"/>
-        <v>118</v>
+        <v>154</v>
       </c>
     </row>
     <row r="23">
@@ -2418,7 +2497,9 @@
         <v>34.0</v>
       </c>
       <c r="F23" s="15"/>
-      <c r="G23" s="13"/>
+      <c r="G23" s="13">
+        <v>40.0</v>
+      </c>
       <c r="H23" s="14"/>
       <c r="I23" s="13"/>
       <c r="J23" s="14"/>
@@ -2440,12 +2521,12 @@
       <c r="Z23" s="17"/>
       <c r="AA23" s="15">
         <f t="shared" si="1"/>
-        <v>34</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="18" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C24" s="13"/>
       <c r="D24" s="14">
@@ -2480,7 +2561,7 @@
     </row>
     <row r="25">
       <c r="B25" s="18" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C25" s="13">
         <v>35.0</v>
@@ -2492,7 +2573,9 @@
         <v>33.0</v>
       </c>
       <c r="F25" s="15"/>
-      <c r="G25" s="13"/>
+      <c r="G25" s="13">
+        <v>33.0</v>
+      </c>
       <c r="H25" s="14"/>
       <c r="I25" s="13"/>
       <c r="J25" s="14"/>
@@ -2514,12 +2597,12 @@
       <c r="Z25" s="17"/>
       <c r="AA25" s="15">
         <f t="shared" si="1"/>
-        <v>93</v>
+        <v>126</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="18" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C26" s="13">
         <v>19.0</v>
@@ -2531,7 +2614,9 @@
       <c r="F26" s="14">
         <v>31.0</v>
       </c>
-      <c r="G26" s="13"/>
+      <c r="G26" s="13">
+        <v>25.0</v>
+      </c>
       <c r="H26" s="14"/>
       <c r="I26" s="13"/>
       <c r="J26" s="14"/>
@@ -2553,7 +2638,7 @@
       <c r="Z26" s="17"/>
       <c r="AA26" s="15">
         <f t="shared" si="1"/>
-        <v>79</v>
+        <v>104</v>
       </c>
     </row>
     <row r="27" ht="9.0" customHeight="1">
@@ -2587,10 +2672,10 @@
         <v>45</v>
       </c>
       <c r="C28" s="24" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D28" s="24" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E28" s="24" t="s">
         <v>34</v>
@@ -2598,7 +2683,9 @@
       <c r="F28" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="G28" s="24"/>
+      <c r="G28" s="24" t="s">
+        <v>66</v>
+      </c>
       <c r="H28" s="24"/>
       <c r="I28" s="24"/>
       <c r="J28" s="24"/>
@@ -2622,7 +2709,7 @@
     </row>
     <row r="29">
       <c r="B29" s="26" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C29" s="27">
         <v>35.0</v>
@@ -2636,7 +2723,9 @@
       <c r="F29" s="27">
         <v>36.0</v>
       </c>
-      <c r="G29" s="27"/>
+      <c r="G29" s="27">
+        <v>40.0</v>
+      </c>
       <c r="H29" s="27"/>
       <c r="I29" s="27"/>
       <c r="J29" s="27"/>
@@ -2680,10 +2769,10 @@
         <v>4</v>
       </c>
       <c r="B1" s="30" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C1" s="31" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2">
@@ -2691,7 +2780,7 @@
         <v>43</v>
       </c>
       <c r="B2" s="33">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
       <c r="C2" s="34">
         <v>14.0</v>
@@ -2710,7 +2799,7 @@
     </row>
     <row r="4">
       <c r="A4" s="18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B4" s="33">
         <v>9.0</v>
@@ -2765,7 +2854,7 @@
     </row>
     <row r="9">
       <c r="A9" s="18" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B9" s="33">
         <v>10.0</v>
@@ -2779,7 +2868,7 @@
         <v>44</v>
       </c>
       <c r="B10" s="33">
-        <v>17.0</v>
+        <v>16.0</v>
       </c>
       <c r="C10" s="34">
         <v>15.0</v>
@@ -2787,10 +2876,10 @@
     </row>
     <row r="11">
       <c r="A11" s="18" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B11" s="33">
-        <v>23.0</v>
+        <v>22.0</v>
       </c>
       <c r="C11" s="34">
         <v>21.0</v>
@@ -2801,15 +2890,15 @@
         <v>37</v>
       </c>
       <c r="B12" s="33">
+        <v>8.0</v>
+      </c>
+      <c r="C12" s="35">
         <v>6.0</v>
-      </c>
-      <c r="C12" s="35">
-        <v>5.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="18" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B13" s="33">
         <v>12.0</v>
@@ -2820,7 +2909,7 @@
     </row>
     <row r="14">
       <c r="A14" s="18" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B14" s="33">
         <v>20.0</v>
@@ -2831,7 +2920,7 @@
     </row>
     <row r="15">
       <c r="A15" s="18" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B15" s="33">
         <v>7.0</v>
@@ -2842,13 +2931,13 @@
     </row>
     <row r="16">
       <c r="A16" s="18" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B16" s="33">
+        <v>15.0</v>
+      </c>
+      <c r="C16" s="34">
         <v>14.0</v>
-      </c>
-      <c r="C16" s="34">
-        <v>13.0</v>
       </c>
     </row>
     <row r="17">
@@ -2864,7 +2953,7 @@
     </row>
     <row r="18">
       <c r="A18" s="18" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B18" s="33">
         <v>-1.0</v>
@@ -2897,13 +2986,13 @@
     </row>
     <row r="21">
       <c r="A21" s="18" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B21" s="33">
+        <v>8.0</v>
+      </c>
+      <c r="C21" s="34">
         <v>7.0</v>
-      </c>
-      <c r="C21" s="34">
-        <v>6.0</v>
       </c>
     </row>
     <row r="22">
@@ -2930,7 +3019,7 @@
     </row>
     <row r="24">
       <c r="A24" s="36" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B24" s="33">
         <v>27.0</v>
@@ -2941,7 +3030,7 @@
     </row>
     <row r="25">
       <c r="A25" s="36" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B25" s="33">
         <v>19.0</v>
@@ -2952,10 +3041,10 @@
     </row>
     <row r="26">
       <c r="A26" s="36" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B26" s="14">
-        <v>13.0</v>
+        <v>12.0</v>
       </c>
       <c r="C26" s="14">
         <v>11.0</v>
@@ -2963,7 +3052,7 @@
     </row>
     <row r="27">
       <c r="A27" s="36" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B27" s="14">
         <v>15.0</v>
@@ -2974,7 +3063,7 @@
     </row>
     <row r="28">
       <c r="A28" s="36" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B28" s="14">
         <v>20.0</v>
@@ -2985,18 +3074,18 @@
     </row>
     <row r="29">
       <c r="A29" s="36" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B29" s="14">
+        <v>23.0</v>
+      </c>
+      <c r="C29" s="14">
         <v>24.0</v>
-      </c>
-      <c r="C29" s="14">
-        <v>25.0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="36" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B30" s="14">
         <v>23.0</v>
@@ -3007,7 +3096,7 @@
     </row>
     <row r="31">
       <c r="A31" s="36" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B31" s="14">
         <v>20.0</v>
@@ -6902,13 +6991,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B1" s="37" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C1" s="38" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2">
@@ -6916,7 +7005,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="40" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C2" s="41" t="s">
         <v>33</v>
@@ -6927,7 +7016,7 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="42" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C3" s="43" t="s">
         <v>35</v>
@@ -6938,7 +7027,7 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="42" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C4" s="43" t="s">
         <v>38</v>
@@ -6949,15 +7038,19 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>75</v>
-      </c>
-      <c r="C5" s="43"/>
+        <v>79</v>
+      </c>
+      <c r="C5" s="43" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="14">
         <v>5.0</v>
       </c>
-      <c r="B6" s="42"/>
+      <c r="B6" s="42" t="s">
+        <v>80</v>
+      </c>
       <c r="C6" s="43"/>
     </row>
     <row r="7">
@@ -11968,19 +12061,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D1" s="44" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
@@ -12060,11 +12153,11 @@
       </c>
       <c r="D5" s="46" t="str">
         <f>'THURSDAY SINGLES'!F21</f>
-        <v/>
-      </c>
-      <c r="E5" s="45" t="str">
+        <v>STEVE  FELLOWS</v>
+      </c>
+      <c r="E5" s="45">
         <f>'THURSDAY SINGLES'!F22</f>
-        <v/>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -12073,11 +12166,11 @@
       </c>
       <c r="B6" s="45" t="str">
         <f>'SUNDAY SINGLES'!G28</f>
-        <v/>
-      </c>
-      <c r="C6" s="45" t="str">
+        <v>STEW TAYLOR</v>
+      </c>
+      <c r="C6" s="45">
         <f>'SUNDAY SINGLES'!G29</f>
-        <v/>
+        <v>40</v>
       </c>
       <c r="D6" s="46" t="str">
         <f>'THURSDAY SINGLES'!G21</f>

</xml_diff>

<commit_message>
Week 5/6 data update
</commit_message>
<xml_diff>
--- a/data/SUMMER_GOLF_2026.xlsx
+++ b/data/SUMMER_GOLF_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="89">
   <si>
     <t>SUMMER GOLF 2026 - THURSDAY SINGLES</t>
   </si>
@@ -27,6 +27,15 @@
   </si>
   <si>
     <t>30/04/26</t>
+  </si>
+  <si>
+    <t>14/05/26</t>
+  </si>
+  <si>
+    <t>21/05/26</t>
+  </si>
+  <si>
+    <t>28/05/26</t>
   </si>
   <si>
     <t>NAME</t>
@@ -218,6 +227,9 @@
     <t>STEW TAYLOR</t>
   </si>
   <si>
+    <t>DAVE CROSSLEY</t>
+  </si>
+  <si>
     <t>WHITE TEES</t>
   </si>
   <si>
@@ -225,9 +237,6 @@
   </si>
   <si>
     <t>CHRIS HARVEY</t>
-  </si>
-  <si>
-    <t>DAVE CROSSLEY</t>
   </si>
   <si>
     <t>LAURIE COOKE</t>
@@ -258,6 +267,9 @@
   </si>
   <si>
     <t>PAUL DIXON/STEW TAYLOR</t>
+  </si>
+  <si>
+    <t>JOHN ANTCLIFFE/DAVE BARNETT</t>
   </si>
   <si>
     <t>SUNDAY</t>
@@ -841,10 +853,18 @@
       <c r="F3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="4"/>
+      <c r="G3" s="3">
+        <v>46208.0</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="K3" s="5"/>
       <c r="L3" s="4"/>
       <c r="M3" s="5"/>
@@ -865,87 +885,87 @@
     </row>
     <row r="4">
       <c r="B4" s="8" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="N4" s="9" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P4" s="9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="Q4" s="9" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="R4" s="9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="T4" s="9" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="U4" s="9" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="V4" s="9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="W4" s="9" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="X4" s="9" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="Y4" s="9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="Z4" s="9" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="AA4" s="11" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="12" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C5" s="13">
         <v>29.0</v>
@@ -957,7 +977,9 @@
       <c r="F5" s="14">
         <v>25.0</v>
       </c>
-      <c r="G5" s="13"/>
+      <c r="G5" s="13">
+        <v>31.0</v>
+      </c>
       <c r="H5" s="14"/>
       <c r="I5" s="13"/>
       <c r="J5" s="14"/>
@@ -979,12 +1001,12 @@
       <c r="Z5" s="17"/>
       <c r="AA5" s="15">
         <f t="shared" ref="AA5:AA19" si="1">sum(C5:Z5)</f>
-        <v>84</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="18" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C6" s="13">
         <v>34.0</v>
@@ -998,7 +1020,9 @@
       <c r="F6" s="14">
         <v>23.0</v>
       </c>
-      <c r="G6" s="13"/>
+      <c r="G6" s="13">
+        <v>32.0</v>
+      </c>
       <c r="H6" s="14"/>
       <c r="I6" s="13"/>
       <c r="J6" s="14"/>
@@ -1020,12 +1044,12 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>116</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="18" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" s="14">
@@ -1037,7 +1061,9 @@
       <c r="F7" s="14">
         <v>27.0</v>
       </c>
-      <c r="G7" s="13"/>
+      <c r="G7" s="13">
+        <v>34.0</v>
+      </c>
       <c r="H7" s="14"/>
       <c r="I7" s="13"/>
       <c r="J7" s="14"/>
@@ -1059,12 +1085,12 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>87</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="18" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C8" s="13">
         <v>36.0</v>
@@ -1078,7 +1104,9 @@
       <c r="F8" s="14">
         <v>29.0</v>
       </c>
-      <c r="G8" s="13"/>
+      <c r="G8" s="13">
+        <v>36.0</v>
+      </c>
       <c r="H8" s="14"/>
       <c r="I8" s="13"/>
       <c r="J8" s="14"/>
@@ -1100,12 +1128,12 @@
       <c r="Z8" s="19"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>129</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="18" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C9" s="13">
         <v>30.0</v>
@@ -1119,7 +1147,9 @@
       <c r="F9" s="14">
         <v>29.0</v>
       </c>
-      <c r="G9" s="13"/>
+      <c r="G9" s="13">
+        <v>36.0</v>
+      </c>
       <c r="H9" s="14"/>
       <c r="I9" s="13"/>
       <c r="J9" s="14"/>
@@ -1141,12 +1171,12 @@
       <c r="Z9" s="17"/>
       <c r="AA9" s="15">
         <f t="shared" si="1"/>
-        <v>113</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="18" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C10" s="13">
         <v>32.0</v>
@@ -1158,7 +1188,9 @@
         <v>25.0</v>
       </c>
       <c r="F10" s="15"/>
-      <c r="G10" s="13"/>
+      <c r="G10" s="13">
+        <v>39.0</v>
+      </c>
       <c r="H10" s="14"/>
       <c r="I10" s="13"/>
       <c r="J10" s="14"/>
@@ -1180,12 +1212,12 @@
       <c r="Z10" s="17"/>
       <c r="AA10" s="15">
         <f t="shared" si="1"/>
-        <v>91</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="18" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C11" s="13">
         <v>39.0</v>
@@ -1226,7 +1258,7 @@
     </row>
     <row r="12">
       <c r="B12" s="18" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="14"/>
@@ -1236,7 +1268,9 @@
       <c r="F12" s="14">
         <v>32.0</v>
       </c>
-      <c r="G12" s="13"/>
+      <c r="G12" s="13">
+        <v>26.0</v>
+      </c>
       <c r="H12" s="14"/>
       <c r="I12" s="13"/>
       <c r="J12" s="14"/>
@@ -1258,12 +1292,12 @@
       <c r="Z12" s="17"/>
       <c r="AA12" s="15">
         <f t="shared" si="1"/>
-        <v>54</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="18" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C13" s="13">
         <v>28.0</v>
@@ -1275,7 +1309,9 @@
         <v>25.0</v>
       </c>
       <c r="F13" s="14"/>
-      <c r="G13" s="13"/>
+      <c r="G13" s="13">
+        <v>33.0</v>
+      </c>
       <c r="H13" s="14"/>
       <c r="I13" s="13"/>
       <c r="J13" s="14"/>
@@ -1297,12 +1333,12 @@
       <c r="Z13" s="17"/>
       <c r="AA13" s="15">
         <f t="shared" si="1"/>
-        <v>82</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C14" s="13">
         <v>30.0</v>
@@ -1341,7 +1377,7 @@
     </row>
     <row r="15">
       <c r="B15" s="18" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="14">
@@ -1353,7 +1389,9 @@
       <c r="F15" s="14">
         <v>21.0</v>
       </c>
-      <c r="G15" s="13"/>
+      <c r="G15" s="13">
+        <v>29.0</v>
+      </c>
       <c r="H15" s="14"/>
       <c r="I15" s="13"/>
       <c r="J15" s="14"/>
@@ -1375,12 +1413,12 @@
       <c r="Z15" s="17"/>
       <c r="AA15" s="15">
         <f t="shared" si="1"/>
-        <v>82</v>
+        <v>111</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="20" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C16" s="17"/>
       <c r="D16" s="14"/>
@@ -1413,7 +1451,7 @@
     </row>
     <row r="17">
       <c r="B17" s="20" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C17" s="17"/>
       <c r="D17" s="14"/>
@@ -1446,7 +1484,7 @@
     </row>
     <row r="18">
       <c r="B18" s="20" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C18" s="17">
         <v>23.0</v>
@@ -1460,7 +1498,9 @@
       <c r="F18" s="14">
         <v>29.0</v>
       </c>
-      <c r="G18" s="13"/>
+      <c r="G18" s="13">
+        <v>29.0</v>
+      </c>
       <c r="H18" s="14"/>
       <c r="I18" s="13"/>
       <c r="J18" s="14"/>
@@ -1482,12 +1522,12 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>95</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="20" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C19" s="17"/>
       <c r="D19" s="14"/>
@@ -1548,21 +1588,23 @@
     </row>
     <row r="21" ht="72.0" customHeight="1">
       <c r="B21" s="23" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C21" s="24" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D21" s="24" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F21" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="G21" s="24"/>
+        <v>49</v>
+      </c>
+      <c r="G21" s="24" t="s">
+        <v>38</v>
+      </c>
       <c r="H21" s="24"/>
       <c r="I21" s="24"/>
       <c r="J21" s="24"/>
@@ -1586,7 +1628,7 @@
     </row>
     <row r="22">
       <c r="B22" s="26" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C22" s="27">
         <v>39.0</v>
@@ -1600,7 +1642,9 @@
       <c r="F22" s="27">
         <v>35.0</v>
       </c>
-      <c r="G22" s="27"/>
+      <c r="G22" s="27">
+        <v>39.0</v>
+      </c>
       <c r="H22" s="27"/>
       <c r="I22" s="27"/>
       <c r="J22" s="27"/>
@@ -1641,7 +1685,7 @@
   <sheetData>
     <row r="2" ht="24.0" customHeight="1">
       <c r="B2" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
@@ -1654,10 +1698,10 @@
         <v>46360.0</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G3" s="3">
         <v>46086.0</v>
@@ -1666,13 +1710,13 @@
         <v>46300.0</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="5"/>
@@ -1693,87 +1737,87 @@
     </row>
     <row r="4">
       <c r="B4" s="8" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="N4" s="9" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P4" s="9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="Q4" s="9" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="R4" s="9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="S4" s="9" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="T4" s="9" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="U4" s="9" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="V4" s="9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="W4" s="9" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="X4" s="9" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="Y4" s="9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="Z4" s="9" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="AA4" s="11" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="12" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C5" s="13">
         <v>24.0</v>
@@ -1812,7 +1856,7 @@
     </row>
     <row r="6">
       <c r="B6" s="18" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C6" s="13">
         <v>28.0</v>
@@ -1827,7 +1871,9 @@
       <c r="G6" s="13">
         <v>31.0</v>
       </c>
-      <c r="H6" s="14"/>
+      <c r="H6" s="14">
+        <v>28.0</v>
+      </c>
       <c r="I6" s="13"/>
       <c r="J6" s="14"/>
       <c r="K6" s="13"/>
@@ -1848,12 +1894,12 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>126</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="18" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C7" s="13">
         <v>24.0</v>
@@ -1870,7 +1916,9 @@
       <c r="G7" s="13">
         <v>30.0</v>
       </c>
-      <c r="H7" s="14"/>
+      <c r="H7" s="14">
+        <v>36.0</v>
+      </c>
       <c r="I7" s="13"/>
       <c r="J7" s="14"/>
       <c r="K7" s="13"/>
@@ -1891,12 +1939,12 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>145</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="18" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C8" s="13">
         <v>24.0</v>
@@ -1911,7 +1959,9 @@
         <v>34.0</v>
       </c>
       <c r="G8" s="13"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14">
+        <v>35.0</v>
+      </c>
       <c r="I8" s="13"/>
       <c r="J8" s="14"/>
       <c r="K8" s="16"/>
@@ -1932,12 +1982,12 @@
       <c r="Z8" s="17"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>108</v>
+        <v>143</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="18" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C9" s="13">
         <v>24.0</v>
@@ -1978,7 +2028,7 @@
     </row>
     <row r="10">
       <c r="B10" s="18" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="14"/>
@@ -2013,7 +2063,7 @@
     </row>
     <row r="11">
       <c r="B11" s="18" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="14">
@@ -2028,7 +2078,9 @@
       <c r="G11" s="13">
         <v>23.0</v>
       </c>
-      <c r="H11" s="15"/>
+      <c r="H11" s="14">
+        <v>32.0</v>
+      </c>
       <c r="I11" s="16"/>
       <c r="J11" s="15"/>
       <c r="K11" s="13"/>
@@ -2049,12 +2101,12 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>124</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="18" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="14"/>
@@ -2087,7 +2139,7 @@
     </row>
     <row r="13">
       <c r="B13" s="18" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C13" s="13">
         <v>31.0</v>
@@ -2126,7 +2178,7 @@
     </row>
     <row r="14">
       <c r="B14" s="18" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C14" s="13">
         <v>28.0</v>
@@ -2137,7 +2189,9 @@
       <c r="G14" s="13">
         <v>21.0</v>
       </c>
-      <c r="H14" s="14"/>
+      <c r="H14" s="14">
+        <v>33.0</v>
+      </c>
       <c r="I14" s="16"/>
       <c r="J14" s="14"/>
       <c r="K14" s="13"/>
@@ -2158,12 +2212,12 @@
       <c r="Z14" s="17"/>
       <c r="AA14" s="15">
         <f t="shared" si="1"/>
-        <v>49</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="18" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C15" s="13">
         <v>23.0</v>
@@ -2178,7 +2232,9 @@
       <c r="G15" s="13">
         <v>21.0</v>
       </c>
-      <c r="H15" s="14"/>
+      <c r="H15" s="14">
+        <v>35.0</v>
+      </c>
       <c r="I15" s="13"/>
       <c r="J15" s="15"/>
       <c r="K15" s="16"/>
@@ -2199,12 +2255,12 @@
       <c r="Z15" s="17"/>
       <c r="AA15" s="15">
         <f t="shared" si="1"/>
-        <v>105</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="18" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="14">
@@ -2219,7 +2275,9 @@
       <c r="G16" s="13">
         <v>32.0</v>
       </c>
-      <c r="H16" s="14"/>
+      <c r="H16" s="14">
+        <v>32.0</v>
+      </c>
       <c r="I16" s="13"/>
       <c r="J16" s="15"/>
       <c r="K16" s="16"/>
@@ -2240,12 +2298,12 @@
       <c r="Z16" s="17"/>
       <c r="AA16" s="15">
         <f t="shared" si="1"/>
-        <v>127</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="18" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C17" s="13">
         <v>20.0</v>
@@ -2262,7 +2320,9 @@
       <c r="G17" s="13">
         <v>20.0</v>
       </c>
-      <c r="H17" s="14"/>
+      <c r="H17" s="14">
+        <v>21.0</v>
+      </c>
       <c r="I17" s="13"/>
       <c r="J17" s="14"/>
       <c r="K17" s="13"/>
@@ -2283,12 +2343,12 @@
       <c r="Z17" s="17"/>
       <c r="AA17" s="15">
         <f t="shared" si="1"/>
-        <v>107</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="18" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C18" s="13">
         <v>32.0</v>
@@ -2303,7 +2363,9 @@
       <c r="G18" s="13">
         <v>39.0</v>
       </c>
-      <c r="H18" s="14"/>
+      <c r="H18" s="14">
+        <v>31.0</v>
+      </c>
       <c r="I18" s="13"/>
       <c r="J18" s="14"/>
       <c r="K18" s="13"/>
@@ -2324,12 +2386,12 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>136</v>
+        <v>167</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="18" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C19" s="13">
         <v>30.0</v>
@@ -2344,7 +2406,9 @@
       <c r="G19" s="13">
         <v>36.0</v>
       </c>
-      <c r="H19" s="14"/>
+      <c r="H19" s="14">
+        <v>33.0</v>
+      </c>
       <c r="I19" s="13"/>
       <c r="J19" s="14"/>
       <c r="K19" s="13"/>
@@ -2365,12 +2429,12 @@
       <c r="Z19" s="17"/>
       <c r="AA19" s="15">
         <f t="shared" si="1"/>
-        <v>122</v>
+        <v>155</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="18" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C20" s="13">
         <v>28.0</v>
@@ -2385,7 +2449,9 @@
       <c r="G20" s="13">
         <v>33.0</v>
       </c>
-      <c r="H20" s="14"/>
+      <c r="H20" s="14">
+        <v>37.0</v>
+      </c>
       <c r="I20" s="13"/>
       <c r="J20" s="14"/>
       <c r="K20" s="13"/>
@@ -2406,12 +2472,12 @@
       <c r="Z20" s="17"/>
       <c r="AA20" s="15">
         <f t="shared" si="1"/>
-        <v>122</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="18" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="14"/>
@@ -2420,7 +2486,9 @@
         <v>36.0</v>
       </c>
       <c r="G21" s="13"/>
-      <c r="H21" s="14"/>
+      <c r="H21" s="14">
+        <v>33.0</v>
+      </c>
       <c r="I21" s="13"/>
       <c r="J21" s="14"/>
       <c r="K21" s="13"/>
@@ -2441,12 +2509,12 @@
       <c r="Z21" s="17"/>
       <c r="AA21" s="15">
         <f t="shared" si="1"/>
-        <v>36</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="18" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C22" s="13">
         <v>20.0</v>
@@ -2463,7 +2531,9 @@
       <c r="G22" s="13">
         <v>36.0</v>
       </c>
-      <c r="H22" s="14"/>
+      <c r="H22" s="14">
+        <v>31.0</v>
+      </c>
       <c r="I22" s="13"/>
       <c r="J22" s="14"/>
       <c r="K22" s="13"/>
@@ -2484,12 +2554,12 @@
       <c r="Z22" s="17"/>
       <c r="AA22" s="15">
         <f t="shared" si="1"/>
-        <v>154</v>
+        <v>185</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="18" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="14"/>
@@ -2500,7 +2570,9 @@
       <c r="G23" s="13">
         <v>40.0</v>
       </c>
-      <c r="H23" s="14"/>
+      <c r="H23" s="14">
+        <v>33.0</v>
+      </c>
       <c r="I23" s="13"/>
       <c r="J23" s="14"/>
       <c r="K23" s="13"/>
@@ -2521,12 +2593,12 @@
       <c r="Z23" s="17"/>
       <c r="AA23" s="15">
         <f t="shared" si="1"/>
-        <v>74</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="18" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C24" s="13"/>
       <c r="D24" s="14">
@@ -2561,7 +2633,7 @@
     </row>
     <row r="25">
       <c r="B25" s="18" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C25" s="13">
         <v>35.0</v>
@@ -2576,7 +2648,9 @@
       <c r="G25" s="13">
         <v>33.0</v>
       </c>
-      <c r="H25" s="14"/>
+      <c r="H25" s="14">
+        <v>35.0</v>
+      </c>
       <c r="I25" s="13"/>
       <c r="J25" s="14"/>
       <c r="K25" s="13"/>
@@ -2597,12 +2671,12 @@
       <c r="Z25" s="17"/>
       <c r="AA25" s="15">
         <f t="shared" si="1"/>
-        <v>126</v>
+        <v>161</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="18" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C26" s="13">
         <v>19.0</v>
@@ -2617,7 +2691,9 @@
       <c r="G26" s="13">
         <v>25.0</v>
       </c>
-      <c r="H26" s="14"/>
+      <c r="H26" s="14">
+        <v>30.0</v>
+      </c>
       <c r="I26" s="13"/>
       <c r="J26" s="14"/>
       <c r="K26" s="13"/>
@@ -2638,7 +2714,7 @@
       <c r="Z26" s="17"/>
       <c r="AA26" s="15">
         <f t="shared" si="1"/>
-        <v>104</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" ht="9.0" customHeight="1">
@@ -2669,24 +2745,26 @@
     </row>
     <row r="28" ht="84.75" customHeight="1">
       <c r="B28" s="23" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C28" s="24" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D28" s="24" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E28" s="24" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F28" s="24" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G28" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="H28" s="24"/>
+        <v>69</v>
+      </c>
+      <c r="H28" s="24" t="s">
+        <v>70</v>
+      </c>
       <c r="I28" s="24"/>
       <c r="J28" s="24"/>
       <c r="K28" s="24"/>
@@ -2709,7 +2787,7 @@
     </row>
     <row r="29">
       <c r="B29" s="26" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C29" s="27">
         <v>35.0</v>
@@ -2726,7 +2804,9 @@
       <c r="G29" s="27">
         <v>40.0</v>
       </c>
-      <c r="H29" s="27"/>
+      <c r="H29" s="27">
+        <v>38.0</v>
+      </c>
       <c r="I29" s="27"/>
       <c r="J29" s="27"/>
       <c r="K29" s="27"/>
@@ -2766,54 +2846,54 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="29" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B1" s="30" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C1" s="31" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="32" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B2" s="33">
+        <v>17.0</v>
+      </c>
+      <c r="C2" s="34">
         <v>16.0</v>
-      </c>
-      <c r="C2" s="34">
-        <v>14.0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="18" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B3" s="33">
+        <v>13.0</v>
+      </c>
+      <c r="C3" s="34">
         <v>12.0</v>
-      </c>
-      <c r="C3" s="34">
-        <v>11.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="18" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B4" s="33">
+        <v>10.0</v>
+      </c>
+      <c r="C4" s="34">
         <v>9.0</v>
-      </c>
-      <c r="C4" s="34">
-        <v>8.0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="18" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B5" s="33">
-        <v>11.0</v>
+        <v>12.0</v>
       </c>
       <c r="C5" s="34">
         <v>10.0</v>
@@ -2821,10 +2901,10 @@
     </row>
     <row r="6">
       <c r="A6" s="18" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B6" s="33">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
       <c r="C6" s="34">
         <v>14.0</v>
@@ -2832,18 +2912,18 @@
     </row>
     <row r="7">
       <c r="A7" s="18" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B7" s="33">
         <v>23.0</v>
       </c>
       <c r="C7" s="34">
-        <v>21.0</v>
+        <v>22.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="18" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B8" s="33">
         <v>33.0</v>
@@ -2854,10 +2934,10 @@
     </row>
     <row r="9">
       <c r="A9" s="18" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B9" s="33">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
       <c r="C9" s="34">
         <v>8.0</v>
@@ -2865,7 +2945,7 @@
     </row>
     <row r="10">
       <c r="A10" s="18" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B10" s="33">
         <v>16.0</v>
@@ -2876,18 +2956,18 @@
     </row>
     <row r="11">
       <c r="A11" s="18" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B11" s="33">
         <v>22.0</v>
       </c>
       <c r="C11" s="34">
-        <v>21.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B12" s="33">
         <v>8.0</v>
@@ -2898,7 +2978,7 @@
     </row>
     <row r="13">
       <c r="A13" s="18" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B13" s="33">
         <v>12.0</v>
@@ -2909,7 +2989,7 @@
     </row>
     <row r="14">
       <c r="A14" s="18" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B14" s="33">
         <v>20.0</v>
@@ -2920,7 +3000,7 @@
     </row>
     <row r="15">
       <c r="A15" s="18" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B15" s="33">
         <v>7.0</v>
@@ -2931,7 +3011,7 @@
     </row>
     <row r="16">
       <c r="A16" s="18" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B16" s="33">
         <v>15.0</v>
@@ -2942,7 +3022,7 @@
     </row>
     <row r="17">
       <c r="A17" s="18" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B17" s="33">
         <v>12.0</v>
@@ -2953,7 +3033,7 @@
     </row>
     <row r="18">
       <c r="A18" s="18" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B18" s="33">
         <v>-1.0</v>
@@ -2964,7 +3044,7 @@
     </row>
     <row r="19">
       <c r="A19" s="18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B19" s="33">
         <v>31.0</v>
@@ -2975,7 +3055,7 @@
     </row>
     <row r="20">
       <c r="A20" s="36" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B20" s="33">
         <v>16.0</v>
@@ -2986,18 +3066,18 @@
     </row>
     <row r="21">
       <c r="A21" s="18" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B21" s="33">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
       <c r="C21" s="34">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="18" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B22" s="33">
         <v>21.0</v>
@@ -3008,7 +3088,7 @@
     </row>
     <row r="23">
       <c r="A23" s="18" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B23" s="33">
         <v>30.0</v>
@@ -3019,7 +3099,7 @@
     </row>
     <row r="24">
       <c r="A24" s="36" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B24" s="33">
         <v>27.0</v>
@@ -3030,7 +3110,7 @@
     </row>
     <row r="25">
       <c r="A25" s="36" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B25" s="33">
         <v>19.0</v>
@@ -3041,7 +3121,7 @@
     </row>
     <row r="26">
       <c r="A26" s="36" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B26" s="14">
         <v>12.0</v>
@@ -3058,23 +3138,23 @@
         <v>15.0</v>
       </c>
       <c r="C27" s="14">
-        <v>13.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="36" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B28" s="14">
-        <v>20.0</v>
+        <v>23.0</v>
       </c>
       <c r="C28" s="14">
-        <v>19.0</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="36" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B29" s="14">
         <v>23.0</v>
@@ -3085,7 +3165,7 @@
     </row>
     <row r="30">
       <c r="A30" s="36" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B30" s="14">
         <v>23.0</v>
@@ -3096,7 +3176,7 @@
     </row>
     <row r="31">
       <c r="A31" s="36" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B31" s="14">
         <v>20.0</v>
@@ -3107,13 +3187,13 @@
     </row>
     <row r="32">
       <c r="A32" s="36" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B32" s="14">
         <v>7.0</v>
       </c>
       <c r="C32" s="14">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="33">
@@ -6991,13 +7071,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B1" s="37" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C1" s="38" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2">
@@ -7005,10 +7085,10 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="40" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C2" s="41" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
@@ -7016,10 +7096,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="42" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C3" s="43" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
@@ -7027,10 +7107,10 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="42" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
@@ -7038,10 +7118,10 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -7049,15 +7129,19 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>80</v>
-      </c>
-      <c r="C6" s="43"/>
+        <v>83</v>
+      </c>
+      <c r="C6" s="43" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="14">
         <v>6.0</v>
       </c>
-      <c r="B7" s="42"/>
+      <c r="B7" s="42" t="s">
+        <v>84</v>
+      </c>
       <c r="C7" s="43"/>
     </row>
     <row r="8">
@@ -12061,19 +12145,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D1" s="44" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2">
@@ -12174,11 +12258,11 @@
       </c>
       <c r="D6" s="46" t="str">
         <f>'THURSDAY SINGLES'!G21</f>
-        <v/>
-      </c>
-      <c r="E6" s="45" t="str">
+        <v>DAVE BARNETT</v>
+      </c>
+      <c r="E6" s="45">
         <f>'THURSDAY SINGLES'!G22</f>
-        <v/>
+        <v>39</v>
       </c>
     </row>
     <row r="7">
@@ -12187,11 +12271,11 @@
       </c>
       <c r="B7" s="45" t="str">
         <f>'SUNDAY SINGLES'!H28</f>
-        <v/>
-      </c>
-      <c r="C7" s="45" t="str">
+        <v>DAVE CROSSLEY</v>
+      </c>
+      <c r="C7" s="45">
         <f>'SUNDAY SINGLES'!H29</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="D7" s="46" t="str">
         <f>'THURSDAY SINGLES'!H21</f>

</xml_diff>

<commit_message>
Week 6/7 data update
</commit_message>
<xml_diff>
--- a/data/SUMMER_GOLF_2026.xlsx
+++ b/data/SUMMER_GOLF_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="90">
   <si>
     <t>SUMMER GOLF 2026 - THURSDAY SINGLES</t>
   </si>
@@ -149,9 +149,6 @@
     <t>SCOTT LEONARDE</t>
   </si>
   <si>
-    <t>JODAN HOWARD</t>
-  </si>
-  <si>
     <t>STEVE CONNOR</t>
   </si>
   <si>
@@ -236,6 +233,9 @@
     <t>YELLOW TEES</t>
   </si>
   <si>
+    <t>JODAN HOWARD</t>
+  </si>
+  <si>
     <t>CHRIS HARVEY</t>
   </si>
   <si>
@@ -270,6 +270,9 @@
   </si>
   <si>
     <t>JOHN ANTCLIFFE/DAVE BARNETT</t>
+  </si>
+  <si>
+    <t>PAUL SHIRLEY</t>
   </si>
   <si>
     <t>SUNDAY</t>
@@ -980,7 +983,9 @@
       <c r="G5" s="13">
         <v>31.0</v>
       </c>
-      <c r="H5" s="14"/>
+      <c r="H5" s="14">
+        <v>35.0</v>
+      </c>
       <c r="I5" s="13"/>
       <c r="J5" s="14"/>
       <c r="K5" s="13"/>
@@ -1000,8 +1005,8 @@
       <c r="Y5" s="16"/>
       <c r="Z5" s="17"/>
       <c r="AA5" s="15">
-        <f t="shared" ref="AA5:AA19" si="1">sum(C5:Z5)</f>
-        <v>115</v>
+        <f t="shared" ref="AA5:AA18" si="1">sum(C5:Z5)</f>
+        <v>150</v>
       </c>
     </row>
     <row r="6">
@@ -1023,7 +1028,9 @@
       <c r="G6" s="13">
         <v>32.0</v>
       </c>
-      <c r="H6" s="14"/>
+      <c r="H6" s="14">
+        <v>33.0</v>
+      </c>
       <c r="I6" s="13"/>
       <c r="J6" s="14"/>
       <c r="K6" s="13"/>
@@ -1044,7 +1051,7 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>148</v>
+        <v>181</v>
       </c>
     </row>
     <row r="7">
@@ -1064,7 +1071,9 @@
       <c r="G7" s="13">
         <v>34.0</v>
       </c>
-      <c r="H7" s="14"/>
+      <c r="H7" s="14">
+        <v>31.0</v>
+      </c>
       <c r="I7" s="13"/>
       <c r="J7" s="14"/>
       <c r="K7" s="16"/>
@@ -1085,7 +1094,7 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>121</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8">
@@ -1107,7 +1116,9 @@
       <c r="G8" s="13">
         <v>36.0</v>
       </c>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14">
+        <v>34.0</v>
+      </c>
       <c r="I8" s="13"/>
       <c r="J8" s="14"/>
       <c r="K8" s="16"/>
@@ -1128,7 +1139,7 @@
       <c r="Z8" s="19"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>165</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9">
@@ -1150,7 +1161,9 @@
       <c r="G9" s="13">
         <v>36.0</v>
       </c>
-      <c r="H9" s="14"/>
+      <c r="H9" s="14">
+        <v>29.0</v>
+      </c>
       <c r="I9" s="13"/>
       <c r="J9" s="14"/>
       <c r="K9" s="13"/>
@@ -1171,7 +1184,7 @@
       <c r="Z9" s="17"/>
       <c r="AA9" s="15">
         <f t="shared" si="1"/>
-        <v>149</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10">
@@ -1191,7 +1204,9 @@
       <c r="G10" s="13">
         <v>39.0</v>
       </c>
-      <c r="H10" s="14"/>
+      <c r="H10" s="14">
+        <v>33.0</v>
+      </c>
       <c r="I10" s="13"/>
       <c r="J10" s="14"/>
       <c r="K10" s="16"/>
@@ -1212,7 +1227,7 @@
       <c r="Z10" s="17"/>
       <c r="AA10" s="15">
         <f t="shared" si="1"/>
-        <v>130</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11">
@@ -1232,7 +1247,9 @@
         <v>29.0</v>
       </c>
       <c r="G11" s="13"/>
-      <c r="H11" s="14"/>
+      <c r="H11" s="14">
+        <v>35.0</v>
+      </c>
       <c r="I11" s="13"/>
       <c r="J11" s="14"/>
       <c r="K11" s="13"/>
@@ -1253,7 +1270,7 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>129</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12">
@@ -1271,7 +1288,9 @@
       <c r="G12" s="13">
         <v>26.0</v>
       </c>
-      <c r="H12" s="14"/>
+      <c r="H12" s="14">
+        <v>36.0</v>
+      </c>
       <c r="I12" s="13"/>
       <c r="J12" s="14"/>
       <c r="K12" s="13"/>
@@ -1292,7 +1311,7 @@
       <c r="Z12" s="17"/>
       <c r="AA12" s="15">
         <f t="shared" si="1"/>
-        <v>80</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13">
@@ -1312,7 +1331,9 @@
       <c r="G13" s="13">
         <v>33.0</v>
       </c>
-      <c r="H13" s="14"/>
+      <c r="H13" s="14">
+        <v>33.0</v>
+      </c>
       <c r="I13" s="13"/>
       <c r="J13" s="14"/>
       <c r="K13" s="13"/>
@@ -1333,7 +1354,7 @@
       <c r="Z13" s="17"/>
       <c r="AA13" s="15">
         <f t="shared" si="1"/>
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14">
@@ -1351,7 +1372,9 @@
       </c>
       <c r="F14" s="14"/>
       <c r="G14" s="13"/>
-      <c r="H14" s="14"/>
+      <c r="H14" s="14">
+        <v>23.0</v>
+      </c>
       <c r="I14" s="13"/>
       <c r="J14" s="14"/>
       <c r="K14" s="13"/>
@@ -1372,7 +1395,7 @@
       <c r="Z14" s="17"/>
       <c r="AA14" s="15">
         <f t="shared" si="1"/>
-        <v>89</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15">
@@ -1425,7 +1448,9 @@
       <c r="E16" s="13"/>
       <c r="F16" s="14"/>
       <c r="G16" s="13"/>
-      <c r="H16" s="14"/>
+      <c r="H16" s="14">
+        <v>21.0</v>
+      </c>
       <c r="I16" s="13"/>
       <c r="J16" s="14"/>
       <c r="K16" s="13"/>
@@ -1446,18 +1471,28 @@
       <c r="Z16" s="17"/>
       <c r="AA16" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="13"/>
+      <c r="C17" s="17">
+        <v>23.0</v>
+      </c>
+      <c r="D17" s="14">
+        <v>21.0</v>
+      </c>
+      <c r="E17" s="13">
+        <v>22.0</v>
+      </c>
+      <c r="F17" s="14">
+        <v>29.0</v>
+      </c>
+      <c r="G17" s="13">
+        <v>29.0</v>
+      </c>
       <c r="H17" s="14"/>
       <c r="I17" s="13"/>
       <c r="J17" s="14"/>
@@ -1479,28 +1514,20 @@
       <c r="Z17" s="17"/>
       <c r="AA17" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="17">
-        <v>23.0</v>
-      </c>
-      <c r="D18" s="14">
-        <v>21.0</v>
-      </c>
-      <c r="E18" s="13">
-        <v>22.0</v>
-      </c>
+      <c r="C18" s="17"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="13"/>
       <c r="F18" s="14">
-        <v>29.0</v>
-      </c>
-      <c r="G18" s="13">
-        <v>29.0</v>
-      </c>
+        <v>27.0</v>
+      </c>
+      <c r="G18" s="13"/>
       <c r="H18" s="14"/>
       <c r="I18" s="13"/>
       <c r="J18" s="14"/>
@@ -1522,148 +1549,117 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>124</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" ht="9.0" customHeight="1">
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="22"/>
+      <c r="N19" s="22"/>
+      <c r="O19" s="22"/>
+      <c r="P19" s="22"/>
+      <c r="Q19" s="22"/>
+      <c r="R19" s="22"/>
+      <c r="S19" s="22"/>
+      <c r="T19" s="22"/>
+      <c r="U19" s="22"/>
+      <c r="V19" s="22"/>
+      <c r="W19" s="22"/>
+      <c r="X19" s="22"/>
+      <c r="Y19" s="22"/>
+      <c r="Z19" s="22"/>
+    </row>
+    <row r="20" ht="72.0" customHeight="1">
+      <c r="B20" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="14">
-        <v>27.0</v>
-      </c>
-      <c r="G19" s="13"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="13"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="15"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="15"/>
-      <c r="O19" s="13"/>
-      <c r="P19" s="14"/>
-      <c r="Q19" s="13"/>
-      <c r="R19" s="14"/>
-      <c r="S19" s="16"/>
-      <c r="T19" s="14"/>
-      <c r="U19" s="13"/>
-      <c r="V19" s="15"/>
-      <c r="W19" s="21"/>
-      <c r="X19" s="15"/>
-      <c r="Y19" s="16"/>
-      <c r="Z19" s="17"/>
-      <c r="AA19" s="15">
-        <f t="shared" si="1"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="20" ht="9.0" customHeight="1">
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
-      <c r="M20" s="22"/>
-      <c r="N20" s="22"/>
-      <c r="O20" s="22"/>
-      <c r="P20" s="22"/>
-      <c r="Q20" s="22"/>
-      <c r="R20" s="22"/>
-      <c r="S20" s="22"/>
-      <c r="T20" s="22"/>
-      <c r="U20" s="22"/>
-      <c r="V20" s="22"/>
-      <c r="W20" s="22"/>
-      <c r="X20" s="22"/>
-      <c r="Y20" s="22"/>
-      <c r="Z20" s="22"/>
-    </row>
-    <row r="21" ht="72.0" customHeight="1">
-      <c r="B21" s="23" t="s">
+      <c r="C20" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="F20" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="D21" s="24" t="s">
-        <v>37</v>
-      </c>
-      <c r="E21" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="F21" s="24" t="s">
+      <c r="G20" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="H20" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24"/>
+      <c r="N20" s="24"/>
+      <c r="O20" s="24"/>
+      <c r="P20" s="24"/>
+      <c r="Q20" s="24"/>
+      <c r="R20" s="24"/>
+      <c r="S20" s="24"/>
+      <c r="T20" s="24"/>
+      <c r="U20" s="24"/>
+      <c r="V20" s="24"/>
+      <c r="W20" s="24"/>
+      <c r="X20" s="24"/>
+      <c r="Y20" s="24"/>
+      <c r="Z20" s="24"/>
+      <c r="AA20" s="25"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="G21" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="H21" s="24"/>
-      <c r="I21" s="24"/>
-      <c r="J21" s="24"/>
-      <c r="K21" s="24"/>
-      <c r="L21" s="24"/>
-      <c r="M21" s="24"/>
-      <c r="N21" s="24"/>
-      <c r="O21" s="24"/>
-      <c r="P21" s="24"/>
-      <c r="Q21" s="24"/>
-      <c r="R21" s="24"/>
-      <c r="S21" s="24"/>
-      <c r="T21" s="24"/>
-      <c r="U21" s="24"/>
-      <c r="V21" s="24"/>
-      <c r="W21" s="24"/>
-      <c r="X21" s="24"/>
-      <c r="Y21" s="24"/>
-      <c r="Z21" s="24"/>
-      <c r="AA21" s="25"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="27">
+      <c r="C21" s="27">
         <v>39.0</v>
       </c>
-      <c r="D22" s="27">
+      <c r="D21" s="27">
         <v>34.0</v>
       </c>
-      <c r="E22" s="27">
+      <c r="E21" s="27">
         <v>33.0</v>
       </c>
-      <c r="F22" s="27">
+      <c r="F21" s="27">
         <v>35.0</v>
       </c>
-      <c r="G22" s="27">
+      <c r="G21" s="27">
         <v>39.0</v>
       </c>
-      <c r="H22" s="27"/>
-      <c r="I22" s="27"/>
-      <c r="J22" s="27"/>
-      <c r="K22" s="27"/>
-      <c r="L22" s="27"/>
-      <c r="M22" s="27"/>
-      <c r="N22" s="27"/>
-      <c r="O22" s="27"/>
-      <c r="P22" s="27"/>
-      <c r="Q22" s="27"/>
-      <c r="R22" s="27"/>
-      <c r="S22" s="27"/>
-      <c r="T22" s="27"/>
-      <c r="U22" s="27"/>
-      <c r="V22" s="27"/>
-      <c r="W22" s="27"/>
-      <c r="X22" s="27"/>
-      <c r="Y22" s="27"/>
-      <c r="Z22" s="27"/>
+      <c r="H21" s="27">
+        <v>36.0</v>
+      </c>
+      <c r="I21" s="27"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="27"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="27"/>
+      <c r="P21" s="27"/>
+      <c r="Q21" s="27"/>
+      <c r="R21" s="27"/>
+      <c r="S21" s="27"/>
+      <c r="T21" s="27"/>
+      <c r="U21" s="27"/>
+      <c r="V21" s="27"/>
+      <c r="W21" s="27"/>
+      <c r="X21" s="27"/>
+      <c r="Y21" s="27"/>
+      <c r="Z21" s="27"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -1685,7 +1681,7 @@
   <sheetData>
     <row r="2" ht="24.0" customHeight="1">
       <c r="B2" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
@@ -1698,10 +1694,10 @@
         <v>46360.0</v>
       </c>
       <c r="E3" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="G3" s="3">
         <v>46086.0</v>
@@ -1710,13 +1706,13 @@
         <v>46300.0</v>
       </c>
       <c r="I3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="J3" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="K3" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>56</v>
       </c>
       <c r="L3" s="4"/>
       <c r="M3" s="5"/>
@@ -1817,7 +1813,7 @@
     </row>
     <row r="5">
       <c r="B5" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C5" s="13">
         <v>24.0</v>
@@ -1850,13 +1846,13 @@
       <c r="Y5" s="16"/>
       <c r="Z5" s="19"/>
       <c r="AA5" s="15">
-        <f t="shared" ref="AA5:AA26" si="1">SUM(C5:Z5)</f>
+        <f t="shared" ref="AA5:AA25" si="1">SUM(C5:Z5)</f>
         <v>80</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C6" s="13">
         <v>28.0</v>
@@ -1919,7 +1915,9 @@
       <c r="H7" s="14">
         <v>36.0</v>
       </c>
-      <c r="I7" s="13"/>
+      <c r="I7" s="13">
+        <v>37.0</v>
+      </c>
       <c r="J7" s="14"/>
       <c r="K7" s="13"/>
       <c r="L7" s="14"/>
@@ -1939,7 +1937,7 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>181</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8">
@@ -1962,7 +1960,9 @@
       <c r="H8" s="14">
         <v>35.0</v>
       </c>
-      <c r="I8" s="13"/>
+      <c r="I8" s="13">
+        <v>31.0</v>
+      </c>
       <c r="J8" s="14"/>
       <c r="K8" s="16"/>
       <c r="L8" s="14"/>
@@ -1982,12 +1982,12 @@
       <c r="Z8" s="17"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>143</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C9" s="13">
         <v>24.0</v>
@@ -2063,7 +2063,7 @@
     </row>
     <row r="11">
       <c r="B11" s="18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="14">
@@ -2081,7 +2081,9 @@
       <c r="H11" s="14">
         <v>32.0</v>
       </c>
-      <c r="I11" s="16"/>
+      <c r="I11" s="13">
+        <v>34.0</v>
+      </c>
       <c r="J11" s="15"/>
       <c r="K11" s="13"/>
       <c r="L11" s="15"/>
@@ -2101,108 +2103,120 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>156</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" s="13"/>
-      <c r="D12" s="14"/>
+        <v>46</v>
+      </c>
+      <c r="C12" s="13">
+        <v>31.0</v>
+      </c>
+      <c r="D12" s="14">
+        <v>28.0</v>
+      </c>
       <c r="E12" s="13"/>
       <c r="F12" s="14"/>
-      <c r="G12" s="13"/>
+      <c r="G12" s="13">
+        <v>26.0</v>
+      </c>
       <c r="H12" s="14"/>
-      <c r="I12" s="13"/>
+      <c r="I12" s="16"/>
       <c r="J12" s="14"/>
       <c r="K12" s="13"/>
       <c r="L12" s="14"/>
       <c r="M12" s="13"/>
       <c r="N12" s="14"/>
-      <c r="O12" s="16"/>
-      <c r="P12" s="14"/>
-      <c r="Q12" s="16"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="15"/>
+      <c r="Q12" s="13"/>
       <c r="R12" s="15"/>
-      <c r="S12" s="13"/>
-      <c r="T12" s="15"/>
+      <c r="S12" s="16"/>
+      <c r="T12" s="14"/>
       <c r="U12" s="13"/>
-      <c r="V12" s="15"/>
+      <c r="V12" s="14"/>
       <c r="W12" s="13"/>
-      <c r="X12" s="14"/>
+      <c r="X12" s="15"/>
       <c r="Y12" s="13"/>
       <c r="Z12" s="17"/>
       <c r="AA12" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="18" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="C13" s="13">
-        <v>31.0</v>
-      </c>
-      <c r="D13" s="14">
         <v>28.0</v>
       </c>
+      <c r="D13" s="14"/>
       <c r="E13" s="13"/>
       <c r="F13" s="14"/>
       <c r="G13" s="13">
-        <v>26.0</v>
-      </c>
-      <c r="H13" s="14"/>
-      <c r="I13" s="16"/>
+        <v>21.0</v>
+      </c>
+      <c r="H13" s="14">
+        <v>33.0</v>
+      </c>
+      <c r="I13" s="13">
+        <v>33.0</v>
+      </c>
       <c r="J13" s="14"/>
       <c r="K13" s="13"/>
       <c r="L13" s="14"/>
       <c r="M13" s="13"/>
       <c r="N13" s="14"/>
       <c r="O13" s="13"/>
-      <c r="P13" s="15"/>
+      <c r="P13" s="14"/>
       <c r="Q13" s="13"/>
-      <c r="R13" s="15"/>
+      <c r="R13" s="14"/>
       <c r="S13" s="16"/>
-      <c r="T13" s="14"/>
+      <c r="T13" s="15"/>
       <c r="U13" s="13"/>
       <c r="V13" s="14"/>
       <c r="W13" s="13"/>
-      <c r="X13" s="15"/>
+      <c r="X13" s="14"/>
       <c r="Y13" s="13"/>
       <c r="Z13" s="17"/>
       <c r="AA13" s="15">
         <f t="shared" si="1"/>
-        <v>85</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="18" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="C14" s="13">
-        <v>28.0</v>
-      </c>
-      <c r="D14" s="14"/>
+        <v>23.0</v>
+      </c>
+      <c r="D14" s="14">
+        <v>34.0</v>
+      </c>
       <c r="E14" s="13"/>
-      <c r="F14" s="14"/>
+      <c r="F14" s="14">
+        <v>27.0</v>
+      </c>
       <c r="G14" s="13">
         <v>21.0</v>
       </c>
       <c r="H14" s="14">
-        <v>33.0</v>
-      </c>
-      <c r="I14" s="16"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="13"/>
+        <v>35.0</v>
+      </c>
+      <c r="I14" s="13"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="16"/>
       <c r="L14" s="14"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="14"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="14"/>
+      <c r="M14" s="16"/>
+      <c r="N14" s="15"/>
+      <c r="O14" s="16"/>
+      <c r="P14" s="15"/>
       <c r="Q14" s="13"/>
       <c r="R14" s="14"/>
-      <c r="S14" s="16"/>
+      <c r="S14" s="13"/>
       <c r="T14" s="15"/>
       <c r="U14" s="13"/>
       <c r="V14" s="14"/>
@@ -2212,37 +2226,39 @@
       <c r="Z14" s="17"/>
       <c r="AA14" s="15">
         <f t="shared" si="1"/>
-        <v>82</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="13">
-        <v>23.0</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="C15" s="13"/>
       <c r="D15" s="14">
-        <v>34.0</v>
-      </c>
-      <c r="E15" s="13"/>
+        <v>27.0</v>
+      </c>
+      <c r="E15" s="13">
+        <v>37.0</v>
+      </c>
       <c r="F15" s="14">
+        <v>31.0</v>
+      </c>
+      <c r="G15" s="13">
+        <v>32.0</v>
+      </c>
+      <c r="H15" s="14">
+        <v>32.0</v>
+      </c>
+      <c r="I15" s="13">
         <v>27.0</v>
       </c>
-      <c r="G15" s="13">
-        <v>21.0</v>
-      </c>
-      <c r="H15" s="14">
-        <v>35.0</v>
-      </c>
-      <c r="I15" s="13"/>
       <c r="J15" s="15"/>
       <c r="K15" s="16"/>
-      <c r="L15" s="14"/>
+      <c r="L15" s="15"/>
       <c r="M15" s="16"/>
-      <c r="N15" s="15"/>
-      <c r="O15" s="16"/>
-      <c r="P15" s="15"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="13"/>
+      <c r="P15" s="14"/>
       <c r="Q15" s="13"/>
       <c r="R15" s="14"/>
       <c r="S15" s="13"/>
@@ -2255,41 +2271,45 @@
       <c r="Z15" s="17"/>
       <c r="AA15" s="15">
         <f t="shared" si="1"/>
-        <v>140</v>
+        <v>186</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" s="13"/>
+        <v>45</v>
+      </c>
+      <c r="C16" s="13">
+        <v>20.0</v>
+      </c>
       <c r="D16" s="14">
-        <v>27.0</v>
+        <v>19.0</v>
       </c>
       <c r="E16" s="13">
-        <v>37.0</v>
+        <v>26.0</v>
       </c>
       <c r="F16" s="14">
-        <v>31.0</v>
+        <v>22.0</v>
       </c>
       <c r="G16" s="13">
-        <v>32.0</v>
+        <v>20.0</v>
       </c>
       <c r="H16" s="14">
-        <v>32.0</v>
-      </c>
-      <c r="I16" s="13"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="16"/>
-      <c r="L16" s="15"/>
-      <c r="M16" s="16"/>
+        <v>21.0</v>
+      </c>
+      <c r="I16" s="13">
+        <v>19.0</v>
+      </c>
+      <c r="J16" s="14"/>
+      <c r="K16" s="13"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="13"/>
       <c r="N16" s="14"/>
       <c r="O16" s="13"/>
-      <c r="P16" s="14"/>
+      <c r="P16" s="15"/>
       <c r="Q16" s="13"/>
       <c r="R16" s="14"/>
       <c r="S16" s="13"/>
-      <c r="T16" s="15"/>
+      <c r="T16" s="14"/>
       <c r="U16" s="13"/>
       <c r="V16" s="14"/>
       <c r="W16" s="13"/>
@@ -2298,30 +2318,28 @@
       <c r="Z16" s="17"/>
       <c r="AA16" s="15">
         <f t="shared" si="1"/>
-        <v>159</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="18" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="C17" s="13">
-        <v>20.0</v>
-      </c>
-      <c r="D17" s="14">
-        <v>19.0</v>
-      </c>
+        <v>32.0</v>
+      </c>
+      <c r="D17" s="14"/>
       <c r="E17" s="13">
-        <v>26.0</v>
+        <v>32.0</v>
       </c>
       <c r="F17" s="14">
-        <v>22.0</v>
+        <v>33.0</v>
       </c>
       <c r="G17" s="13">
-        <v>20.0</v>
+        <v>39.0</v>
       </c>
       <c r="H17" s="14">
-        <v>21.0</v>
+        <v>31.0</v>
       </c>
       <c r="I17" s="13"/>
       <c r="J17" s="14"/>
@@ -2330,10 +2348,10 @@
       <c r="M17" s="13"/>
       <c r="N17" s="14"/>
       <c r="O17" s="13"/>
-      <c r="P17" s="15"/>
+      <c r="P17" s="14"/>
       <c r="Q17" s="13"/>
-      <c r="R17" s="14"/>
-      <c r="S17" s="13"/>
+      <c r="R17" s="15"/>
+      <c r="S17" s="16"/>
       <c r="T17" s="14"/>
       <c r="U17" s="13"/>
       <c r="V17" s="14"/>
@@ -2343,7 +2361,7 @@
       <c r="Z17" s="17"/>
       <c r="AA17" s="15">
         <f t="shared" si="1"/>
-        <v>128</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18">
@@ -2351,33 +2369,33 @@
         <v>62</v>
       </c>
       <c r="C18" s="13">
-        <v>32.0</v>
-      </c>
-      <c r="D18" s="14"/>
+        <v>30.0</v>
+      </c>
+      <c r="D18" s="14">
+        <v>30.0</v>
+      </c>
       <c r="E18" s="13">
-        <v>32.0</v>
-      </c>
-      <c r="F18" s="14">
+        <v>26.0</v>
+      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="13">
+        <v>36.0</v>
+      </c>
+      <c r="H18" s="14">
         <v>33.0</v>
-      </c>
-      <c r="G18" s="13">
-        <v>39.0</v>
-      </c>
-      <c r="H18" s="14">
-        <v>31.0</v>
       </c>
       <c r="I18" s="13"/>
       <c r="J18" s="14"/>
       <c r="K18" s="13"/>
       <c r="L18" s="14"/>
       <c r="M18" s="13"/>
-      <c r="N18" s="14"/>
-      <c r="O18" s="13"/>
-      <c r="P18" s="14"/>
+      <c r="N18" s="15"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="15"/>
       <c r="Q18" s="13"/>
-      <c r="R18" s="15"/>
-      <c r="S18" s="16"/>
-      <c r="T18" s="14"/>
+      <c r="R18" s="14"/>
+      <c r="S18" s="13"/>
+      <c r="T18" s="15"/>
       <c r="U18" s="13"/>
       <c r="V18" s="14"/>
       <c r="W18" s="13"/>
@@ -2386,7 +2404,7 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>167</v>
+        <v>155</v>
       </c>
     </row>
     <row r="19">
@@ -2394,33 +2412,35 @@
         <v>63</v>
       </c>
       <c r="C19" s="13">
+        <v>28.0</v>
+      </c>
+      <c r="D19" s="14"/>
+      <c r="E19" s="13">
         <v>30.0</v>
       </c>
-      <c r="D19" s="14">
-        <v>30.0</v>
-      </c>
-      <c r="E19" s="13">
-        <v>26.0</v>
-      </c>
-      <c r="F19" s="14"/>
+      <c r="F19" s="14">
+        <v>31.0</v>
+      </c>
       <c r="G19" s="13">
-        <v>36.0</v>
+        <v>33.0</v>
       </c>
       <c r="H19" s="14">
-        <v>33.0</v>
-      </c>
-      <c r="I19" s="13"/>
+        <v>37.0</v>
+      </c>
+      <c r="I19" s="13">
+        <v>27.0</v>
+      </c>
       <c r="J19" s="14"/>
       <c r="K19" s="13"/>
       <c r="L19" s="14"/>
       <c r="M19" s="13"/>
-      <c r="N19" s="15"/>
-      <c r="O19" s="16"/>
+      <c r="N19" s="14"/>
+      <c r="O19" s="13"/>
       <c r="P19" s="15"/>
       <c r="Q19" s="13"/>
       <c r="R19" s="14"/>
       <c r="S19" s="13"/>
-      <c r="T19" s="15"/>
+      <c r="T19" s="14"/>
       <c r="U19" s="13"/>
       <c r="V19" s="14"/>
       <c r="W19" s="13"/>
@@ -2429,30 +2449,26 @@
       <c r="Z19" s="17"/>
       <c r="AA19" s="15">
         <f t="shared" si="1"/>
-        <v>155</v>
+        <v>186</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="C20" s="13">
-        <v>28.0</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="C20" s="13"/>
       <c r="D20" s="14"/>
-      <c r="E20" s="13">
+      <c r="E20" s="13"/>
+      <c r="F20" s="14">
+        <v>36.0</v>
+      </c>
+      <c r="G20" s="13"/>
+      <c r="H20" s="14">
+        <v>33.0</v>
+      </c>
+      <c r="I20" s="13">
         <v>30.0</v>
       </c>
-      <c r="F20" s="14">
-        <v>31.0</v>
-      </c>
-      <c r="G20" s="13">
-        <v>33.0</v>
-      </c>
-      <c r="H20" s="14">
-        <v>37.0</v>
-      </c>
-      <c r="I20" s="13"/>
       <c r="J20" s="14"/>
       <c r="K20" s="13"/>
       <c r="L20" s="14"/>
@@ -2472,24 +2488,34 @@
       <c r="Z20" s="17"/>
       <c r="AA20" s="15">
         <f t="shared" si="1"/>
-        <v>159</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="13"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="13"/>
+        <v>64</v>
+      </c>
+      <c r="C21" s="13">
+        <v>20.0</v>
+      </c>
+      <c r="D21" s="14">
+        <v>39.0</v>
+      </c>
+      <c r="E21" s="13">
+        <v>27.0</v>
+      </c>
       <c r="F21" s="14">
+        <v>32.0</v>
+      </c>
+      <c r="G21" s="13">
         <v>36.0</v>
       </c>
-      <c r="G21" s="13"/>
       <c r="H21" s="14">
-        <v>33.0</v>
-      </c>
-      <c r="I21" s="13"/>
+        <v>31.0</v>
+      </c>
+      <c r="I21" s="13">
+        <v>28.0</v>
+      </c>
       <c r="J21" s="14"/>
       <c r="K21" s="13"/>
       <c r="L21" s="14"/>
@@ -2509,30 +2535,24 @@
       <c r="Z21" s="17"/>
       <c r="AA21" s="15">
         <f t="shared" si="1"/>
-        <v>69</v>
+        <v>213</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="C22" s="13">
-        <v>20.0</v>
-      </c>
-      <c r="D22" s="14">
-        <v>39.0</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="C22" s="13"/>
+      <c r="D22" s="14"/>
       <c r="E22" s="13">
-        <v>27.0</v>
-      </c>
-      <c r="F22" s="14">
-        <v>32.0</v>
-      </c>
+        <v>34.0</v>
+      </c>
+      <c r="F22" s="15"/>
       <c r="G22" s="13">
-        <v>36.0</v>
+        <v>40.0</v>
       </c>
       <c r="H22" s="14">
-        <v>31.0</v>
+        <v>33.0</v>
       </c>
       <c r="I22" s="13"/>
       <c r="J22" s="14"/>
@@ -2554,25 +2574,21 @@
       <c r="Z22" s="17"/>
       <c r="AA22" s="15">
         <f t="shared" si="1"/>
-        <v>185</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="18" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="C23" s="13"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="13">
-        <v>34.0</v>
-      </c>
+      <c r="D23" s="14">
+        <v>25.0</v>
+      </c>
+      <c r="E23" s="13"/>
       <c r="F23" s="15"/>
-      <c r="G23" s="13">
-        <v>40.0</v>
-      </c>
-      <c r="H23" s="14">
-        <v>33.0</v>
-      </c>
+      <c r="G23" s="13"/>
+      <c r="H23" s="14"/>
       <c r="I23" s="13"/>
       <c r="J23" s="14"/>
       <c r="K23" s="13"/>
@@ -2593,22 +2609,32 @@
       <c r="Z23" s="17"/>
       <c r="AA23" s="15">
         <f t="shared" si="1"/>
-        <v>107</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="13"/>
+      <c r="C24" s="13">
+        <v>35.0</v>
+      </c>
       <c r="D24" s="14">
         <v>25.0</v>
       </c>
-      <c r="E24" s="13"/>
+      <c r="E24" s="13">
+        <v>33.0</v>
+      </c>
       <c r="F24" s="15"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="13"/>
+      <c r="G24" s="13">
+        <v>33.0</v>
+      </c>
+      <c r="H24" s="14">
+        <v>35.0</v>
+      </c>
+      <c r="I24" s="13">
+        <v>35.0</v>
+      </c>
       <c r="J24" s="14"/>
       <c r="K24" s="13"/>
       <c r="L24" s="14"/>
@@ -2628,7 +2654,7 @@
       <c r="Z24" s="17"/>
       <c r="AA24" s="15">
         <f t="shared" si="1"/>
-        <v>25</v>
+        <v>196</v>
       </c>
     </row>
     <row r="25">
@@ -2636,22 +2662,24 @@
         <v>67</v>
       </c>
       <c r="C25" s="13">
-        <v>35.0</v>
-      </c>
-      <c r="D25" s="14">
+        <v>19.0</v>
+      </c>
+      <c r="D25" s="14"/>
+      <c r="E25" s="13">
+        <v>29.0</v>
+      </c>
+      <c r="F25" s="14">
+        <v>31.0</v>
+      </c>
+      <c r="G25" s="13">
         <v>25.0</v>
       </c>
-      <c r="E25" s="13">
-        <v>33.0</v>
-      </c>
-      <c r="F25" s="15"/>
-      <c r="G25" s="13">
-        <v>33.0</v>
-      </c>
       <c r="H25" s="14">
-        <v>35.0</v>
-      </c>
-      <c r="I25" s="13"/>
+        <v>30.0</v>
+      </c>
+      <c r="I25" s="13">
+        <v>34.0</v>
+      </c>
       <c r="J25" s="14"/>
       <c r="K25" s="13"/>
       <c r="L25" s="14"/>
@@ -2671,161 +2699,122 @@
       <c r="Z25" s="17"/>
       <c r="AA25" s="15">
         <f t="shared" si="1"/>
-        <v>161</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="18" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="26" ht="9.0" customHeight="1">
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="22"/>
+      <c r="J26" s="22"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="22"/>
+      <c r="M26" s="22"/>
+      <c r="N26" s="22"/>
+      <c r="O26" s="22"/>
+      <c r="P26" s="22"/>
+      <c r="Q26" s="22"/>
+      <c r="R26" s="22"/>
+      <c r="S26" s="22"/>
+      <c r="T26" s="22"/>
+      <c r="U26" s="22"/>
+      <c r="V26" s="22"/>
+      <c r="W26" s="22"/>
+      <c r="X26" s="22"/>
+      <c r="Y26" s="22"/>
+      <c r="Z26" s="22"/>
+    </row>
+    <row r="27" ht="84.75" customHeight="1">
+      <c r="B27" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E27" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="F27" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G27" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="C26" s="13">
-        <v>19.0</v>
-      </c>
-      <c r="D26" s="14"/>
-      <c r="E26" s="13">
-        <v>29.0</v>
-      </c>
-      <c r="F26" s="14">
-        <v>31.0</v>
-      </c>
-      <c r="G26" s="13">
-        <v>25.0</v>
-      </c>
-      <c r="H26" s="14">
-        <v>30.0</v>
-      </c>
-      <c r="I26" s="13"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="13"/>
-      <c r="L26" s="14"/>
-      <c r="M26" s="13"/>
-      <c r="N26" s="14"/>
-      <c r="O26" s="13"/>
-      <c r="P26" s="15"/>
-      <c r="Q26" s="13"/>
-      <c r="R26" s="14"/>
-      <c r="S26" s="13"/>
-      <c r="T26" s="14"/>
-      <c r="U26" s="13"/>
-      <c r="V26" s="14"/>
-      <c r="W26" s="13"/>
-      <c r="X26" s="14"/>
-      <c r="Y26" s="13"/>
-      <c r="Z26" s="17"/>
-      <c r="AA26" s="15">
-        <f t="shared" si="1"/>
-        <v>134</v>
-      </c>
-    </row>
-    <row r="27" ht="9.0" customHeight="1">
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="22"/>
-      <c r="K27" s="22"/>
-      <c r="L27" s="22"/>
-      <c r="M27" s="22"/>
-      <c r="N27" s="22"/>
-      <c r="O27" s="22"/>
-      <c r="P27" s="22"/>
-      <c r="Q27" s="22"/>
-      <c r="R27" s="22"/>
-      <c r="S27" s="22"/>
-      <c r="T27" s="22"/>
-      <c r="U27" s="22"/>
-      <c r="V27" s="22"/>
-      <c r="W27" s="22"/>
-      <c r="X27" s="22"/>
-      <c r="Y27" s="22"/>
-      <c r="Z27" s="22"/>
-    </row>
-    <row r="28" ht="84.75" customHeight="1">
-      <c r="B28" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="C28" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="D28" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="E28" s="24" t="s">
-        <v>37</v>
-      </c>
-      <c r="F28" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="G28" s="24" t="s">
+      <c r="H27" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="H28" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="I28" s="24"/>
-      <c r="J28" s="24"/>
-      <c r="K28" s="24"/>
-      <c r="L28" s="24"/>
-      <c r="M28" s="24"/>
-      <c r="N28" s="24"/>
-      <c r="O28" s="24"/>
-      <c r="P28" s="24"/>
-      <c r="Q28" s="24"/>
-      <c r="R28" s="24"/>
-      <c r="S28" s="24"/>
-      <c r="T28" s="24"/>
-      <c r="U28" s="24"/>
-      <c r="V28" s="24"/>
-      <c r="W28" s="24"/>
-      <c r="X28" s="24"/>
-      <c r="Y28" s="24"/>
-      <c r="Z28" s="24"/>
-      <c r="AA28" s="28"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="C29" s="27">
+      <c r="I27" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="J27" s="24"/>
+      <c r="K27" s="24"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="24"/>
+      <c r="N27" s="24"/>
+      <c r="O27" s="24"/>
+      <c r="P27" s="24"/>
+      <c r="Q27" s="24"/>
+      <c r="R27" s="24"/>
+      <c r="S27" s="24"/>
+      <c r="T27" s="24"/>
+      <c r="U27" s="24"/>
+      <c r="V27" s="24"/>
+      <c r="W27" s="24"/>
+      <c r="X27" s="24"/>
+      <c r="Y27" s="24"/>
+      <c r="Z27" s="24"/>
+      <c r="AA27" s="28"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="27">
         <v>35.0</v>
       </c>
-      <c r="D29" s="27">
+      <c r="D28" s="27">
         <v>39.0</v>
       </c>
-      <c r="E29" s="27">
+      <c r="E28" s="27">
         <v>37.0</v>
       </c>
-      <c r="F29" s="27">
+      <c r="F28" s="27">
         <v>36.0</v>
       </c>
-      <c r="G29" s="27">
+      <c r="G28" s="27">
         <v>40.0</v>
       </c>
-      <c r="H29" s="27">
+      <c r="H28" s="27">
         <v>38.0</v>
       </c>
-      <c r="I29" s="27"/>
-      <c r="J29" s="27"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="27"/>
-      <c r="M29" s="27"/>
-      <c r="N29" s="27"/>
-      <c r="O29" s="27"/>
-      <c r="P29" s="27"/>
-      <c r="Q29" s="27"/>
-      <c r="R29" s="27"/>
-      <c r="S29" s="27"/>
-      <c r="T29" s="27"/>
-      <c r="U29" s="27"/>
-      <c r="V29" s="27"/>
-      <c r="W29" s="27"/>
-      <c r="X29" s="27"/>
-      <c r="Y29" s="27"/>
-      <c r="Z29" s="27"/>
-      <c r="AA29" s="15"/>
+      <c r="I28" s="27">
+        <v>37.0</v>
+      </c>
+      <c r="J28" s="27"/>
+      <c r="K28" s="27"/>
+      <c r="L28" s="27"/>
+      <c r="M28" s="27"/>
+      <c r="N28" s="27"/>
+      <c r="O28" s="27"/>
+      <c r="P28" s="27"/>
+      <c r="Q28" s="27"/>
+      <c r="R28" s="27"/>
+      <c r="S28" s="27"/>
+      <c r="T28" s="27"/>
+      <c r="U28" s="27"/>
+      <c r="V28" s="27"/>
+      <c r="W28" s="27"/>
+      <c r="X28" s="27"/>
+      <c r="Y28" s="27"/>
+      <c r="Z28" s="27"/>
+      <c r="AA28" s="15"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -2849,15 +2838,15 @@
         <v>7</v>
       </c>
       <c r="B1" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="31" t="s">
         <v>71</v>
-      </c>
-      <c r="C1" s="31" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="32" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B2" s="33">
         <v>17.0</v>
@@ -2871,7 +2860,7 @@
         <v>33</v>
       </c>
       <c r="B3" s="33">
-        <v>13.0</v>
+        <v>14.0</v>
       </c>
       <c r="C3" s="34">
         <v>12.0</v>
@@ -2879,7 +2868,7 @@
     </row>
     <row r="4">
       <c r="A4" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B4" s="33">
         <v>10.0</v>
@@ -2893,7 +2882,7 @@
         <v>35</v>
       </c>
       <c r="B5" s="33">
-        <v>12.0</v>
+        <v>11.0</v>
       </c>
       <c r="C5" s="34">
         <v>10.0</v>
@@ -2907,7 +2896,7 @@
         <v>16.0</v>
       </c>
       <c r="C6" s="34">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="7">
@@ -2926,7 +2915,7 @@
         <v>37</v>
       </c>
       <c r="B8" s="33">
-        <v>33.0</v>
+        <v>32.0</v>
       </c>
       <c r="C8" s="34">
         <v>31.0</v>
@@ -2934,7 +2923,7 @@
     </row>
     <row r="9">
       <c r="A9" s="18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B9" s="33">
         <v>9.0</v>
@@ -2945,7 +2934,7 @@
     </row>
     <row r="10">
       <c r="A10" s="18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" s="33">
         <v>16.0</v>
@@ -2956,7 +2945,7 @@
     </row>
     <row r="11">
       <c r="A11" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B11" s="33">
         <v>22.0</v>
@@ -2970,15 +2959,15 @@
         <v>40</v>
       </c>
       <c r="B12" s="33">
-        <v>8.0</v>
+        <v>9.0</v>
       </c>
       <c r="C12" s="35">
-        <v>6.0</v>
+        <v>7.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B13" s="33">
         <v>12.0</v>
@@ -2989,7 +2978,7 @@
     </row>
     <row r="14">
       <c r="A14" s="18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B14" s="33">
         <v>20.0</v>
@@ -3000,7 +2989,7 @@
     </row>
     <row r="15">
       <c r="A15" s="18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B15" s="33">
         <v>7.0</v>
@@ -3011,7 +3000,7 @@
     </row>
     <row r="16">
       <c r="A16" s="18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B16" s="33">
         <v>15.0</v>
@@ -3033,7 +3022,7 @@
     </row>
     <row r="18">
       <c r="A18" s="18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B18" s="33">
         <v>-1.0</v>
@@ -3058,15 +3047,15 @@
         <v>38</v>
       </c>
       <c r="B20" s="33">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
       <c r="C20" s="34">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B21" s="33">
         <v>7.0</v>
@@ -3077,7 +3066,7 @@
     </row>
     <row r="22">
       <c r="A22" s="18" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="B22" s="33">
         <v>21.0</v>
@@ -3088,18 +3077,18 @@
     </row>
     <row r="23">
       <c r="A23" s="18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23" s="33">
-        <v>30.0</v>
+        <v>33.0</v>
       </c>
       <c r="C23" s="34">
-        <v>29.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="36" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B24" s="33">
         <v>27.0</v>
@@ -3110,7 +3099,7 @@
     </row>
     <row r="25">
       <c r="A25" s="36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B25" s="33">
         <v>19.0</v>
@@ -3124,7 +3113,7 @@
         <v>73</v>
       </c>
       <c r="B26" s="14">
-        <v>12.0</v>
+        <v>13.0</v>
       </c>
       <c r="C26" s="14">
         <v>11.0</v>
@@ -3132,7 +3121,7 @@
     </row>
     <row r="27">
       <c r="A27" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B27" s="14">
         <v>15.0</v>
@@ -3143,7 +3132,7 @@
     </row>
     <row r="28">
       <c r="A28" s="36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B28" s="14">
         <v>23.0</v>
@@ -3154,7 +3143,7 @@
     </row>
     <row r="29">
       <c r="A29" s="36" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B29" s="14">
         <v>23.0</v>
@@ -3193,7 +3182,7 @@
         <v>7.0</v>
       </c>
       <c r="C32" s="14">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="33">
@@ -7121,7 +7110,7 @@
         <v>82</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -7142,13 +7131,17 @@
       <c r="B7" s="42" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="43"/>
+      <c r="C7" s="43" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="14">
         <v>7.0</v>
       </c>
-      <c r="B8" s="42"/>
+      <c r="B8" s="42" t="s">
+        <v>85</v>
+      </c>
       <c r="C8" s="43"/>
     </row>
     <row r="9">
@@ -12148,16 +12141,16 @@
         <v>76</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D1" s="44" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2">
@@ -12165,19 +12158,19 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="45" t="str">
+        <f>'SUNDAY SINGLES'!C27</f>
+        <v>PAUL HANCOX</v>
+      </c>
+      <c r="C2" s="45">
         <f>'SUNDAY SINGLES'!C28</f>
-        <v>PAUL HANCOX</v>
-      </c>
-      <c r="C2" s="45">
-        <f>'SUNDAY SINGLES'!C29</f>
         <v>35</v>
       </c>
       <c r="D2" s="46" t="str">
+        <f>'THURSDAY SINGLES'!C20</f>
+        <v>MARTIN BROCK</v>
+      </c>
+      <c r="E2" s="45">
         <f>'THURSDAY SINGLES'!C21</f>
-        <v>MARTIN BROCK</v>
-      </c>
-      <c r="E2" s="45">
-        <f>'THURSDAY SINGLES'!C22</f>
         <v>39</v>
       </c>
     </row>
@@ -12186,19 +12179,19 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="45" t="str">
+        <f>'SUNDAY SINGLES'!D27</f>
+        <v>ARTHUR YOUNG</v>
+      </c>
+      <c r="C3" s="45">
         <f>'SUNDAY SINGLES'!D28</f>
-        <v>ARTHUR YOUNG</v>
-      </c>
-      <c r="C3" s="45">
-        <f>'SUNDAY SINGLES'!D29</f>
         <v>39</v>
       </c>
       <c r="D3" s="46" t="str">
+        <f>'THURSDAY SINGLES'!D20</f>
+        <v>KEN PEEL</v>
+      </c>
+      <c r="E3" s="45">
         <f>'THURSDAY SINGLES'!D21</f>
-        <v>KEN PEEL</v>
-      </c>
-      <c r="E3" s="45">
-        <f>'THURSDAY SINGLES'!D22</f>
         <v>34</v>
       </c>
     </row>
@@ -12207,19 +12200,19 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="45" t="str">
+        <f>'SUNDAY SINGLES'!E27</f>
+        <v>KEN PEEL</v>
+      </c>
+      <c r="C4" s="45">
         <f>'SUNDAY SINGLES'!E28</f>
-        <v>KEN PEEL</v>
-      </c>
-      <c r="C4" s="45">
-        <f>'SUNDAY SINGLES'!E29</f>
         <v>37</v>
       </c>
       <c r="D4" s="46" t="str">
+        <f>'THURSDAY SINGLES'!E20</f>
+        <v>SCOTT LEONARDE</v>
+      </c>
+      <c r="E4" s="45">
         <f>'THURSDAY SINGLES'!E21</f>
-        <v>SCOTT LEONARDE</v>
-      </c>
-      <c r="E4" s="45">
-        <f>'THURSDAY SINGLES'!E22</f>
         <v>33</v>
       </c>
     </row>
@@ -12228,19 +12221,19 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="45" t="str">
+        <f>'SUNDAY SINGLES'!F27</f>
+        <v>SCOTT LEONARDE</v>
+      </c>
+      <c r="C5" s="45">
         <f>'SUNDAY SINGLES'!F28</f>
-        <v>SCOTT LEONARDE</v>
-      </c>
-      <c r="C5" s="45">
-        <f>'SUNDAY SINGLES'!F29</f>
         <v>36</v>
       </c>
       <c r="D5" s="46" t="str">
+        <f>'THURSDAY SINGLES'!F20</f>
+        <v>STEVE  FELLOWS</v>
+      </c>
+      <c r="E5" s="45">
         <f>'THURSDAY SINGLES'!F21</f>
-        <v>STEVE  FELLOWS</v>
-      </c>
-      <c r="E5" s="45">
-        <f>'THURSDAY SINGLES'!F22</f>
         <v>35</v>
       </c>
     </row>
@@ -12249,19 +12242,19 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="45" t="str">
+        <f>'SUNDAY SINGLES'!G27</f>
+        <v>STEW TAYLOR</v>
+      </c>
+      <c r="C6" s="45">
         <f>'SUNDAY SINGLES'!G28</f>
-        <v>STEW TAYLOR</v>
-      </c>
-      <c r="C6" s="45">
-        <f>'SUNDAY SINGLES'!G29</f>
         <v>40</v>
       </c>
       <c r="D6" s="46" t="str">
+        <f>'THURSDAY SINGLES'!G20</f>
+        <v>DAVE BARNETT</v>
+      </c>
+      <c r="E6" s="45">
         <f>'THURSDAY SINGLES'!G21</f>
-        <v>DAVE BARNETT</v>
-      </c>
-      <c r="E6" s="45">
-        <f>'THURSDAY SINGLES'!G22</f>
         <v>39</v>
       </c>
     </row>
@@ -12270,20 +12263,20 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="45" t="str">
+        <f>'SUNDAY SINGLES'!H27</f>
+        <v>DAVE CROSSLEY</v>
+      </c>
+      <c r="C7" s="45">
         <f>'SUNDAY SINGLES'!H28</f>
-        <v>DAVE CROSSLEY</v>
-      </c>
-      <c r="C7" s="45">
-        <f>'SUNDAY SINGLES'!H29</f>
         <v>38</v>
       </c>
       <c r="D7" s="46" t="str">
+        <f>'THURSDAY SINGLES'!H20</f>
+        <v>ALBIE GILLESPIE</v>
+      </c>
+      <c r="E7" s="45">
         <f>'THURSDAY SINGLES'!H21</f>
-        <v/>
-      </c>
-      <c r="E7" s="45" t="str">
-        <f>'THURSDAY SINGLES'!H22</f>
-        <v/>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
@@ -12291,19 +12284,19 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="45" t="str">
+        <f>'SUNDAY SINGLES'!I27</f>
+        <v>LES DOBBINS</v>
+      </c>
+      <c r="C8" s="45">
         <f>'SUNDAY SINGLES'!I28</f>
+        <v>37</v>
+      </c>
+      <c r="D8" s="46" t="str">
+        <f>'THURSDAY SINGLES'!I20</f>
         <v/>
       </c>
-      <c r="C8" s="45" t="str">
-        <f>'SUNDAY SINGLES'!I29</f>
-        <v/>
-      </c>
-      <c r="D8" s="46" t="str">
-        <f>'THURSDAY SINGLES'!I21</f>
-        <v/>
-      </c>
       <c r="E8" s="45" t="str">
-        <f>'THURSDAY SINGLES'!I$22</f>
+        <f>'THURSDAY SINGLES'!I$21</f>
         <v/>
       </c>
     </row>
@@ -12312,19 +12305,19 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="45" t="str">
+        <f>'SUNDAY SINGLES'!J27</f>
+        <v/>
+      </c>
+      <c r="C9" s="45" t="str">
         <f>'SUNDAY SINGLES'!J28</f>
         <v/>
       </c>
-      <c r="C9" s="45" t="str">
-        <f>'SUNDAY SINGLES'!J29</f>
+      <c r="D9" s="46" t="str">
+        <f>'THURSDAY SINGLES'!J20</f>
         <v/>
       </c>
-      <c r="D9" s="46" t="str">
-        <f>'THURSDAY SINGLES'!J21</f>
-        <v/>
-      </c>
       <c r="E9" s="45" t="str">
-        <f>'THURSDAY SINGLES'!J$22</f>
+        <f>'THURSDAY SINGLES'!J$21</f>
         <v/>
       </c>
     </row>
@@ -12333,19 +12326,19 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="45" t="str">
+        <f>'SUNDAY SINGLES'!K27</f>
+        <v/>
+      </c>
+      <c r="C10" s="45" t="str">
         <f>'SUNDAY SINGLES'!K28</f>
         <v/>
       </c>
-      <c r="C10" s="45" t="str">
-        <f>'SUNDAY SINGLES'!K29</f>
+      <c r="D10" s="46" t="str">
+        <f>'THURSDAY SINGLES'!K20</f>
         <v/>
       </c>
-      <c r="D10" s="46" t="str">
-        <f>'THURSDAY SINGLES'!K21</f>
-        <v/>
-      </c>
       <c r="E10" s="45" t="str">
-        <f>'THURSDAY SINGLES'!K$22</f>
+        <f>'THURSDAY SINGLES'!K$21</f>
         <v/>
       </c>
     </row>
@@ -12354,19 +12347,19 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="45" t="str">
+        <f>'SUNDAY SINGLES'!L27</f>
+        <v/>
+      </c>
+      <c r="C11" s="45" t="str">
         <f>'SUNDAY SINGLES'!L28</f>
         <v/>
       </c>
-      <c r="C11" s="45" t="str">
-        <f>'SUNDAY SINGLES'!L29</f>
+      <c r="D11" s="46" t="str">
+        <f>'THURSDAY SINGLES'!L20</f>
         <v/>
       </c>
-      <c r="D11" s="46" t="str">
-        <f>'THURSDAY SINGLES'!L21</f>
-        <v/>
-      </c>
       <c r="E11" s="45" t="str">
-        <f>'THURSDAY SINGLES'!L$22</f>
+        <f>'THURSDAY SINGLES'!L$21</f>
         <v/>
       </c>
     </row>
@@ -12375,19 +12368,19 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="45" t="str">
+        <f>'SUNDAY SINGLES'!M27</f>
+        <v/>
+      </c>
+      <c r="C12" s="45" t="str">
         <f>'SUNDAY SINGLES'!M28</f>
         <v/>
       </c>
-      <c r="C12" s="45" t="str">
-        <f>'SUNDAY SINGLES'!M29</f>
+      <c r="D12" s="46" t="str">
+        <f>'THURSDAY SINGLES'!M20</f>
         <v/>
       </c>
-      <c r="D12" s="46" t="str">
+      <c r="E12" s="45" t="str">
         <f>'THURSDAY SINGLES'!M21</f>
-        <v/>
-      </c>
-      <c r="E12" s="45" t="str">
-        <f>'THURSDAY SINGLES'!M22</f>
         <v/>
       </c>
     </row>
@@ -12396,19 +12389,19 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="45" t="str">
+        <f>'SUNDAY SINGLES'!N27</f>
+        <v/>
+      </c>
+      <c r="C13" s="45" t="str">
         <f>'SUNDAY SINGLES'!N28</f>
         <v/>
       </c>
-      <c r="C13" s="45" t="str">
-        <f>'SUNDAY SINGLES'!N29</f>
+      <c r="D13" s="46" t="str">
+        <f>'THURSDAY SINGLES'!N20</f>
         <v/>
       </c>
-      <c r="D13" s="46" t="str">
-        <f>'THURSDAY SINGLES'!N21</f>
-        <v/>
-      </c>
       <c r="E13" s="45" t="str">
-        <f>'THURSDAY SINGLES'!N$22</f>
+        <f>'THURSDAY SINGLES'!N$21</f>
         <v/>
       </c>
     </row>
@@ -12417,19 +12410,19 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="45" t="str">
+        <f>'SUNDAY SINGLES'!O27</f>
+        <v/>
+      </c>
+      <c r="C14" s="45" t="str">
         <f>'SUNDAY SINGLES'!O28</f>
         <v/>
       </c>
-      <c r="C14" s="45" t="str">
-        <f>'SUNDAY SINGLES'!O29</f>
+      <c r="D14" s="46" t="str">
+        <f>'THURSDAY SINGLES'!O20</f>
         <v/>
       </c>
-      <c r="D14" s="46" t="str">
+      <c r="E14" s="45" t="str">
         <f>'THURSDAY SINGLES'!O21</f>
-        <v/>
-      </c>
-      <c r="E14" s="45" t="str">
-        <f>'THURSDAY SINGLES'!O22</f>
         <v/>
       </c>
     </row>
@@ -12438,19 +12431,19 @@
         <v>14.0</v>
       </c>
       <c r="B15" s="45" t="str">
+        <f>'SUNDAY SINGLES'!P27</f>
+        <v/>
+      </c>
+      <c r="C15" s="45" t="str">
         <f>'SUNDAY SINGLES'!P28</f>
         <v/>
       </c>
-      <c r="C15" s="45" t="str">
-        <f>'SUNDAY SINGLES'!P29</f>
+      <c r="D15" s="46" t="str">
+        <f>'THURSDAY SINGLES'!P20</f>
         <v/>
       </c>
-      <c r="D15" s="46" t="str">
+      <c r="E15" s="45" t="str">
         <f>'THURSDAY SINGLES'!P21</f>
-        <v/>
-      </c>
-      <c r="E15" s="45" t="str">
-        <f>'THURSDAY SINGLES'!P22</f>
         <v/>
       </c>
     </row>
@@ -12459,19 +12452,19 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="45" t="str">
+        <f>'SUNDAY SINGLES'!Q27</f>
+        <v/>
+      </c>
+      <c r="C16" s="45" t="str">
         <f>'SUNDAY SINGLES'!Q28</f>
         <v/>
       </c>
-      <c r="C16" s="45" t="str">
-        <f>'SUNDAY SINGLES'!Q29</f>
+      <c r="D16" s="46" t="str">
+        <f>'THURSDAY SINGLES'!Q20</f>
         <v/>
       </c>
-      <c r="D16" s="46" t="str">
+      <c r="E16" s="45" t="str">
         <f>'THURSDAY SINGLES'!Q21</f>
-        <v/>
-      </c>
-      <c r="E16" s="45" t="str">
-        <f>'THURSDAY SINGLES'!Q22</f>
         <v/>
       </c>
     </row>
@@ -12480,19 +12473,19 @@
         <v>16.0</v>
       </c>
       <c r="B17" s="45" t="str">
+        <f>'SUNDAY SINGLES'!R27</f>
+        <v/>
+      </c>
+      <c r="C17" s="45" t="str">
         <f>'SUNDAY SINGLES'!R28</f>
         <v/>
       </c>
-      <c r="C17" s="45" t="str">
-        <f>'SUNDAY SINGLES'!R29</f>
+      <c r="D17" s="46" t="str">
+        <f>'THURSDAY SINGLES'!R20</f>
         <v/>
       </c>
-      <c r="D17" s="46" t="str">
+      <c r="E17" s="45" t="str">
         <f>'THURSDAY SINGLES'!R21</f>
-        <v/>
-      </c>
-      <c r="E17" s="45" t="str">
-        <f>'THURSDAY SINGLES'!R22</f>
         <v/>
       </c>
     </row>
@@ -12501,19 +12494,19 @@
         <v>17.0</v>
       </c>
       <c r="B18" s="45" t="str">
+        <f>'SUNDAY SINGLES'!S27</f>
+        <v/>
+      </c>
+      <c r="C18" s="45" t="str">
         <f>'SUNDAY SINGLES'!S28</f>
         <v/>
       </c>
-      <c r="C18" s="45" t="str">
-        <f>'SUNDAY SINGLES'!S29</f>
+      <c r="D18" s="46" t="str">
+        <f>'THURSDAY SINGLES'!S20</f>
         <v/>
       </c>
-      <c r="D18" s="46" t="str">
+      <c r="E18" s="45" t="str">
         <f>'THURSDAY SINGLES'!S21</f>
-        <v/>
-      </c>
-      <c r="E18" s="45" t="str">
-        <f>'THURSDAY SINGLES'!S22</f>
         <v/>
       </c>
     </row>
@@ -12522,19 +12515,19 @@
         <v>18.0</v>
       </c>
       <c r="B19" s="45" t="str">
+        <f>'SUNDAY SINGLES'!T27</f>
+        <v/>
+      </c>
+      <c r="C19" s="45" t="str">
         <f>'SUNDAY SINGLES'!T28</f>
         <v/>
       </c>
-      <c r="C19" s="45" t="str">
-        <f>'SUNDAY SINGLES'!T29</f>
+      <c r="D19" s="46" t="str">
+        <f>'THURSDAY SINGLES'!T20</f>
         <v/>
       </c>
-      <c r="D19" s="46" t="str">
+      <c r="E19" s="45" t="str">
         <f>'THURSDAY SINGLES'!T21</f>
-        <v/>
-      </c>
-      <c r="E19" s="45" t="str">
-        <f>'THURSDAY SINGLES'!T22</f>
         <v/>
       </c>
     </row>
@@ -12543,19 +12536,19 @@
         <v>19.0</v>
       </c>
       <c r="B20" s="45" t="str">
+        <f>'SUNDAY SINGLES'!U27</f>
+        <v/>
+      </c>
+      <c r="C20" s="45" t="str">
         <f>'SUNDAY SINGLES'!U28</f>
         <v/>
       </c>
-      <c r="C20" s="45" t="str">
-        <f>'SUNDAY SINGLES'!U29</f>
+      <c r="D20" s="46" t="str">
+        <f>'THURSDAY SINGLES'!U20</f>
         <v/>
       </c>
-      <c r="D20" s="46" t="str">
+      <c r="E20" s="45" t="str">
         <f>'THURSDAY SINGLES'!U21</f>
-        <v/>
-      </c>
-      <c r="E20" s="45" t="str">
-        <f>'THURSDAY SINGLES'!U22</f>
         <v/>
       </c>
     </row>
@@ -12564,19 +12557,19 @@
         <v>20.0</v>
       </c>
       <c r="B21" s="45" t="str">
+        <f>'SUNDAY SINGLES'!V27</f>
+        <v/>
+      </c>
+      <c r="C21" s="45" t="str">
         <f>'SUNDAY SINGLES'!V28</f>
         <v/>
       </c>
-      <c r="C21" s="45" t="str">
-        <f>'SUNDAY SINGLES'!V29</f>
+      <c r="D21" s="46" t="str">
+        <f>'THURSDAY SINGLES'!V20</f>
         <v/>
       </c>
-      <c r="D21" s="46" t="str">
+      <c r="E21" s="45" t="str">
         <f>'THURSDAY SINGLES'!V21</f>
-        <v/>
-      </c>
-      <c r="E21" s="45" t="str">
-        <f>'THURSDAY SINGLES'!V22</f>
         <v/>
       </c>
     </row>
@@ -12585,19 +12578,19 @@
         <v>21.0</v>
       </c>
       <c r="B22" s="45" t="str">
+        <f>'SUNDAY SINGLES'!W27</f>
+        <v/>
+      </c>
+      <c r="C22" s="45" t="str">
         <f>'SUNDAY SINGLES'!W28</f>
         <v/>
       </c>
-      <c r="C22" s="45" t="str">
-        <f>'SUNDAY SINGLES'!W29</f>
+      <c r="D22" s="46" t="str">
+        <f>'THURSDAY SINGLES'!W20</f>
         <v/>
       </c>
-      <c r="D22" s="46" t="str">
+      <c r="E22" s="45" t="str">
         <f>'THURSDAY SINGLES'!W21</f>
-        <v/>
-      </c>
-      <c r="E22" s="45" t="str">
-        <f>'THURSDAY SINGLES'!W22</f>
         <v/>
       </c>
     </row>
@@ -12606,19 +12599,19 @@
         <v>22.0</v>
       </c>
       <c r="B23" s="45" t="str">
+        <f>'SUNDAY SINGLES'!X27</f>
+        <v/>
+      </c>
+      <c r="C23" s="45" t="str">
         <f>'SUNDAY SINGLES'!X28</f>
         <v/>
       </c>
-      <c r="C23" s="45" t="str">
-        <f>'SUNDAY SINGLES'!X29</f>
+      <c r="D23" s="46" t="str">
+        <f>'THURSDAY SINGLES'!X20</f>
         <v/>
       </c>
-      <c r="D23" s="46" t="str">
+      <c r="E23" s="45" t="str">
         <f>'THURSDAY SINGLES'!X21</f>
-        <v/>
-      </c>
-      <c r="E23" s="45" t="str">
-        <f>'THURSDAY SINGLES'!X22</f>
         <v/>
       </c>
     </row>
@@ -12627,19 +12620,19 @@
         <v>23.0</v>
       </c>
       <c r="B24" s="45" t="str">
+        <f>'SUNDAY SINGLES'!Y27</f>
+        <v/>
+      </c>
+      <c r="C24" s="45" t="str">
         <f>'SUNDAY SINGLES'!Y28</f>
         <v/>
       </c>
-      <c r="C24" s="45" t="str">
-        <f>'SUNDAY SINGLES'!Y29</f>
+      <c r="D24" s="46" t="str">
+        <f>'THURSDAY SINGLES'!Y20</f>
         <v/>
       </c>
-      <c r="D24" s="46" t="str">
+      <c r="E24" s="45" t="str">
         <f>'THURSDAY SINGLES'!Y21</f>
-        <v/>
-      </c>
-      <c r="E24" s="45" t="str">
-        <f>'THURSDAY SINGLES'!Y22</f>
         <v/>
       </c>
     </row>
@@ -12648,19 +12641,19 @@
         <v>24.0</v>
       </c>
       <c r="B25" s="45" t="str">
+        <f>'SUNDAY SINGLES'!Z27</f>
+        <v/>
+      </c>
+      <c r="C25" s="45" t="str">
         <f>'SUNDAY SINGLES'!Z28</f>
         <v/>
       </c>
-      <c r="C25" s="45" t="str">
-        <f>'SUNDAY SINGLES'!Z29</f>
+      <c r="D25" s="46" t="str">
+        <f>'THURSDAY SINGLES'!Z20</f>
         <v/>
       </c>
-      <c r="D25" s="46" t="str">
+      <c r="E25" s="45" t="str">
         <f>'THURSDAY SINGLES'!Z21</f>
-        <v/>
-      </c>
-      <c r="E25" s="45" t="str">
-        <f>'THURSDAY SINGLES'!Z22</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
098 Week 7/8 data update
</commit_message>
<xml_diff>
--- a/data/SUMMER_GOLF_2026.xlsx
+++ b/data/SUMMER_GOLF_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="91">
   <si>
     <t>SUMMER GOLF 2026 - THURSDAY SINGLES</t>
   </si>
@@ -273,6 +273,9 @@
   </si>
   <si>
     <t>PAUL SHIRLEY</t>
+  </si>
+  <si>
+    <t>ANDY THOMPSON/DAVE CROSSLEY</t>
   </si>
   <si>
     <t>SUNDAY</t>
@@ -1031,7 +1034,9 @@
       <c r="H6" s="14">
         <v>33.0</v>
       </c>
-      <c r="I6" s="13"/>
+      <c r="I6" s="13">
+        <v>28.0</v>
+      </c>
       <c r="J6" s="14"/>
       <c r="K6" s="13"/>
       <c r="L6" s="14"/>
@@ -1051,7 +1056,7 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>181</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7">
@@ -1119,7 +1124,9 @@
       <c r="H8" s="14">
         <v>34.0</v>
       </c>
-      <c r="I8" s="13"/>
+      <c r="I8" s="13">
+        <v>35.0</v>
+      </c>
       <c r="J8" s="14"/>
       <c r="K8" s="16"/>
       <c r="L8" s="15"/>
@@ -1139,7 +1146,7 @@
       <c r="Z8" s="19"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>199</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9">
@@ -1164,7 +1171,9 @@
       <c r="H9" s="14">
         <v>29.0</v>
       </c>
-      <c r="I9" s="13"/>
+      <c r="I9" s="13">
+        <v>29.0</v>
+      </c>
       <c r="J9" s="14"/>
       <c r="K9" s="13"/>
       <c r="L9" s="14"/>
@@ -1184,7 +1193,7 @@
       <c r="Z9" s="17"/>
       <c r="AA9" s="15">
         <f t="shared" si="1"/>
-        <v>178</v>
+        <v>207</v>
       </c>
     </row>
     <row r="10">
@@ -1207,7 +1216,9 @@
       <c r="H10" s="14">
         <v>33.0</v>
       </c>
-      <c r="I10" s="13"/>
+      <c r="I10" s="13">
+        <v>32.0</v>
+      </c>
       <c r="J10" s="14"/>
       <c r="K10" s="16"/>
       <c r="L10" s="15"/>
@@ -1227,7 +1238,7 @@
       <c r="Z10" s="17"/>
       <c r="AA10" s="15">
         <f t="shared" si="1"/>
-        <v>163</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11">
@@ -1291,7 +1302,9 @@
       <c r="H12" s="14">
         <v>36.0</v>
       </c>
-      <c r="I12" s="13"/>
+      <c r="I12" s="13">
+        <v>30.0</v>
+      </c>
       <c r="J12" s="14"/>
       <c r="K12" s="13"/>
       <c r="L12" s="14"/>
@@ -1311,7 +1324,7 @@
       <c r="Z12" s="17"/>
       <c r="AA12" s="15">
         <f t="shared" si="1"/>
-        <v>116</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13">
@@ -1334,7 +1347,9 @@
       <c r="H13" s="14">
         <v>33.0</v>
       </c>
-      <c r="I13" s="13"/>
+      <c r="I13" s="13">
+        <v>32.0</v>
+      </c>
       <c r="J13" s="14"/>
       <c r="K13" s="13"/>
       <c r="L13" s="15"/>
@@ -1354,7 +1369,7 @@
       <c r="Z13" s="17"/>
       <c r="AA13" s="15">
         <f t="shared" si="1"/>
-        <v>148</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14">
@@ -1375,7 +1390,9 @@
       <c r="H14" s="14">
         <v>23.0</v>
       </c>
-      <c r="I14" s="13"/>
+      <c r="I14" s="13">
+        <v>30.0</v>
+      </c>
       <c r="J14" s="14"/>
       <c r="K14" s="13"/>
       <c r="L14" s="14"/>
@@ -1395,7 +1412,7 @@
       <c r="Z14" s="17"/>
       <c r="AA14" s="15">
         <f t="shared" si="1"/>
-        <v>112</v>
+        <v>142</v>
       </c>
     </row>
     <row r="15">
@@ -1416,7 +1433,9 @@
         <v>29.0</v>
       </c>
       <c r="H15" s="14"/>
-      <c r="I15" s="13"/>
+      <c r="I15" s="13">
+        <v>25.0</v>
+      </c>
       <c r="J15" s="14"/>
       <c r="K15" s="13"/>
       <c r="L15" s="14"/>
@@ -1436,7 +1455,7 @@
       <c r="Z15" s="17"/>
       <c r="AA15" s="15">
         <f t="shared" si="1"/>
-        <v>111</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16">
@@ -1451,7 +1470,9 @@
       <c r="H16" s="14">
         <v>21.0</v>
       </c>
-      <c r="I16" s="13"/>
+      <c r="I16" s="13">
+        <v>27.0</v>
+      </c>
       <c r="J16" s="14"/>
       <c r="K16" s="13"/>
       <c r="L16" s="15"/>
@@ -1471,7 +1492,7 @@
       <c r="Z16" s="17"/>
       <c r="AA16" s="15">
         <f t="shared" si="1"/>
-        <v>21</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17">
@@ -1494,7 +1515,9 @@
         <v>29.0</v>
       </c>
       <c r="H17" s="14"/>
-      <c r="I17" s="13"/>
+      <c r="I17" s="13">
+        <v>22.0</v>
+      </c>
       <c r="J17" s="14"/>
       <c r="K17" s="13"/>
       <c r="L17" s="15"/>
@@ -1514,7 +1537,7 @@
       <c r="Z17" s="17"/>
       <c r="AA17" s="15">
         <f t="shared" si="1"/>
-        <v>124</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18">
@@ -1529,7 +1552,9 @@
       </c>
       <c r="G18" s="13"/>
       <c r="H18" s="14"/>
-      <c r="I18" s="13"/>
+      <c r="I18" s="13">
+        <v>27.0</v>
+      </c>
       <c r="J18" s="14"/>
       <c r="K18" s="13"/>
       <c r="L18" s="15"/>
@@ -1549,7 +1574,7 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>27</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" ht="9.0" customHeight="1">
@@ -1600,7 +1625,9 @@
       <c r="H20" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="I20" s="24"/>
+      <c r="I20" s="24" t="s">
+        <v>36</v>
+      </c>
       <c r="J20" s="24"/>
       <c r="K20" s="24"/>
       <c r="L20" s="24"/>
@@ -1642,7 +1669,9 @@
       <c r="H21" s="27">
         <v>36.0</v>
       </c>
-      <c r="I21" s="27"/>
+      <c r="I21" s="27">
+        <v>35.0</v>
+      </c>
       <c r="J21" s="27"/>
       <c r="K21" s="27"/>
       <c r="L21" s="27"/>
@@ -1871,7 +1900,9 @@
         <v>28.0</v>
       </c>
       <c r="I6" s="13"/>
-      <c r="J6" s="14"/>
+      <c r="J6" s="14">
+        <v>32.0</v>
+      </c>
       <c r="K6" s="13"/>
       <c r="L6" s="15"/>
       <c r="M6" s="13"/>
@@ -1890,7 +1921,7 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>154</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7">
@@ -1918,7 +1949,9 @@
       <c r="I7" s="13">
         <v>37.0</v>
       </c>
-      <c r="J7" s="14"/>
+      <c r="J7" s="14">
+        <v>38.0</v>
+      </c>
       <c r="K7" s="13"/>
       <c r="L7" s="14"/>
       <c r="M7" s="13"/>
@@ -1937,7 +1970,7 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>218</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8">
@@ -1963,7 +1996,9 @@
       <c r="I8" s="13">
         <v>31.0</v>
       </c>
-      <c r="J8" s="14"/>
+      <c r="J8" s="14">
+        <v>36.0</v>
+      </c>
       <c r="K8" s="16"/>
       <c r="L8" s="14"/>
       <c r="M8" s="13"/>
@@ -1982,7 +2017,7 @@
       <c r="Z8" s="17"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>174</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9">
@@ -2039,7 +2074,9 @@
       </c>
       <c r="H10" s="14"/>
       <c r="I10" s="13"/>
-      <c r="J10" s="14"/>
+      <c r="J10" s="14">
+        <v>27.0</v>
+      </c>
       <c r="K10" s="13"/>
       <c r="L10" s="14"/>
       <c r="M10" s="13"/>
@@ -2058,7 +2095,7 @@
       <c r="Z10" s="19"/>
       <c r="AA10" s="15">
         <f t="shared" si="1"/>
-        <v>25</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11">
@@ -2084,7 +2121,9 @@
       <c r="I11" s="13">
         <v>34.0</v>
       </c>
-      <c r="J11" s="15"/>
+      <c r="J11" s="14">
+        <v>34.0</v>
+      </c>
       <c r="K11" s="13"/>
       <c r="L11" s="15"/>
       <c r="M11" s="13"/>
@@ -2103,7 +2142,7 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>190</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12">
@@ -2164,7 +2203,9 @@
       <c r="I13" s="13">
         <v>33.0</v>
       </c>
-      <c r="J13" s="14"/>
+      <c r="J13" s="14">
+        <v>31.0</v>
+      </c>
       <c r="K13" s="13"/>
       <c r="L13" s="14"/>
       <c r="M13" s="13"/>
@@ -2183,7 +2224,7 @@
       <c r="Z13" s="17"/>
       <c r="AA13" s="15">
         <f t="shared" si="1"/>
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14">
@@ -2207,7 +2248,9 @@
         <v>35.0</v>
       </c>
       <c r="I14" s="13"/>
-      <c r="J14" s="15"/>
+      <c r="J14" s="14">
+        <v>32.0</v>
+      </c>
       <c r="K14" s="16"/>
       <c r="L14" s="14"/>
       <c r="M14" s="16"/>
@@ -2226,7 +2269,7 @@
       <c r="Z14" s="17"/>
       <c r="AA14" s="15">
         <f t="shared" si="1"/>
-        <v>140</v>
+        <v>172</v>
       </c>
     </row>
     <row r="15">
@@ -2252,7 +2295,9 @@
       <c r="I15" s="13">
         <v>27.0</v>
       </c>
-      <c r="J15" s="15"/>
+      <c r="J15" s="14">
+        <v>21.0</v>
+      </c>
       <c r="K15" s="16"/>
       <c r="L15" s="15"/>
       <c r="M15" s="16"/>
@@ -2271,7 +2316,7 @@
       <c r="Z15" s="17"/>
       <c r="AA15" s="15">
         <f t="shared" si="1"/>
-        <v>186</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16">
@@ -2299,7 +2344,9 @@
       <c r="I16" s="13">
         <v>19.0</v>
       </c>
-      <c r="J16" s="14"/>
+      <c r="J16" s="14">
+        <v>25.0</v>
+      </c>
       <c r="K16" s="13"/>
       <c r="L16" s="14"/>
       <c r="M16" s="13"/>
@@ -2318,7 +2365,7 @@
       <c r="Z16" s="17"/>
       <c r="AA16" s="15">
         <f t="shared" si="1"/>
-        <v>147</v>
+        <v>172</v>
       </c>
     </row>
     <row r="17">
@@ -2342,7 +2389,9 @@
         <v>31.0</v>
       </c>
       <c r="I17" s="13"/>
-      <c r="J17" s="14"/>
+      <c r="J17" s="14">
+        <v>35.0</v>
+      </c>
       <c r="K17" s="13"/>
       <c r="L17" s="14"/>
       <c r="M17" s="13"/>
@@ -2361,7 +2410,7 @@
       <c r="Z17" s="17"/>
       <c r="AA17" s="15">
         <f t="shared" si="1"/>
-        <v>167</v>
+        <v>202</v>
       </c>
     </row>
     <row r="18">
@@ -2385,7 +2434,9 @@
         <v>33.0</v>
       </c>
       <c r="I18" s="13"/>
-      <c r="J18" s="14"/>
+      <c r="J18" s="14">
+        <v>34.0</v>
+      </c>
       <c r="K18" s="13"/>
       <c r="L18" s="14"/>
       <c r="M18" s="13"/>
@@ -2404,7 +2455,7 @@
       <c r="Z18" s="17"/>
       <c r="AA18" s="15">
         <f t="shared" si="1"/>
-        <v>155</v>
+        <v>189</v>
       </c>
     </row>
     <row r="19">
@@ -2430,7 +2481,9 @@
       <c r="I19" s="13">
         <v>27.0</v>
       </c>
-      <c r="J19" s="14"/>
+      <c r="J19" s="14">
+        <v>37.0</v>
+      </c>
       <c r="K19" s="13"/>
       <c r="L19" s="14"/>
       <c r="M19" s="13"/>
@@ -2449,7 +2502,7 @@
       <c r="Z19" s="17"/>
       <c r="AA19" s="15">
         <f t="shared" si="1"/>
-        <v>186</v>
+        <v>223</v>
       </c>
     </row>
     <row r="20">
@@ -2516,7 +2569,9 @@
       <c r="I21" s="13">
         <v>28.0</v>
       </c>
-      <c r="J21" s="14"/>
+      <c r="J21" s="14">
+        <v>23.0</v>
+      </c>
       <c r="K21" s="13"/>
       <c r="L21" s="14"/>
       <c r="M21" s="13"/>
@@ -2535,7 +2590,7 @@
       <c r="Z21" s="17"/>
       <c r="AA21" s="15">
         <f t="shared" si="1"/>
-        <v>213</v>
+        <v>236</v>
       </c>
     </row>
     <row r="22">
@@ -2555,7 +2610,9 @@
         <v>33.0</v>
       </c>
       <c r="I22" s="13"/>
-      <c r="J22" s="14"/>
+      <c r="J22" s="14">
+        <v>40.0</v>
+      </c>
       <c r="K22" s="13"/>
       <c r="L22" s="14"/>
       <c r="M22" s="13"/>
@@ -2574,7 +2631,7 @@
       <c r="Z22" s="17"/>
       <c r="AA22" s="15">
         <f t="shared" si="1"/>
-        <v>107</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23">
@@ -2590,7 +2647,9 @@
       <c r="G23" s="13"/>
       <c r="H23" s="14"/>
       <c r="I23" s="13"/>
-      <c r="J23" s="14"/>
+      <c r="J23" s="14">
+        <v>14.0</v>
+      </c>
       <c r="K23" s="13"/>
       <c r="L23" s="14"/>
       <c r="M23" s="13"/>
@@ -2609,7 +2668,7 @@
       <c r="Z23" s="17"/>
       <c r="AA23" s="15">
         <f t="shared" si="1"/>
-        <v>25</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24">
@@ -2635,7 +2694,9 @@
       <c r="I24" s="13">
         <v>35.0</v>
       </c>
-      <c r="J24" s="14"/>
+      <c r="J24" s="14">
+        <v>29.0</v>
+      </c>
       <c r="K24" s="13"/>
       <c r="L24" s="14"/>
       <c r="M24" s="13"/>
@@ -2654,7 +2715,7 @@
       <c r="Z24" s="17"/>
       <c r="AA24" s="15">
         <f t="shared" si="1"/>
-        <v>196</v>
+        <v>225</v>
       </c>
     </row>
     <row r="25">
@@ -2680,7 +2741,9 @@
       <c r="I25" s="13">
         <v>34.0</v>
       </c>
-      <c r="J25" s="14"/>
+      <c r="J25" s="14">
+        <v>32.0</v>
+      </c>
       <c r="K25" s="13"/>
       <c r="L25" s="14"/>
       <c r="M25" s="13"/>
@@ -2699,7 +2762,7 @@
       <c r="Z25" s="17"/>
       <c r="AA25" s="15">
         <f t="shared" si="1"/>
-        <v>168</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26" ht="9.0" customHeight="1">
@@ -2753,7 +2816,9 @@
       <c r="I27" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="J27" s="24"/>
+      <c r="J27" s="24" t="s">
+        <v>34</v>
+      </c>
       <c r="K27" s="24"/>
       <c r="L27" s="24"/>
       <c r="M27" s="24"/>
@@ -2797,7 +2862,9 @@
       <c r="I28" s="27">
         <v>37.0</v>
       </c>
-      <c r="J28" s="27"/>
+      <c r="J28" s="27">
+        <v>40.0</v>
+      </c>
       <c r="K28" s="27"/>
       <c r="L28" s="27"/>
       <c r="M28" s="27"/>
@@ -2849,10 +2916,10 @@
         <v>45</v>
       </c>
       <c r="B2" s="33">
+        <v>18.0</v>
+      </c>
+      <c r="C2" s="34">
         <v>17.0</v>
-      </c>
-      <c r="C2" s="34">
-        <v>16.0</v>
       </c>
     </row>
     <row r="3">
@@ -2915,7 +2982,7 @@
         <v>37</v>
       </c>
       <c r="B8" s="33">
-        <v>32.0</v>
+        <v>33.0</v>
       </c>
       <c r="C8" s="34">
         <v>31.0</v>
@@ -2940,7 +3007,7 @@
         <v>16.0</v>
       </c>
       <c r="C10" s="34">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="11">
@@ -2951,7 +3018,7 @@
         <v>22.0</v>
       </c>
       <c r="C11" s="34">
-        <v>20.0</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="12">
@@ -3036,10 +3103,10 @@
         <v>42</v>
       </c>
       <c r="B19" s="33">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
       <c r="C19" s="34">
-        <v>29.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="20">
@@ -7142,13 +7209,17 @@
       <c r="B8" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="C8" s="43"/>
+      <c r="C8" s="43" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="14">
         <v>8.0</v>
       </c>
-      <c r="B9" s="42"/>
+      <c r="B9" s="42" t="s">
+        <v>86</v>
+      </c>
       <c r="C9" s="43"/>
     </row>
     <row r="10">
@@ -12141,16 +12212,16 @@
         <v>76</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D1" s="44" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2">
@@ -12293,11 +12364,11 @@
       </c>
       <c r="D8" s="46" t="str">
         <f>'THURSDAY SINGLES'!I20</f>
-        <v/>
-      </c>
-      <c r="E8" s="45" t="str">
+        <v>LES DOBBINS</v>
+      </c>
+      <c r="E8" s="45">
         <f>'THURSDAY SINGLES'!I$21</f>
-        <v/>
+        <v>35</v>
       </c>
     </row>
     <row r="9">
@@ -12306,11 +12377,11 @@
       </c>
       <c r="B9" s="45" t="str">
         <f>'SUNDAY SINGLES'!J27</f>
-        <v/>
-      </c>
-      <c r="C9" s="45" t="str">
+        <v>STEWART TAYLOR</v>
+      </c>
+      <c r="C9" s="45">
         <f>'SUNDAY SINGLES'!J28</f>
-        <v/>
+        <v>40</v>
       </c>
       <c r="D9" s="46" t="str">
         <f>'THURSDAY SINGLES'!J20</f>

</xml_diff>

<commit_message>
099 Week 8/9 data update
</commit_message>
<xml_diff>
--- a/data/SUMMER_GOLF_2026.xlsx
+++ b/data/SUMMER_GOLF_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="92">
   <si>
     <t>SUMMER GOLF 2026 - THURSDAY SINGLES</t>
   </si>
@@ -276,6 +276,9 @@
   </si>
   <si>
     <t>ANDY THOMPSON/DAVE CROSSLEY</t>
+  </si>
+  <si>
+    <t>BAZ MASON/TONI SHIRLEY</t>
   </si>
   <si>
     <t>SUNDAY</t>
@@ -990,7 +993,9 @@
         <v>35.0</v>
       </c>
       <c r="I5" s="13"/>
-      <c r="J5" s="14"/>
+      <c r="J5" s="14">
+        <v>30.0</v>
+      </c>
       <c r="K5" s="13"/>
       <c r="L5" s="15"/>
       <c r="M5" s="13"/>
@@ -1009,7 +1014,7 @@
       <c r="Z5" s="17"/>
       <c r="AA5" s="15">
         <f t="shared" ref="AA5:AA18" si="1">sum(C5:Z5)</f>
-        <v>150</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6">
@@ -1037,7 +1042,9 @@
       <c r="I6" s="13">
         <v>28.0</v>
       </c>
-      <c r="J6" s="14"/>
+      <c r="J6" s="14">
+        <v>29.0</v>
+      </c>
       <c r="K6" s="13"/>
       <c r="L6" s="14"/>
       <c r="M6" s="13"/>
@@ -1056,7 +1063,7 @@
       <c r="Z6" s="17"/>
       <c r="AA6" s="15">
         <f t="shared" si="1"/>
-        <v>209</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7">
@@ -1080,7 +1087,9 @@
         <v>31.0</v>
       </c>
       <c r="I7" s="13"/>
-      <c r="J7" s="14"/>
+      <c r="J7" s="14">
+        <v>38.0</v>
+      </c>
       <c r="K7" s="16"/>
       <c r="L7" s="14"/>
       <c r="M7" s="13"/>
@@ -1099,7 +1108,7 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>152</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8">
@@ -1127,7 +1136,9 @@
       <c r="I8" s="13">
         <v>35.0</v>
       </c>
-      <c r="J8" s="14"/>
+      <c r="J8" s="14">
+        <v>27.0</v>
+      </c>
       <c r="K8" s="16"/>
       <c r="L8" s="15"/>
       <c r="M8" s="13"/>
@@ -1146,7 +1157,7 @@
       <c r="Z8" s="19"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>234</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9">
@@ -1174,7 +1185,9 @@
       <c r="I9" s="13">
         <v>29.0</v>
       </c>
-      <c r="J9" s="14"/>
+      <c r="J9" s="14">
+        <v>36.0</v>
+      </c>
       <c r="K9" s="13"/>
       <c r="L9" s="14"/>
       <c r="M9" s="13"/>
@@ -1193,7 +1206,7 @@
       <c r="Z9" s="17"/>
       <c r="AA9" s="15">
         <f t="shared" si="1"/>
-        <v>207</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10">
@@ -1219,7 +1232,9 @@
       <c r="I10" s="13">
         <v>32.0</v>
       </c>
-      <c r="J10" s="14"/>
+      <c r="J10" s="14">
+        <v>26.0</v>
+      </c>
       <c r="K10" s="16"/>
       <c r="L10" s="15"/>
       <c r="M10" s="13"/>
@@ -1238,7 +1253,7 @@
       <c r="Z10" s="17"/>
       <c r="AA10" s="15">
         <f t="shared" si="1"/>
-        <v>195</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11">
@@ -1262,7 +1277,9 @@
         <v>35.0</v>
       </c>
       <c r="I11" s="13"/>
-      <c r="J11" s="14"/>
+      <c r="J11" s="14">
+        <v>32.0</v>
+      </c>
       <c r="K11" s="13"/>
       <c r="L11" s="14"/>
       <c r="M11" s="16"/>
@@ -1281,7 +1298,7 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>164</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12">
@@ -1305,7 +1322,9 @@
       <c r="I12" s="13">
         <v>30.0</v>
       </c>
-      <c r="J12" s="14"/>
+      <c r="J12" s="14">
+        <v>35.0</v>
+      </c>
       <c r="K12" s="13"/>
       <c r="L12" s="14"/>
       <c r="M12" s="13"/>
@@ -1324,7 +1343,7 @@
       <c r="Z12" s="17"/>
       <c r="AA12" s="15">
         <f t="shared" si="1"/>
-        <v>146</v>
+        <v>181</v>
       </c>
     </row>
     <row r="13">
@@ -1350,7 +1369,9 @@
       <c r="I13" s="13">
         <v>32.0</v>
       </c>
-      <c r="J13" s="14"/>
+      <c r="J13" s="14">
+        <v>38.0</v>
+      </c>
       <c r="K13" s="13"/>
       <c r="L13" s="15"/>
       <c r="M13" s="16"/>
@@ -1369,7 +1390,7 @@
       <c r="Z13" s="17"/>
       <c r="AA13" s="15">
         <f t="shared" si="1"/>
-        <v>180</v>
+        <v>218</v>
       </c>
     </row>
     <row r="14">
@@ -1393,7 +1414,9 @@
       <c r="I14" s="13">
         <v>30.0</v>
       </c>
-      <c r="J14" s="14"/>
+      <c r="J14" s="14">
+        <v>37.0</v>
+      </c>
       <c r="K14" s="13"/>
       <c r="L14" s="14"/>
       <c r="M14" s="13"/>
@@ -1412,7 +1435,7 @@
       <c r="Z14" s="17"/>
       <c r="AA14" s="15">
         <f t="shared" si="1"/>
-        <v>142</v>
+        <v>179</v>
       </c>
     </row>
     <row r="15">
@@ -1473,7 +1496,9 @@
       <c r="I16" s="13">
         <v>27.0</v>
       </c>
-      <c r="J16" s="14"/>
+      <c r="J16" s="14">
+        <v>30.0</v>
+      </c>
       <c r="K16" s="13"/>
       <c r="L16" s="15"/>
       <c r="M16" s="16"/>
@@ -1492,7 +1517,7 @@
       <c r="Z16" s="17"/>
       <c r="AA16" s="15">
         <f t="shared" si="1"/>
-        <v>48</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17">
@@ -1518,7 +1543,9 @@
       <c r="I17" s="13">
         <v>22.0</v>
       </c>
-      <c r="J17" s="14"/>
+      <c r="J17" s="14">
+        <v>31.0</v>
+      </c>
       <c r="K17" s="13"/>
       <c r="L17" s="15"/>
       <c r="M17" s="16"/>
@@ -1537,7 +1564,7 @@
       <c r="Z17" s="17"/>
       <c r="AA17" s="15">
         <f t="shared" si="1"/>
-        <v>146</v>
+        <v>177</v>
       </c>
     </row>
     <row r="18">
@@ -1628,7 +1655,9 @@
       <c r="I20" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="J20" s="24"/>
+      <c r="J20" s="24" t="s">
+        <v>41</v>
+      </c>
       <c r="K20" s="24"/>
       <c r="L20" s="24"/>
       <c r="M20" s="24"/>
@@ -1672,7 +1701,9 @@
       <c r="I21" s="27">
         <v>35.0</v>
       </c>
-      <c r="J21" s="27"/>
+      <c r="J21" s="27">
+        <v>38.0</v>
+      </c>
       <c r="K21" s="27"/>
       <c r="L21" s="27"/>
       <c r="M21" s="27"/>
@@ -1858,7 +1889,9 @@
       <c r="H5" s="15"/>
       <c r="I5" s="13"/>
       <c r="J5" s="14"/>
-      <c r="K5" s="13"/>
+      <c r="K5" s="13">
+        <v>36.0</v>
+      </c>
       <c r="L5" s="15"/>
       <c r="M5" s="16"/>
       <c r="N5" s="14"/>
@@ -1876,7 +1909,7 @@
       <c r="Z5" s="19"/>
       <c r="AA5" s="15">
         <f t="shared" ref="AA5:AA25" si="1">SUM(C5:Z5)</f>
-        <v>80</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6">
@@ -1952,7 +1985,9 @@
       <c r="J7" s="14">
         <v>38.0</v>
       </c>
-      <c r="K7" s="13"/>
+      <c r="K7" s="13">
+        <v>32.0</v>
+      </c>
       <c r="L7" s="14"/>
       <c r="M7" s="13"/>
       <c r="N7" s="14"/>
@@ -1970,7 +2005,7 @@
       <c r="Z7" s="17"/>
       <c r="AA7" s="15">
         <f t="shared" si="1"/>
-        <v>256</v>
+        <v>288</v>
       </c>
     </row>
     <row r="8">
@@ -1999,7 +2034,9 @@
       <c r="J8" s="14">
         <v>36.0</v>
       </c>
-      <c r="K8" s="16"/>
+      <c r="K8" s="13">
+        <v>33.0</v>
+      </c>
       <c r="L8" s="14"/>
       <c r="M8" s="13"/>
       <c r="N8" s="14"/>
@@ -2017,7 +2054,7 @@
       <c r="Z8" s="17"/>
       <c r="AA8" s="15">
         <f t="shared" si="1"/>
-        <v>210</v>
+        <v>243</v>
       </c>
     </row>
     <row r="9">
@@ -2040,7 +2077,9 @@
       <c r="H9" s="14"/>
       <c r="I9" s="16"/>
       <c r="J9" s="15"/>
-      <c r="K9" s="13"/>
+      <c r="K9" s="13">
+        <v>33.0</v>
+      </c>
       <c r="L9" s="14"/>
       <c r="M9" s="13"/>
       <c r="N9" s="14"/>
@@ -2058,7 +2097,7 @@
       <c r="Z9" s="17"/>
       <c r="AA9" s="15">
         <f t="shared" si="1"/>
-        <v>112</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10">
@@ -2077,7 +2116,9 @@
       <c r="J10" s="14">
         <v>27.0</v>
       </c>
-      <c r="K10" s="13"/>
+      <c r="K10" s="13">
+        <v>29.0</v>
+      </c>
       <c r="L10" s="14"/>
       <c r="M10" s="13"/>
       <c r="N10" s="14"/>
@@ -2095,7 +2136,7 @@
       <c r="Z10" s="19"/>
       <c r="AA10" s="15">
         <f t="shared" si="1"/>
-        <v>52</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11">
@@ -2124,7 +2165,9 @@
       <c r="J11" s="14">
         <v>34.0</v>
       </c>
-      <c r="K11" s="13"/>
+      <c r="K11" s="13">
+        <v>35.0</v>
+      </c>
       <c r="L11" s="15"/>
       <c r="M11" s="13"/>
       <c r="N11" s="15"/>
@@ -2142,7 +2185,7 @@
       <c r="Z11" s="17"/>
       <c r="AA11" s="15">
         <f t="shared" si="1"/>
-        <v>224</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12">
@@ -2251,7 +2294,9 @@
       <c r="J14" s="14">
         <v>32.0</v>
       </c>
-      <c r="K14" s="16"/>
+      <c r="K14" s="13">
+        <v>32.0</v>
+      </c>
       <c r="L14" s="14"/>
       <c r="M14" s="16"/>
       <c r="N14" s="15"/>
@@ -2269,7 +2314,7 @@
       <c r="Z14" s="17"/>
       <c r="AA14" s="15">
         <f t="shared" si="1"/>
-        <v>172</v>
+        <v>204</v>
       </c>
     </row>
     <row r="15">
@@ -2347,7 +2392,9 @@
       <c r="J16" s="14">
         <v>25.0</v>
       </c>
-      <c r="K16" s="13"/>
+      <c r="K16" s="13">
+        <v>27.0</v>
+      </c>
       <c r="L16" s="14"/>
       <c r="M16" s="13"/>
       <c r="N16" s="14"/>
@@ -2365,7 +2412,7 @@
       <c r="Z16" s="17"/>
       <c r="AA16" s="15">
         <f t="shared" si="1"/>
-        <v>172</v>
+        <v>199</v>
       </c>
     </row>
     <row r="17">
@@ -2392,7 +2439,9 @@
       <c r="J17" s="14">
         <v>35.0</v>
       </c>
-      <c r="K17" s="13"/>
+      <c r="K17" s="13">
+        <v>33.0</v>
+      </c>
       <c r="L17" s="14"/>
       <c r="M17" s="13"/>
       <c r="N17" s="14"/>
@@ -2410,7 +2459,7 @@
       <c r="Z17" s="17"/>
       <c r="AA17" s="15">
         <f t="shared" si="1"/>
-        <v>202</v>
+        <v>235</v>
       </c>
     </row>
     <row r="18">
@@ -2484,7 +2533,9 @@
       <c r="J19" s="14">
         <v>37.0</v>
       </c>
-      <c r="K19" s="13"/>
+      <c r="K19" s="13">
+        <v>33.0</v>
+      </c>
       <c r="L19" s="14"/>
       <c r="M19" s="13"/>
       <c r="N19" s="14"/>
@@ -2502,7 +2553,7 @@
       <c r="Z19" s="17"/>
       <c r="AA19" s="15">
         <f t="shared" si="1"/>
-        <v>223</v>
+        <v>256</v>
       </c>
     </row>
     <row r="20">
@@ -2572,7 +2623,9 @@
       <c r="J21" s="14">
         <v>23.0</v>
       </c>
-      <c r="K21" s="13"/>
+      <c r="K21" s="13">
+        <v>30.0</v>
+      </c>
       <c r="L21" s="14"/>
       <c r="M21" s="13"/>
       <c r="N21" s="14"/>
@@ -2590,7 +2643,7 @@
       <c r="Z21" s="17"/>
       <c r="AA21" s="15">
         <f t="shared" si="1"/>
-        <v>236</v>
+        <v>266</v>
       </c>
     </row>
     <row r="22">
@@ -2650,7 +2703,9 @@
       <c r="J23" s="14">
         <v>14.0</v>
       </c>
-      <c r="K23" s="13"/>
+      <c r="K23" s="13">
+        <v>25.0</v>
+      </c>
       <c r="L23" s="14"/>
       <c r="M23" s="13"/>
       <c r="N23" s="14"/>
@@ -2668,7 +2723,7 @@
       <c r="Z23" s="17"/>
       <c r="AA23" s="15">
         <f t="shared" si="1"/>
-        <v>39</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24">
@@ -2697,7 +2752,9 @@
       <c r="J24" s="14">
         <v>29.0</v>
       </c>
-      <c r="K24" s="13"/>
+      <c r="K24" s="13">
+        <v>31.0</v>
+      </c>
       <c r="L24" s="14"/>
       <c r="M24" s="13"/>
       <c r="N24" s="14"/>
@@ -2715,7 +2772,7 @@
       <c r="Z24" s="17"/>
       <c r="AA24" s="15">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>256</v>
       </c>
     </row>
     <row r="25">
@@ -2744,7 +2801,9 @@
       <c r="J25" s="14">
         <v>32.0</v>
       </c>
-      <c r="K25" s="13"/>
+      <c r="K25" s="13">
+        <v>35.0</v>
+      </c>
       <c r="L25" s="14"/>
       <c r="M25" s="13"/>
       <c r="N25" s="14"/>
@@ -2762,7 +2821,7 @@
       <c r="Z25" s="17"/>
       <c r="AA25" s="15">
         <f t="shared" si="1"/>
-        <v>200</v>
+        <v>235</v>
       </c>
     </row>
     <row r="26" ht="9.0" customHeight="1">
@@ -2819,7 +2878,9 @@
       <c r="J27" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="K27" s="24"/>
+      <c r="K27" s="24" t="s">
+        <v>39</v>
+      </c>
       <c r="L27" s="24"/>
       <c r="M27" s="24"/>
       <c r="N27" s="24"/>
@@ -2865,7 +2926,9 @@
       <c r="J28" s="27">
         <v>40.0</v>
       </c>
-      <c r="K28" s="27"/>
+      <c r="K28" s="27">
+        <v>38.0</v>
+      </c>
       <c r="L28" s="27"/>
       <c r="M28" s="27"/>
       <c r="N28" s="27"/>
@@ -7220,13 +7283,17 @@
       <c r="B9" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="C9" s="43"/>
+      <c r="C9" s="43" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14">
         <v>9.0</v>
       </c>
-      <c r="B10" s="42"/>
+      <c r="B10" s="42" t="s">
+        <v>87</v>
+      </c>
       <c r="C10" s="43"/>
       <c r="G10" s="15"/>
     </row>
@@ -12212,16 +12279,16 @@
         <v>76</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D1" s="44" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2">
@@ -12385,11 +12452,11 @@
       </c>
       <c r="D9" s="46" t="str">
         <f>'THURSDAY SINGLES'!J20</f>
-        <v/>
-      </c>
-      <c r="E9" s="45" t="str">
+        <v>JOHN ANTCLIFFE</v>
+      </c>
+      <c r="E9" s="45">
         <f>'THURSDAY SINGLES'!J$21</f>
-        <v/>
+        <v>38</v>
       </c>
     </row>
     <row r="10">
@@ -12398,11 +12465,11 @@
       </c>
       <c r="B10" s="45" t="str">
         <f>'SUNDAY SINGLES'!K27</f>
-        <v/>
-      </c>
-      <c r="C10" s="45" t="str">
+        <v>MARTIN BROCK</v>
+      </c>
+      <c r="C10" s="45">
         <f>'SUNDAY SINGLES'!K28</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="D10" s="46" t="str">
         <f>'THURSDAY SINGLES'!K20</f>

</xml_diff>

<commit_message>
101 Week 11 data update
</commit_message>
<xml_diff>
--- a/data/SUMMER_GOLF_2026.xlsx
+++ b/data/SUMMER_GOLF_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="99">
   <si>
     <t>SUMMER GOLF 2026 - THURSDAY SINGLES</t>
   </si>
@@ -1933,7 +1933,9 @@
         <v>36.0</v>
       </c>
       <c r="L5" s="16"/>
-      <c r="M5" s="17"/>
+      <c r="M5" s="14">
+        <v>24.0</v>
+      </c>
       <c r="N5" s="15"/>
       <c r="O5" s="17"/>
       <c r="P5" s="15"/>
@@ -1949,7 +1951,7 @@
       <c r="Z5" s="20"/>
       <c r="AA5" s="16">
         <f t="shared" ref="AA5:AA25" si="1">SUM(C5:Z5)</f>
-        <v>116</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6">
@@ -2029,7 +2031,9 @@
         <v>32.0</v>
       </c>
       <c r="L7" s="15"/>
-      <c r="M7" s="14"/>
+      <c r="M7" s="14">
+        <v>25.0</v>
+      </c>
       <c r="N7" s="15"/>
       <c r="O7" s="17"/>
       <c r="P7" s="15"/>
@@ -2045,7 +2049,7 @@
       <c r="Z7" s="18"/>
       <c r="AA7" s="16">
         <f t="shared" si="1"/>
-        <v>288</v>
+        <v>313</v>
       </c>
     </row>
     <row r="8">
@@ -2078,7 +2082,9 @@
         <v>33.0</v>
       </c>
       <c r="L8" s="15"/>
-      <c r="M8" s="14"/>
+      <c r="M8" s="14">
+        <v>39.0</v>
+      </c>
       <c r="N8" s="15"/>
       <c r="O8" s="14"/>
       <c r="P8" s="15"/>
@@ -2094,7 +2100,7 @@
       <c r="Z8" s="18"/>
       <c r="AA8" s="16">
         <f t="shared" si="1"/>
-        <v>243</v>
+        <v>282</v>
       </c>
     </row>
     <row r="9">
@@ -2121,7 +2127,9 @@
         <v>33.0</v>
       </c>
       <c r="L9" s="15"/>
-      <c r="M9" s="14"/>
+      <c r="M9" s="14">
+        <v>31.0</v>
+      </c>
       <c r="N9" s="15"/>
       <c r="O9" s="14"/>
       <c r="P9" s="16"/>
@@ -2137,7 +2145,7 @@
       <c r="Z9" s="18"/>
       <c r="AA9" s="16">
         <f t="shared" si="1"/>
-        <v>145</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10">
@@ -2160,7 +2168,9 @@
         <v>29.0</v>
       </c>
       <c r="L10" s="15"/>
-      <c r="M10" s="14"/>
+      <c r="M10" s="14">
+        <v>39.0</v>
+      </c>
       <c r="N10" s="15"/>
       <c r="O10" s="14"/>
       <c r="P10" s="16"/>
@@ -2176,7 +2186,7 @@
       <c r="Z10" s="20"/>
       <c r="AA10" s="16">
         <f t="shared" si="1"/>
-        <v>81</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11">
@@ -2209,7 +2219,9 @@
         <v>35.0</v>
       </c>
       <c r="L11" s="16"/>
-      <c r="M11" s="14"/>
+      <c r="M11" s="14">
+        <v>27.0</v>
+      </c>
       <c r="N11" s="16"/>
       <c r="O11" s="14"/>
       <c r="P11" s="15"/>
@@ -2225,7 +2237,7 @@
       <c r="Z11" s="18"/>
       <c r="AA11" s="16">
         <f t="shared" si="1"/>
-        <v>259</v>
+        <v>286</v>
       </c>
     </row>
     <row r="12">
@@ -2291,7 +2303,9 @@
       </c>
       <c r="K13" s="14"/>
       <c r="L13" s="15"/>
-      <c r="M13" s="14"/>
+      <c r="M13" s="14">
+        <v>39.0</v>
+      </c>
       <c r="N13" s="15"/>
       <c r="O13" s="14"/>
       <c r="P13" s="15"/>
@@ -2307,7 +2321,7 @@
       <c r="Z13" s="18"/>
       <c r="AA13" s="16">
         <f t="shared" si="1"/>
-        <v>146</v>
+        <v>185</v>
       </c>
     </row>
     <row r="14">
@@ -2338,7 +2352,9 @@
         <v>32.0</v>
       </c>
       <c r="L14" s="15"/>
-      <c r="M14" s="17"/>
+      <c r="M14" s="14">
+        <v>36.0</v>
+      </c>
       <c r="N14" s="16"/>
       <c r="O14" s="17"/>
       <c r="P14" s="16"/>
@@ -2354,7 +2370,7 @@
       <c r="Z14" s="18"/>
       <c r="AA14" s="16">
         <f t="shared" si="1"/>
-        <v>204</v>
+        <v>240</v>
       </c>
     </row>
     <row r="15">
@@ -2385,7 +2401,9 @@
       </c>
       <c r="K15" s="17"/>
       <c r="L15" s="16"/>
-      <c r="M15" s="17"/>
+      <c r="M15" s="14">
+        <v>28.0</v>
+      </c>
       <c r="N15" s="15"/>
       <c r="O15" s="14"/>
       <c r="P15" s="15"/>
@@ -2401,7 +2419,7 @@
       <c r="Z15" s="18"/>
       <c r="AA15" s="16">
         <f t="shared" si="1"/>
-        <v>207</v>
+        <v>235</v>
       </c>
     </row>
     <row r="16">
@@ -2483,7 +2501,9 @@
         <v>33.0</v>
       </c>
       <c r="L17" s="15"/>
-      <c r="M17" s="14"/>
+      <c r="M17" s="14">
+        <v>33.0</v>
+      </c>
       <c r="N17" s="15"/>
       <c r="O17" s="14"/>
       <c r="P17" s="15"/>
@@ -2499,7 +2519,7 @@
       <c r="Z17" s="18"/>
       <c r="AA17" s="16">
         <f t="shared" si="1"/>
-        <v>235</v>
+        <v>268</v>
       </c>
     </row>
     <row r="18">
@@ -2528,7 +2548,9 @@
       </c>
       <c r="K18" s="14"/>
       <c r="L18" s="15"/>
-      <c r="M18" s="14"/>
+      <c r="M18" s="14">
+        <v>31.0</v>
+      </c>
       <c r="N18" s="16"/>
       <c r="O18" s="17"/>
       <c r="P18" s="16"/>
@@ -2544,7 +2566,7 @@
       <c r="Z18" s="18"/>
       <c r="AA18" s="16">
         <f t="shared" si="1"/>
-        <v>189</v>
+        <v>220</v>
       </c>
     </row>
     <row r="19">
@@ -2671,7 +2693,9 @@
       <c r="L21" s="15">
         <v>29.0</v>
       </c>
-      <c r="M21" s="14"/>
+      <c r="M21" s="14">
+        <v>28.0</v>
+      </c>
       <c r="N21" s="15"/>
       <c r="O21" s="14"/>
       <c r="P21" s="16"/>
@@ -2687,7 +2711,7 @@
       <c r="Z21" s="18"/>
       <c r="AA21" s="16">
         <f t="shared" si="1"/>
-        <v>295</v>
+        <v>323</v>
       </c>
     </row>
     <row r="22">
@@ -2712,7 +2736,9 @@
       </c>
       <c r="K22" s="14"/>
       <c r="L22" s="15"/>
-      <c r="M22" s="14"/>
+      <c r="M22" s="14">
+        <v>32.0</v>
+      </c>
       <c r="N22" s="15"/>
       <c r="O22" s="14"/>
       <c r="P22" s="16"/>
@@ -2728,7 +2754,7 @@
       <c r="Z22" s="18"/>
       <c r="AA22" s="16">
         <f t="shared" si="1"/>
-        <v>147</v>
+        <v>179</v>
       </c>
     </row>
     <row r="23">
@@ -2851,7 +2877,9 @@
         <v>35.0</v>
       </c>
       <c r="L25" s="15"/>
-      <c r="M25" s="14"/>
+      <c r="M25" s="14">
+        <v>40.0</v>
+      </c>
       <c r="N25" s="15"/>
       <c r="O25" s="14"/>
       <c r="P25" s="16"/>
@@ -2867,7 +2895,7 @@
       <c r="Z25" s="18"/>
       <c r="AA25" s="16">
         <f t="shared" si="1"/>
-        <v>235</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26" ht="9.0" customHeight="1">
@@ -2930,7 +2958,9 @@
       <c r="L27" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="M27" s="25"/>
+      <c r="M27" s="25" t="s">
+        <v>72</v>
+      </c>
       <c r="N27" s="25"/>
       <c r="O27" s="25"/>
       <c r="P27" s="25"/>
@@ -2980,7 +3010,9 @@
       <c r="L28" s="28">
         <v>34.0</v>
       </c>
-      <c r="M28" s="28"/>
+      <c r="M28" s="28">
+        <v>40.0</v>
+      </c>
       <c r="N28" s="28"/>
       <c r="O28" s="28"/>
       <c r="P28" s="28"/>
@@ -3029,10 +3061,10 @@
         <v>47</v>
       </c>
       <c r="B2" s="34">
+        <v>19.0</v>
+      </c>
+      <c r="C2" s="35">
         <v>18.0</v>
-      </c>
-      <c r="C2" s="35">
-        <v>17.0</v>
       </c>
     </row>
     <row r="3">
@@ -3040,10 +3072,10 @@
         <v>35</v>
       </c>
       <c r="B3" s="34">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
       <c r="C3" s="35">
-        <v>12.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="4">
@@ -3065,7 +3097,7 @@
         <v>11.0</v>
       </c>
       <c r="C5" s="35">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="6">
@@ -3095,7 +3127,7 @@
         <v>39</v>
       </c>
       <c r="B8" s="34">
-        <v>33.0</v>
+        <v>32.0</v>
       </c>
       <c r="C8" s="35">
         <v>31.0</v>
@@ -3128,7 +3160,7 @@
         <v>65</v>
       </c>
       <c r="B11" s="34">
-        <v>22.0</v>
+        <v>23.0</v>
       </c>
       <c r="C11" s="35">
         <v>21.0</v>
@@ -3139,10 +3171,10 @@
         <v>42</v>
       </c>
       <c r="B12" s="34">
-        <v>9.0</v>
+        <v>10.0</v>
       </c>
       <c r="C12" s="36">
-        <v>7.0</v>
+        <v>8.0</v>
       </c>
     </row>
     <row r="13">
@@ -3194,10 +3226,10 @@
         <v>41</v>
       </c>
       <c r="B17" s="34">
+        <v>13.0</v>
+      </c>
+      <c r="C17" s="35">
         <v>12.0</v>
-      </c>
-      <c r="C17" s="35">
-        <v>11.0</v>
       </c>
     </row>
     <row r="18">
@@ -3205,10 +3237,10 @@
         <v>63</v>
       </c>
       <c r="B18" s="34">
+        <v>0.0</v>
+      </c>
+      <c r="C18" s="35">
         <v>-1.0</v>
-      </c>
-      <c r="C18" s="35">
-        <v>-2.0</v>
       </c>
     </row>
     <row r="19">
@@ -3227,7 +3259,7 @@
         <v>40</v>
       </c>
       <c r="B20" s="34">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
       <c r="C20" s="35">
         <v>14.0</v>
@@ -3263,7 +3295,7 @@
         <v>33.0</v>
       </c>
       <c r="C23" s="35">
-        <v>32.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="24">
@@ -3318,7 +3350,7 @@
         <v>23.0</v>
       </c>
       <c r="C28" s="15">
-        <v>21.0</v>
+        <v>22.0</v>
       </c>
     </row>
     <row r="29">
@@ -7356,13 +7388,17 @@
       <c r="B11" s="43" t="s">
         <v>94</v>
       </c>
-      <c r="C11" s="44"/>
+      <c r="C11" s="44" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="15">
         <v>11.0</v>
       </c>
-      <c r="B12" s="43"/>
+      <c r="B12" s="43" t="s">
+        <v>75</v>
+      </c>
       <c r="C12" s="44"/>
     </row>
     <row r="13">
@@ -12561,11 +12597,11 @@
       </c>
       <c r="B12" s="46" t="str">
         <f>'SUNDAY SINGLES'!M27</f>
-        <v/>
-      </c>
-      <c r="C12" s="46" t="str">
+        <v>HELEN RIGG</v>
+      </c>
+      <c r="C12" s="46">
         <f>'SUNDAY SINGLES'!M28</f>
-        <v/>
+        <v>40</v>
       </c>
       <c r="D12" s="47" t="str">
         <f>'THURSDAY SINGLES'!M20</f>

</xml_diff>

<commit_message>
102 Week 11/12 data update
</commit_message>
<xml_diff>
--- a/data/SUMMER_GOLF_2026.xlsx
+++ b/data/SUMMER_GOLF_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="100">
   <si>
     <t>SUMMER GOLF 2026 - THURSDAY SINGLES</t>
   </si>
@@ -170,6 +170,9 @@
     <t>STEVE  FELLOWS</t>
   </si>
   <si>
+    <t>STEW TAYLOR</t>
+  </si>
+  <si>
     <t>WINNERS SCORE</t>
   </si>
   <si>
@@ -236,9 +239,6 @@
     <t>HELEN RIGG</t>
   </si>
   <si>
-    <t>STEW TAYLOR</t>
-  </si>
-  <si>
     <t>DAVE CROSSLEY</t>
   </si>
   <si>
@@ -300,6 +300,9 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>ARTHUR YOUNG/RYAN JACKSON</t>
   </si>
   <si>
     <t>SUNDAY</t>
@@ -1030,7 +1033,9 @@
       </c>
       <c r="K5" s="14"/>
       <c r="L5" s="16"/>
-      <c r="M5" s="14"/>
+      <c r="M5" s="14">
+        <v>31.0</v>
+      </c>
       <c r="N5" s="16"/>
       <c r="O5" s="14"/>
       <c r="P5" s="15"/>
@@ -1046,7 +1051,7 @@
       <c r="Z5" s="18"/>
       <c r="AA5" s="16">
         <f t="shared" ref="AA5:AA18" si="1">sum(C5:Z5)</f>
-        <v>180</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6">
@@ -1079,7 +1084,9 @@
       </c>
       <c r="K6" s="14"/>
       <c r="L6" s="15"/>
-      <c r="M6" s="14"/>
+      <c r="M6" s="14">
+        <v>36.0</v>
+      </c>
       <c r="N6" s="15"/>
       <c r="O6" s="17"/>
       <c r="P6" s="15"/>
@@ -1095,7 +1102,7 @@
       <c r="Z6" s="18"/>
       <c r="AA6" s="16">
         <f t="shared" si="1"/>
-        <v>238</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7">
@@ -1173,7 +1180,9 @@
       </c>
       <c r="K8" s="17"/>
       <c r="L8" s="16"/>
-      <c r="M8" s="14"/>
+      <c r="M8" s="14">
+        <v>33.0</v>
+      </c>
       <c r="N8" s="15"/>
       <c r="O8" s="14"/>
       <c r="P8" s="15"/>
@@ -1189,7 +1198,7 @@
       <c r="Z8" s="20"/>
       <c r="AA8" s="16">
         <f t="shared" si="1"/>
-        <v>261</v>
+        <v>294</v>
       </c>
     </row>
     <row r="9">
@@ -1222,7 +1231,9 @@
       </c>
       <c r="K9" s="14"/>
       <c r="L9" s="15"/>
-      <c r="M9" s="14"/>
+      <c r="M9" s="14">
+        <v>33.0</v>
+      </c>
       <c r="N9" s="15"/>
       <c r="O9" s="14"/>
       <c r="P9" s="15"/>
@@ -1238,7 +1249,7 @@
       <c r="Z9" s="18"/>
       <c r="AA9" s="16">
         <f t="shared" si="1"/>
-        <v>243</v>
+        <v>276</v>
       </c>
     </row>
     <row r="10">
@@ -1269,7 +1280,9 @@
       </c>
       <c r="K10" s="17"/>
       <c r="L10" s="16"/>
-      <c r="M10" s="14"/>
+      <c r="M10" s="14">
+        <v>32.0</v>
+      </c>
       <c r="N10" s="15"/>
       <c r="O10" s="17"/>
       <c r="P10" s="15"/>
@@ -1285,7 +1298,7 @@
       <c r="Z10" s="18"/>
       <c r="AA10" s="16">
         <f t="shared" si="1"/>
-        <v>221</v>
+        <v>253</v>
       </c>
     </row>
     <row r="11">
@@ -1406,7 +1419,9 @@
       </c>
       <c r="K13" s="14"/>
       <c r="L13" s="16"/>
-      <c r="M13" s="17"/>
+      <c r="M13" s="14">
+        <v>36.0</v>
+      </c>
       <c r="N13" s="16"/>
       <c r="O13" s="17"/>
       <c r="P13" s="15"/>
@@ -1422,7 +1437,7 @@
       <c r="Z13" s="18"/>
       <c r="AA13" s="16">
         <f t="shared" si="1"/>
-        <v>218</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14">
@@ -1451,7 +1466,9 @@
       </c>
       <c r="K14" s="14"/>
       <c r="L14" s="15"/>
-      <c r="M14" s="14"/>
+      <c r="M14" s="14">
+        <v>29.0</v>
+      </c>
       <c r="N14" s="15"/>
       <c r="O14" s="14"/>
       <c r="P14" s="15"/>
@@ -1467,7 +1484,7 @@
       <c r="Z14" s="18"/>
       <c r="AA14" s="16">
         <f t="shared" si="1"/>
-        <v>179</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15">
@@ -1580,7 +1597,9 @@
       </c>
       <c r="K17" s="14"/>
       <c r="L17" s="16"/>
-      <c r="M17" s="17"/>
+      <c r="M17" s="14">
+        <v>29.0</v>
+      </c>
       <c r="N17" s="16"/>
       <c r="O17" s="14"/>
       <c r="P17" s="15"/>
@@ -1596,7 +1615,7 @@
       <c r="Z17" s="18"/>
       <c r="AA17" s="16">
         <f t="shared" si="1"/>
-        <v>177</v>
+        <v>206</v>
       </c>
     </row>
     <row r="18">
@@ -1692,7 +1711,9 @@
       </c>
       <c r="K20" s="25"/>
       <c r="L20" s="25"/>
-      <c r="M20" s="25"/>
+      <c r="M20" s="25" t="s">
+        <v>51</v>
+      </c>
       <c r="N20" s="25"/>
       <c r="O20" s="25"/>
       <c r="P20" s="25"/>
@@ -1710,7 +1731,7 @@
     </row>
     <row r="21">
       <c r="B21" s="27" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C21" s="28">
         <v>39.0</v>
@@ -1738,7 +1759,9 @@
       </c>
       <c r="K21" s="28"/>
       <c r="L21" s="28"/>
-      <c r="M21" s="28"/>
+      <c r="M21" s="28">
+        <v>36.0</v>
+      </c>
       <c r="N21" s="28"/>
       <c r="O21" s="28"/>
       <c r="P21" s="28"/>
@@ -1773,7 +1796,7 @@
   <sheetData>
     <row r="2" ht="24.0" customHeight="1">
       <c r="B2" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
@@ -1786,10 +1809,10 @@
         <v>46360.0</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G3" s="3">
         <v>46086.0</v>
@@ -1798,25 +1821,25 @@
         <v>46300.0</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L3" s="6">
         <v>46209.0</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="P3" s="4"/>
       <c r="Q3" s="5"/>
@@ -1913,7 +1936,7 @@
     </row>
     <row r="5">
       <c r="B5" s="13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C5" s="14">
         <v>24.0</v>
@@ -1936,7 +1959,9 @@
       <c r="M5" s="14">
         <v>24.0</v>
       </c>
-      <c r="N5" s="15"/>
+      <c r="N5" s="15">
+        <v>33.0</v>
+      </c>
       <c r="O5" s="17"/>
       <c r="P5" s="15"/>
       <c r="Q5" s="14"/>
@@ -1951,12 +1976,12 @@
       <c r="Z5" s="20"/>
       <c r="AA5" s="16">
         <f t="shared" ref="AA5:AA25" si="1">SUM(C5:Z5)</f>
-        <v>140</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C6" s="14">
         <v>28.0</v>
@@ -1981,7 +2006,9 @@
       <c r="K6" s="14"/>
       <c r="L6" s="16"/>
       <c r="M6" s="14"/>
-      <c r="N6" s="15"/>
+      <c r="N6" s="15">
+        <v>29.0</v>
+      </c>
       <c r="O6" s="14"/>
       <c r="P6" s="16"/>
       <c r="Q6" s="17"/>
@@ -1996,7 +2023,7 @@
       <c r="Z6" s="18"/>
       <c r="AA6" s="16">
         <f t="shared" si="1"/>
-        <v>186</v>
+        <v>215</v>
       </c>
     </row>
     <row r="7">
@@ -2034,7 +2061,9 @@
       <c r="M7" s="14">
         <v>25.0</v>
       </c>
-      <c r="N7" s="15"/>
+      <c r="N7" s="15">
+        <v>36.0</v>
+      </c>
       <c r="O7" s="17"/>
       <c r="P7" s="15"/>
       <c r="Q7" s="14"/>
@@ -2049,7 +2078,7 @@
       <c r="Z7" s="18"/>
       <c r="AA7" s="16">
         <f t="shared" si="1"/>
-        <v>313</v>
+        <v>349</v>
       </c>
     </row>
     <row r="8">
@@ -2105,7 +2134,7 @@
     </row>
     <row r="9">
       <c r="B9" s="19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C9" s="14">
         <v>24.0</v>
@@ -2130,7 +2159,9 @@
       <c r="M9" s="14">
         <v>31.0</v>
       </c>
-      <c r="N9" s="15"/>
+      <c r="N9" s="15">
+        <v>29.0</v>
+      </c>
       <c r="O9" s="14"/>
       <c r="P9" s="16"/>
       <c r="Q9" s="17"/>
@@ -2145,7 +2176,7 @@
       <c r="Z9" s="18"/>
       <c r="AA9" s="16">
         <f t="shared" si="1"/>
-        <v>176</v>
+        <v>205</v>
       </c>
     </row>
     <row r="10">
@@ -2171,7 +2202,9 @@
       <c r="M10" s="14">
         <v>39.0</v>
       </c>
-      <c r="N10" s="15"/>
+      <c r="N10" s="15">
+        <v>35.0</v>
+      </c>
       <c r="O10" s="14"/>
       <c r="P10" s="16"/>
       <c r="Q10" s="14"/>
@@ -2186,12 +2219,12 @@
       <c r="Z10" s="20"/>
       <c r="AA10" s="16">
         <f t="shared" si="1"/>
-        <v>120</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="19" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="15">
@@ -2222,7 +2255,9 @@
       <c r="M11" s="14">
         <v>27.0</v>
       </c>
-      <c r="N11" s="16"/>
+      <c r="N11" s="15">
+        <v>39.0</v>
+      </c>
       <c r="O11" s="14"/>
       <c r="P11" s="15"/>
       <c r="Q11" s="14"/>
@@ -2237,7 +2272,7 @@
       <c r="Z11" s="18"/>
       <c r="AA11" s="16">
         <f t="shared" si="1"/>
-        <v>286</v>
+        <v>325</v>
       </c>
     </row>
     <row r="12">
@@ -2281,7 +2316,7 @@
     </row>
     <row r="13">
       <c r="B13" s="19" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C13" s="14">
         <v>28.0</v>
@@ -2306,7 +2341,9 @@
       <c r="M13" s="14">
         <v>39.0</v>
       </c>
-      <c r="N13" s="15"/>
+      <c r="N13" s="15">
+        <v>30.0</v>
+      </c>
       <c r="O13" s="14"/>
       <c r="P13" s="15"/>
       <c r="Q13" s="14"/>
@@ -2321,7 +2358,7 @@
       <c r="Z13" s="18"/>
       <c r="AA13" s="16">
         <f t="shared" si="1"/>
-        <v>185</v>
+        <v>215</v>
       </c>
     </row>
     <row r="14">
@@ -2355,7 +2392,9 @@
       <c r="M14" s="14">
         <v>36.0</v>
       </c>
-      <c r="N14" s="16"/>
+      <c r="N14" s="15">
+        <v>34.0</v>
+      </c>
       <c r="O14" s="17"/>
       <c r="P14" s="16"/>
       <c r="Q14" s="14"/>
@@ -2370,7 +2409,7 @@
       <c r="Z14" s="18"/>
       <c r="AA14" s="16">
         <f t="shared" si="1"/>
-        <v>240</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15">
@@ -2404,7 +2443,9 @@
       <c r="M15" s="14">
         <v>28.0</v>
       </c>
-      <c r="N15" s="15"/>
+      <c r="N15" s="15">
+        <v>38.0</v>
+      </c>
       <c r="O15" s="14"/>
       <c r="P15" s="15"/>
       <c r="Q15" s="14"/>
@@ -2419,7 +2460,7 @@
       <c r="Z15" s="18"/>
       <c r="AA15" s="16">
         <f t="shared" si="1"/>
-        <v>235</v>
+        <v>273</v>
       </c>
     </row>
     <row r="16">
@@ -2455,7 +2496,9 @@
       </c>
       <c r="L16" s="15"/>
       <c r="M16" s="14"/>
-      <c r="N16" s="15"/>
+      <c r="N16" s="15">
+        <v>32.0</v>
+      </c>
       <c r="O16" s="14"/>
       <c r="P16" s="16"/>
       <c r="Q16" s="14"/>
@@ -2470,12 +2513,12 @@
       <c r="Z16" s="18"/>
       <c r="AA16" s="16">
         <f t="shared" si="1"/>
-        <v>199</v>
+        <v>231</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="19" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C17" s="14">
         <v>32.0</v>
@@ -2504,7 +2547,9 @@
       <c r="M17" s="14">
         <v>33.0</v>
       </c>
-      <c r="N17" s="15"/>
+      <c r="N17" s="15">
+        <v>37.0</v>
+      </c>
       <c r="O17" s="14"/>
       <c r="P17" s="15"/>
       <c r="Q17" s="14"/>
@@ -2519,12 +2564,12 @@
       <c r="Z17" s="18"/>
       <c r="AA17" s="16">
         <f t="shared" si="1"/>
-        <v>268</v>
+        <v>305</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C18" s="14">
         <v>30.0</v>
@@ -2551,7 +2596,9 @@
       <c r="M18" s="14">
         <v>31.0</v>
       </c>
-      <c r="N18" s="16"/>
+      <c r="N18" s="15">
+        <v>31.0</v>
+      </c>
       <c r="O18" s="17"/>
       <c r="P18" s="16"/>
       <c r="Q18" s="14"/>
@@ -2566,12 +2613,12 @@
       <c r="Z18" s="18"/>
       <c r="AA18" s="16">
         <f t="shared" si="1"/>
-        <v>220</v>
+        <v>251</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C19" s="14">
         <v>28.0</v>
@@ -2661,7 +2708,7 @@
     </row>
     <row r="21">
       <c r="B21" s="19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C21" s="14">
         <v>20.0</v>
@@ -2696,7 +2743,9 @@
       <c r="M21" s="14">
         <v>28.0</v>
       </c>
-      <c r="N21" s="15"/>
+      <c r="N21" s="15">
+        <v>32.0</v>
+      </c>
       <c r="O21" s="14"/>
       <c r="P21" s="16"/>
       <c r="Q21" s="14"/>
@@ -2711,7 +2760,7 @@
       <c r="Z21" s="18"/>
       <c r="AA21" s="16">
         <f t="shared" si="1"/>
-        <v>323</v>
+        <v>355</v>
       </c>
     </row>
     <row r="22">
@@ -2759,7 +2808,7 @@
     </row>
     <row r="23">
       <c r="B23" s="19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C23" s="14"/>
       <c r="D23" s="15">
@@ -2800,7 +2849,7 @@
     </row>
     <row r="24">
       <c r="B24" s="19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C24" s="14">
         <v>35.0</v>
@@ -2829,7 +2878,9 @@
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="14"/>
-      <c r="N24" s="15"/>
+      <c r="N24" s="15">
+        <v>25.0</v>
+      </c>
       <c r="O24" s="14"/>
       <c r="P24" s="16"/>
       <c r="Q24" s="14"/>
@@ -2844,12 +2895,12 @@
       <c r="Z24" s="18"/>
       <c r="AA24" s="16">
         <f t="shared" si="1"/>
-        <v>256</v>
+        <v>281</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C25" s="14">
         <v>19.0</v>
@@ -2929,10 +2980,10 @@
         <v>49</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E27" s="25" t="s">
         <v>39</v>
@@ -2941,7 +2992,7 @@
         <v>45</v>
       </c>
       <c r="G27" s="25" t="s">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="H27" s="25" t="s">
         <v>74</v>
@@ -2959,9 +3010,11 @@
         <v>75</v>
       </c>
       <c r="M27" s="25" t="s">
-        <v>72</v>
-      </c>
-      <c r="N27" s="25"/>
+        <v>73</v>
+      </c>
+      <c r="N27" s="25" t="s">
+        <v>65</v>
+      </c>
       <c r="O27" s="25"/>
       <c r="P27" s="25"/>
       <c r="Q27" s="25"/>
@@ -2978,7 +3031,7 @@
     </row>
     <row r="28">
       <c r="B28" s="27" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C28" s="28">
         <v>35.0</v>
@@ -3013,7 +3066,9 @@
       <c r="M28" s="28">
         <v>40.0</v>
       </c>
-      <c r="N28" s="28"/>
+      <c r="N28" s="28">
+        <v>39.0</v>
+      </c>
       <c r="O28" s="28"/>
       <c r="P28" s="28"/>
       <c r="Q28" s="28"/>
@@ -3080,7 +3135,7 @@
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="B4" s="34">
         <v>10.0</v>
@@ -3135,7 +3190,7 @@
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B9" s="34">
         <v>9.0</v>
@@ -3157,7 +3212,7 @@
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B11" s="34">
         <v>23.0</v>
@@ -3179,7 +3234,7 @@
     </row>
     <row r="13">
       <c r="A13" s="19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B13" s="34">
         <v>12.0</v>
@@ -3190,7 +3245,7 @@
     </row>
     <row r="14">
       <c r="A14" s="19" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B14" s="34">
         <v>20.0</v>
@@ -3201,7 +3256,7 @@
     </row>
     <row r="15">
       <c r="A15" s="19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B15" s="34">
         <v>7.0</v>
@@ -3212,7 +3267,7 @@
     </row>
     <row r="16">
       <c r="A16" s="19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B16" s="34">
         <v>15.0</v>
@@ -3234,7 +3289,7 @@
     </row>
     <row r="18">
       <c r="A18" s="19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B18" s="34">
         <v>0.0</v>
@@ -3267,7 +3322,7 @@
     </row>
     <row r="21">
       <c r="A21" s="19" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B21" s="34">
         <v>7.0</v>
@@ -3300,7 +3355,7 @@
     </row>
     <row r="24">
       <c r="A24" s="37" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B24" s="34">
         <v>27.0</v>
@@ -3311,7 +3366,7 @@
     </row>
     <row r="25">
       <c r="A25" s="37" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B25" s="34">
         <v>19.0</v>
@@ -3344,7 +3399,7 @@
     </row>
     <row r="28">
       <c r="A28" s="37" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B28" s="15">
         <v>23.0</v>
@@ -3355,7 +3410,7 @@
     </row>
     <row r="29">
       <c r="A29" s="37" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B29" s="15">
         <v>23.0</v>
@@ -7322,7 +7377,7 @@
         <v>88</v>
       </c>
       <c r="C5" s="44" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6">
@@ -7399,13 +7454,17 @@
       <c r="B12" s="43" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="44"/>
+      <c r="C12" s="44" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="15">
         <v>12.0</v>
       </c>
-      <c r="B13" s="43"/>
+      <c r="B13" s="43" t="s">
+        <v>95</v>
+      </c>
       <c r="C13" s="44"/>
     </row>
     <row r="14">
@@ -12369,16 +12428,16 @@
         <v>82</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2">
@@ -12605,11 +12664,11 @@
       </c>
       <c r="D12" s="47" t="str">
         <f>'THURSDAY SINGLES'!M20</f>
-        <v/>
-      </c>
-      <c r="E12" s="46" t="str">
+        <v>STEW TAYLOR</v>
+      </c>
+      <c r="E12" s="46">
         <f>'THURSDAY SINGLES'!M21</f>
-        <v/>
+        <v>36</v>
       </c>
     </row>
     <row r="13">
@@ -12618,11 +12677,11 @@
       </c>
       <c r="B13" s="46" t="str">
         <f>'SUNDAY SINGLES'!N27</f>
-        <v/>
-      </c>
-      <c r="C13" s="46" t="str">
+        <v>CHRIS DUFFY</v>
+      </c>
+      <c r="C13" s="46">
         <f>'SUNDAY SINGLES'!N28</f>
-        <v/>
+        <v>39</v>
       </c>
       <c r="D13" s="47" t="str">
         <f>'THURSDAY SINGLES'!N20</f>

</xml_diff>

<commit_message>
Week 12/13 data update
</commit_message>
<xml_diff>
--- a/data/SUMMER_GOLF_2026.xlsx
+++ b/data/SUMMER_GOLF_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="101">
   <si>
     <t>SUMMER GOLF 2026 - THURSDAY SINGLES</t>
   </si>
@@ -303,6 +303,9 @@
   </si>
   <si>
     <t>ARTHUR YOUNG/RYAN JACKSON</t>
+  </si>
+  <si>
+    <t>HELEN RIGG/BAZ MASON</t>
   </si>
   <si>
     <t>SUNDAY</t>
@@ -1036,7 +1039,9 @@
       <c r="M5" s="14">
         <v>31.0</v>
       </c>
-      <c r="N5" s="16"/>
+      <c r="N5" s="15">
+        <v>37.0</v>
+      </c>
       <c r="O5" s="14"/>
       <c r="P5" s="15"/>
       <c r="Q5" s="17"/>
@@ -1051,7 +1056,7 @@
       <c r="Z5" s="18"/>
       <c r="AA5" s="16">
         <f t="shared" ref="AA5:AA18" si="1">sum(C5:Z5)</f>
-        <v>211</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6">
@@ -1087,7 +1092,9 @@
       <c r="M6" s="14">
         <v>36.0</v>
       </c>
-      <c r="N6" s="15"/>
+      <c r="N6" s="15">
+        <v>38.0</v>
+      </c>
       <c r="O6" s="17"/>
       <c r="P6" s="15"/>
       <c r="Q6" s="14"/>
@@ -1102,7 +1109,7 @@
       <c r="Z6" s="18"/>
       <c r="AA6" s="16">
         <f t="shared" si="1"/>
-        <v>274</v>
+        <v>312</v>
       </c>
     </row>
     <row r="7">
@@ -1132,7 +1139,9 @@
       <c r="K7" s="17"/>
       <c r="L7" s="15"/>
       <c r="M7" s="14"/>
-      <c r="N7" s="15"/>
+      <c r="N7" s="15">
+        <v>37.0</v>
+      </c>
       <c r="O7" s="14"/>
       <c r="P7" s="15"/>
       <c r="Q7" s="14"/>
@@ -1147,7 +1156,7 @@
       <c r="Z7" s="18"/>
       <c r="AA7" s="16">
         <f t="shared" si="1"/>
-        <v>190</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8">
@@ -1183,7 +1192,9 @@
       <c r="M8" s="14">
         <v>33.0</v>
       </c>
-      <c r="N8" s="15"/>
+      <c r="N8" s="15">
+        <v>36.0</v>
+      </c>
       <c r="O8" s="14"/>
       <c r="P8" s="15"/>
       <c r="Q8" s="14"/>
@@ -1198,7 +1209,7 @@
       <c r="Z8" s="20"/>
       <c r="AA8" s="16">
         <f t="shared" si="1"/>
-        <v>294</v>
+        <v>330</v>
       </c>
     </row>
     <row r="9">
@@ -1283,7 +1294,9 @@
       <c r="M10" s="14">
         <v>32.0</v>
       </c>
-      <c r="N10" s="15"/>
+      <c r="N10" s="15">
+        <v>34.0</v>
+      </c>
       <c r="O10" s="17"/>
       <c r="P10" s="15"/>
       <c r="Q10" s="14"/>
@@ -1298,7 +1311,7 @@
       <c r="Z10" s="18"/>
       <c r="AA10" s="16">
         <f t="shared" si="1"/>
-        <v>253</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11">
@@ -1373,7 +1386,9 @@
       <c r="K12" s="14"/>
       <c r="L12" s="15"/>
       <c r="M12" s="14"/>
-      <c r="N12" s="16"/>
+      <c r="N12" s="15">
+        <v>37.0</v>
+      </c>
       <c r="O12" s="14"/>
       <c r="P12" s="15"/>
       <c r="Q12" s="14"/>
@@ -1388,7 +1403,7 @@
       <c r="Z12" s="18"/>
       <c r="AA12" s="16">
         <f t="shared" si="1"/>
-        <v>181</v>
+        <v>218</v>
       </c>
     </row>
     <row r="13">
@@ -1422,7 +1437,9 @@
       <c r="M13" s="14">
         <v>36.0</v>
       </c>
-      <c r="N13" s="16"/>
+      <c r="N13" s="15">
+        <v>36.0</v>
+      </c>
       <c r="O13" s="17"/>
       <c r="P13" s="15"/>
       <c r="Q13" s="14"/>
@@ -1437,7 +1454,7 @@
       <c r="Z13" s="18"/>
       <c r="AA13" s="16">
         <f t="shared" si="1"/>
-        <v>254</v>
+        <v>290</v>
       </c>
     </row>
     <row r="14">
@@ -1469,7 +1486,9 @@
       <c r="M14" s="14">
         <v>29.0</v>
       </c>
-      <c r="N14" s="15"/>
+      <c r="N14" s="15">
+        <v>36.0</v>
+      </c>
       <c r="O14" s="14"/>
       <c r="P14" s="15"/>
       <c r="Q14" s="14"/>
@@ -1484,7 +1503,7 @@
       <c r="Z14" s="18"/>
       <c r="AA14" s="16">
         <f t="shared" si="1"/>
-        <v>208</v>
+        <v>244</v>
       </c>
     </row>
     <row r="15">
@@ -1551,7 +1570,9 @@
       <c r="K16" s="14"/>
       <c r="L16" s="16"/>
       <c r="M16" s="17"/>
-      <c r="N16" s="16"/>
+      <c r="N16" s="15">
+        <v>32.0</v>
+      </c>
       <c r="O16" s="14"/>
       <c r="P16" s="15"/>
       <c r="Q16" s="14"/>
@@ -1566,7 +1587,7 @@
       <c r="Z16" s="18"/>
       <c r="AA16" s="16">
         <f t="shared" si="1"/>
-        <v>78</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17">
@@ -1714,7 +1735,9 @@
       <c r="M20" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="N20" s="25"/>
+      <c r="N20" s="25" t="s">
+        <v>51</v>
+      </c>
       <c r="O20" s="25"/>
       <c r="P20" s="25"/>
       <c r="Q20" s="25"/>
@@ -1762,7 +1785,9 @@
       <c r="M21" s="28">
         <v>36.0</v>
       </c>
-      <c r="N21" s="28"/>
+      <c r="N21" s="28">
+        <v>38.0</v>
+      </c>
       <c r="O21" s="28"/>
       <c r="P21" s="28"/>
       <c r="Q21" s="28"/>
@@ -1962,7 +1987,9 @@
       <c r="N5" s="15">
         <v>33.0</v>
       </c>
-      <c r="O5" s="17"/>
+      <c r="O5" s="14">
+        <v>32.0</v>
+      </c>
       <c r="P5" s="15"/>
       <c r="Q5" s="14"/>
       <c r="R5" s="15"/>
@@ -1976,7 +2003,7 @@
       <c r="Z5" s="20"/>
       <c r="AA5" s="16">
         <f t="shared" ref="AA5:AA25" si="1">SUM(C5:Z5)</f>
-        <v>173</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6">
@@ -2064,7 +2091,9 @@
       <c r="N7" s="15">
         <v>36.0</v>
       </c>
-      <c r="O7" s="17"/>
+      <c r="O7" s="14">
+        <v>36.0</v>
+      </c>
       <c r="P7" s="15"/>
       <c r="Q7" s="14"/>
       <c r="R7" s="15"/>
@@ -2078,7 +2107,7 @@
       <c r="Z7" s="18"/>
       <c r="AA7" s="16">
         <f t="shared" si="1"/>
-        <v>349</v>
+        <v>385</v>
       </c>
     </row>
     <row r="8">
@@ -2115,7 +2144,9 @@
         <v>39.0</v>
       </c>
       <c r="N8" s="15"/>
-      <c r="O8" s="14"/>
+      <c r="O8" s="14">
+        <v>36.0</v>
+      </c>
       <c r="P8" s="15"/>
       <c r="Q8" s="14"/>
       <c r="R8" s="15"/>
@@ -2129,7 +2160,7 @@
       <c r="Z8" s="18"/>
       <c r="AA8" s="16">
         <f t="shared" si="1"/>
-        <v>282</v>
+        <v>318</v>
       </c>
     </row>
     <row r="9">
@@ -2162,7 +2193,9 @@
       <c r="N9" s="15">
         <v>29.0</v>
       </c>
-      <c r="O9" s="14"/>
+      <c r="O9" s="14">
+        <v>38.0</v>
+      </c>
       <c r="P9" s="16"/>
       <c r="Q9" s="17"/>
       <c r="R9" s="16"/>
@@ -2176,7 +2209,7 @@
       <c r="Z9" s="18"/>
       <c r="AA9" s="16">
         <f t="shared" si="1"/>
-        <v>205</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10">
@@ -2205,7 +2238,9 @@
       <c r="N10" s="15">
         <v>35.0</v>
       </c>
-      <c r="O10" s="14"/>
+      <c r="O10" s="14">
+        <v>21.0</v>
+      </c>
       <c r="P10" s="16"/>
       <c r="Q10" s="14"/>
       <c r="R10" s="15"/>
@@ -2219,7 +2254,7 @@
       <c r="Z10" s="20"/>
       <c r="AA10" s="16">
         <f t="shared" si="1"/>
-        <v>155</v>
+        <v>176</v>
       </c>
     </row>
     <row r="11">
@@ -2258,7 +2293,9 @@
       <c r="N11" s="15">
         <v>39.0</v>
       </c>
-      <c r="O11" s="14"/>
+      <c r="O11" s="14">
+        <v>28.0</v>
+      </c>
       <c r="P11" s="15"/>
       <c r="Q11" s="14"/>
       <c r="R11" s="15"/>
@@ -2272,7 +2309,7 @@
       <c r="Z11" s="18"/>
       <c r="AA11" s="16">
         <f t="shared" si="1"/>
-        <v>325</v>
+        <v>353</v>
       </c>
     </row>
     <row r="12">
@@ -2344,7 +2381,9 @@
       <c r="N13" s="15">
         <v>30.0</v>
       </c>
-      <c r="O13" s="14"/>
+      <c r="O13" s="14">
+        <v>33.0</v>
+      </c>
       <c r="P13" s="15"/>
       <c r="Q13" s="14"/>
       <c r="R13" s="15"/>
@@ -2358,7 +2397,7 @@
       <c r="Z13" s="18"/>
       <c r="AA13" s="16">
         <f t="shared" si="1"/>
-        <v>215</v>
+        <v>248</v>
       </c>
     </row>
     <row r="14">
@@ -2446,7 +2485,9 @@
       <c r="N15" s="15">
         <v>38.0</v>
       </c>
-      <c r="O15" s="14"/>
+      <c r="O15" s="14">
+        <v>33.0</v>
+      </c>
       <c r="P15" s="15"/>
       <c r="Q15" s="14"/>
       <c r="R15" s="15"/>
@@ -2460,7 +2501,7 @@
       <c r="Z15" s="18"/>
       <c r="AA15" s="16">
         <f t="shared" si="1"/>
-        <v>273</v>
+        <v>306</v>
       </c>
     </row>
     <row r="16">
@@ -2499,7 +2540,9 @@
       <c r="N16" s="15">
         <v>32.0</v>
       </c>
-      <c r="O16" s="14"/>
+      <c r="O16" s="14">
+        <v>31.0</v>
+      </c>
       <c r="P16" s="16"/>
       <c r="Q16" s="14"/>
       <c r="R16" s="15"/>
@@ -2513,7 +2556,7 @@
       <c r="Z16" s="18"/>
       <c r="AA16" s="16">
         <f t="shared" si="1"/>
-        <v>231</v>
+        <v>262</v>
       </c>
     </row>
     <row r="17">
@@ -2550,7 +2593,9 @@
       <c r="N17" s="15">
         <v>37.0</v>
       </c>
-      <c r="O17" s="14"/>
+      <c r="O17" s="14">
+        <v>35.0</v>
+      </c>
       <c r="P17" s="15"/>
       <c r="Q17" s="14"/>
       <c r="R17" s="16"/>
@@ -2564,7 +2609,7 @@
       <c r="Z17" s="18"/>
       <c r="AA17" s="16">
         <f t="shared" si="1"/>
-        <v>305</v>
+        <v>340</v>
       </c>
     </row>
     <row r="18">
@@ -2599,7 +2644,9 @@
       <c r="N18" s="15">
         <v>31.0</v>
       </c>
-      <c r="O18" s="17"/>
+      <c r="O18" s="14">
+        <v>35.0</v>
+      </c>
       <c r="P18" s="16"/>
       <c r="Q18" s="14"/>
       <c r="R18" s="15"/>
@@ -2613,7 +2660,7 @@
       <c r="Z18" s="18"/>
       <c r="AA18" s="16">
         <f t="shared" si="1"/>
-        <v>251</v>
+        <v>286</v>
       </c>
     </row>
     <row r="19">
@@ -2648,7 +2695,9 @@
       <c r="L19" s="15"/>
       <c r="M19" s="14"/>
       <c r="N19" s="15"/>
-      <c r="O19" s="14"/>
+      <c r="O19" s="14">
+        <v>34.0</v>
+      </c>
       <c r="P19" s="16"/>
       <c r="Q19" s="14"/>
       <c r="R19" s="15"/>
@@ -2662,7 +2711,7 @@
       <c r="Z19" s="18"/>
       <c r="AA19" s="16">
         <f t="shared" si="1"/>
-        <v>256</v>
+        <v>290</v>
       </c>
     </row>
     <row r="20">
@@ -2746,7 +2795,9 @@
       <c r="N21" s="15">
         <v>32.0</v>
       </c>
-      <c r="O21" s="14"/>
+      <c r="O21" s="14">
+        <v>31.0</v>
+      </c>
       <c r="P21" s="16"/>
       <c r="Q21" s="14"/>
       <c r="R21" s="15"/>
@@ -2760,7 +2811,7 @@
       <c r="Z21" s="18"/>
       <c r="AA21" s="16">
         <f t="shared" si="1"/>
-        <v>355</v>
+        <v>386</v>
       </c>
     </row>
     <row r="22">
@@ -2789,7 +2840,9 @@
         <v>32.0</v>
       </c>
       <c r="N22" s="15"/>
-      <c r="O22" s="14"/>
+      <c r="O22" s="14">
+        <v>31.0</v>
+      </c>
       <c r="P22" s="16"/>
       <c r="Q22" s="14"/>
       <c r="R22" s="15"/>
@@ -2803,7 +2856,7 @@
       <c r="Z22" s="18"/>
       <c r="AA22" s="16">
         <f t="shared" si="1"/>
-        <v>179</v>
+        <v>210</v>
       </c>
     </row>
     <row r="23">
@@ -2830,7 +2883,9 @@
       </c>
       <c r="M23" s="14"/>
       <c r="N23" s="15"/>
-      <c r="O23" s="14"/>
+      <c r="O23" s="14">
+        <v>24.0</v>
+      </c>
       <c r="P23" s="16"/>
       <c r="Q23" s="14"/>
       <c r="R23" s="15"/>
@@ -2844,7 +2899,7 @@
       <c r="Z23" s="18"/>
       <c r="AA23" s="16">
         <f t="shared" si="1"/>
-        <v>86</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24">
@@ -2932,7 +2987,9 @@
         <v>40.0</v>
       </c>
       <c r="N25" s="15"/>
-      <c r="O25" s="14"/>
+      <c r="O25" s="14">
+        <v>42.0</v>
+      </c>
       <c r="P25" s="16"/>
       <c r="Q25" s="14"/>
       <c r="R25" s="15"/>
@@ -2946,7 +3003,7 @@
       <c r="Z25" s="18"/>
       <c r="AA25" s="16">
         <f t="shared" si="1"/>
-        <v>275</v>
+        <v>317</v>
       </c>
     </row>
     <row r="26" ht="9.0" customHeight="1">
@@ -3015,7 +3072,9 @@
       <c r="N27" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="O27" s="25"/>
+      <c r="O27" s="25" t="s">
+        <v>73</v>
+      </c>
       <c r="P27" s="25"/>
       <c r="Q27" s="25"/>
       <c r="R27" s="25"/>
@@ -3069,7 +3128,9 @@
       <c r="N28" s="28">
         <v>39.0</v>
       </c>
-      <c r="O28" s="28"/>
+      <c r="O28" s="28">
+        <v>42.0</v>
+      </c>
       <c r="P28" s="28"/>
       <c r="Q28" s="28"/>
       <c r="R28" s="28"/>
@@ -3116,7 +3177,7 @@
         <v>47</v>
       </c>
       <c r="B2" s="34">
-        <v>19.0</v>
+        <v>20.0</v>
       </c>
       <c r="C2" s="35">
         <v>18.0</v>
@@ -3127,7 +3188,7 @@
         <v>35</v>
       </c>
       <c r="B3" s="34">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
       <c r="C3" s="35">
         <v>13.0</v>
@@ -3152,7 +3213,7 @@
         <v>11.0</v>
       </c>
       <c r="C5" s="35">
-        <v>9.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="6">
@@ -3163,7 +3224,7 @@
         <v>16.0</v>
       </c>
       <c r="C6" s="35">
-        <v>15.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="7">
@@ -3174,7 +3235,7 @@
         <v>23.0</v>
       </c>
       <c r="C7" s="35">
-        <v>22.0</v>
+        <v>21.0</v>
       </c>
     </row>
     <row r="8">
@@ -3185,7 +3246,7 @@
         <v>32.0</v>
       </c>
       <c r="C8" s="35">
-        <v>31.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="9">
@@ -3248,10 +3309,10 @@
         <v>65</v>
       </c>
       <c r="B14" s="34">
-        <v>20.0</v>
+        <v>19.0</v>
       </c>
       <c r="C14" s="35">
-        <v>19.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="15">
@@ -3303,7 +3364,7 @@
         <v>44</v>
       </c>
       <c r="B19" s="34">
-        <v>32.0</v>
+        <v>31.0</v>
       </c>
       <c r="C19" s="35">
         <v>30.0</v>
@@ -3314,7 +3375,7 @@
         <v>40</v>
       </c>
       <c r="B20" s="34">
-        <v>16.0</v>
+        <v>15.0</v>
       </c>
       <c r="C20" s="35">
         <v>14.0</v>
@@ -3328,7 +3389,7 @@
         <v>7.0</v>
       </c>
       <c r="C21" s="35">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="22">
@@ -3358,10 +3419,10 @@
         <v>73</v>
       </c>
       <c r="B24" s="34">
+        <v>26.0</v>
+      </c>
+      <c r="C24" s="35">
         <v>27.0</v>
-      </c>
-      <c r="C24" s="35">
-        <v>28.0</v>
       </c>
     </row>
     <row r="25">
@@ -3369,7 +3430,7 @@
         <v>70</v>
       </c>
       <c r="B25" s="34">
-        <v>19.0</v>
+        <v>20.0</v>
       </c>
       <c r="C25" s="35">
         <v>18.0</v>
@@ -3383,7 +3444,7 @@
         <v>13.0</v>
       </c>
       <c r="C26" s="15">
-        <v>11.0</v>
+        <v>12.0</v>
       </c>
     </row>
     <row r="27">
@@ -3402,7 +3463,7 @@
         <v>71</v>
       </c>
       <c r="B28" s="15">
-        <v>23.0</v>
+        <v>24.0</v>
       </c>
       <c r="C28" s="15">
         <v>22.0</v>
@@ -7465,13 +7526,17 @@
       <c r="B13" s="43" t="s">
         <v>95</v>
       </c>
-      <c r="C13" s="44"/>
+      <c r="C13" s="44" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="15">
         <v>13.0</v>
       </c>
-      <c r="B14" s="43"/>
+      <c r="B14" s="43" t="s">
+        <v>96</v>
+      </c>
       <c r="C14" s="44"/>
     </row>
     <row r="15">
@@ -12428,16 +12493,16 @@
         <v>82</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2">
@@ -12685,11 +12750,11 @@
       </c>
       <c r="D13" s="47" t="str">
         <f>'THURSDAY SINGLES'!N20</f>
-        <v/>
-      </c>
-      <c r="E13" s="46" t="str">
+        <v>STEW TAYLOR</v>
+      </c>
+      <c r="E13" s="46">
         <f>'THURSDAY SINGLES'!N$21</f>
-        <v/>
+        <v>38</v>
       </c>
     </row>
     <row r="14">
@@ -12698,11 +12763,11 @@
       </c>
       <c r="B14" s="46" t="str">
         <f>'SUNDAY SINGLES'!O27</f>
-        <v/>
-      </c>
-      <c r="C14" s="46" t="str">
+        <v>HELEN RIGG</v>
+      </c>
+      <c r="C14" s="46">
         <f>'SUNDAY SINGLES'!O28</f>
-        <v/>
+        <v>42</v>
       </c>
       <c r="D14" s="47" t="str">
         <f>'THURSDAY SINGLES'!O20</f>

</xml_diff>

<commit_message>
104 Week 13/14 data update
</commit_message>
<xml_diff>
--- a/data/SUMMER_GOLF_2026.xlsx
+++ b/data/SUMMER_GOLF_2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="106">
   <si>
     <t>SUMMER GOLF 2026 - THURSDAY SINGLES</t>
   </si>
@@ -42,6 +42,15 @@
   </si>
   <si>
     <t>25/06/26</t>
+  </si>
+  <si>
+    <t>16/07/26</t>
+  </si>
+  <si>
+    <t>23/07/26</t>
+  </si>
+  <si>
+    <t>30/07/26</t>
   </si>
   <si>
     <t>NAME</t>
@@ -203,6 +212,9 @@
     <t>28/06/26</t>
   </si>
   <si>
+    <t>19/07/26</t>
+  </si>
+  <si>
     <t>TONI SHIRLEY</t>
   </si>
   <si>
@@ -306,6 +318,9 @@
   </si>
   <si>
     <t>HELEN RIGG/BAZ MASON</t>
+  </si>
+  <si>
+    <t>PAUL DIXON/SIMON CALLENDER</t>
   </si>
   <si>
     <t>SUNDAY</t>
@@ -916,11 +931,21 @@
       <c r="N3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="O3" s="5"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="5"/>
+      <c r="O3" s="3">
+        <v>46060.0</v>
+      </c>
+      <c r="P3" s="6">
+        <v>46272.0</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="T3" s="4"/>
       <c r="U3" s="5"/>
       <c r="V3" s="4"/>
@@ -932,87 +957,87 @@
     </row>
     <row r="4">
       <c r="B4" s="9" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="N4" s="10" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="O4" s="10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q4" s="10" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="R4" s="10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="S4" s="10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="T4" s="10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="U4" s="10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="V4" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="W4" s="10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="X4" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Y4" s="10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="Z4" s="10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="AA4" s="12" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="13" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C5" s="14">
         <v>29.0</v>
@@ -1042,7 +1067,9 @@
       <c r="N5" s="15">
         <v>37.0</v>
       </c>
-      <c r="O5" s="14"/>
+      <c r="O5" s="14">
+        <v>34.0</v>
+      </c>
       <c r="P5" s="15"/>
       <c r="Q5" s="17"/>
       <c r="R5" s="15"/>
@@ -1056,12 +1083,12 @@
       <c r="Z5" s="18"/>
       <c r="AA5" s="16">
         <f t="shared" ref="AA5:AA18" si="1">sum(C5:Z5)</f>
-        <v>248</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="19" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C6" s="14">
         <v>34.0</v>
@@ -1095,7 +1122,9 @@
       <c r="N6" s="15">
         <v>38.0</v>
       </c>
-      <c r="O6" s="17"/>
+      <c r="O6" s="14">
+        <v>34.0</v>
+      </c>
       <c r="P6" s="15"/>
       <c r="Q6" s="14"/>
       <c r="R6" s="15"/>
@@ -1109,12 +1138,12 @@
       <c r="Z6" s="18"/>
       <c r="AA6" s="16">
         <f t="shared" si="1"/>
-        <v>312</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="19" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="15">
@@ -1142,7 +1171,9 @@
       <c r="N7" s="15">
         <v>37.0</v>
       </c>
-      <c r="O7" s="14"/>
+      <c r="O7" s="14">
+        <v>29.0</v>
+      </c>
       <c r="P7" s="15"/>
       <c r="Q7" s="14"/>
       <c r="R7" s="15"/>
@@ -1156,12 +1187,12 @@
       <c r="Z7" s="18"/>
       <c r="AA7" s="16">
         <f t="shared" si="1"/>
-        <v>227</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="19" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C8" s="14">
         <v>36.0</v>
@@ -1195,7 +1226,9 @@
       <c r="N8" s="15">
         <v>36.0</v>
       </c>
-      <c r="O8" s="14"/>
+      <c r="O8" s="14">
+        <v>33.0</v>
+      </c>
       <c r="P8" s="15"/>
       <c r="Q8" s="14"/>
       <c r="R8" s="15"/>
@@ -1209,12 +1242,12 @@
       <c r="Z8" s="20"/>
       <c r="AA8" s="16">
         <f t="shared" si="1"/>
-        <v>330</v>
+        <v>363</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="19" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C9" s="14">
         <v>30.0</v>
@@ -1246,7 +1279,9 @@
         <v>33.0</v>
       </c>
       <c r="N9" s="15"/>
-      <c r="O9" s="14"/>
+      <c r="O9" s="14">
+        <v>41.0</v>
+      </c>
       <c r="P9" s="15"/>
       <c r="Q9" s="14"/>
       <c r="R9" s="15"/>
@@ -1260,12 +1295,12 @@
       <c r="Z9" s="18"/>
       <c r="AA9" s="16">
         <f t="shared" si="1"/>
-        <v>276</v>
+        <v>317</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="19" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C10" s="14">
         <v>32.0</v>
@@ -1297,7 +1332,9 @@
       <c r="N10" s="15">
         <v>34.0</v>
       </c>
-      <c r="O10" s="17"/>
+      <c r="O10" s="14">
+        <v>23.0</v>
+      </c>
       <c r="P10" s="15"/>
       <c r="Q10" s="14"/>
       <c r="R10" s="15"/>
@@ -1311,12 +1348,12 @@
       <c r="Z10" s="18"/>
       <c r="AA10" s="16">
         <f t="shared" si="1"/>
-        <v>287</v>
+        <v>310</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="19" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C11" s="14">
         <v>39.0</v>
@@ -1342,7 +1379,9 @@
       <c r="L11" s="15"/>
       <c r="M11" s="17"/>
       <c r="N11" s="16"/>
-      <c r="O11" s="14"/>
+      <c r="O11" s="14">
+        <v>38.0</v>
+      </c>
       <c r="P11" s="16"/>
       <c r="Q11" s="14"/>
       <c r="R11" s="15"/>
@@ -1356,12 +1395,12 @@
       <c r="Z11" s="18"/>
       <c r="AA11" s="16">
         <f t="shared" si="1"/>
-        <v>196</v>
+        <v>234</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="19" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="15"/>
@@ -1389,7 +1428,9 @@
       <c r="N12" s="15">
         <v>37.0</v>
       </c>
-      <c r="O12" s="14"/>
+      <c r="O12" s="14">
+        <v>32.0</v>
+      </c>
       <c r="P12" s="15"/>
       <c r="Q12" s="14"/>
       <c r="R12" s="15"/>
@@ -1403,12 +1444,12 @@
       <c r="Z12" s="18"/>
       <c r="AA12" s="16">
         <f t="shared" si="1"/>
-        <v>218</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="19" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C13" s="14">
         <v>28.0</v>
@@ -1459,7 +1500,7 @@
     </row>
     <row r="14">
       <c r="B14" s="19" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C14" s="14">
         <v>30.0</v>
@@ -1489,7 +1530,9 @@
       <c r="N14" s="15">
         <v>36.0</v>
       </c>
-      <c r="O14" s="14"/>
+      <c r="O14" s="14">
+        <v>30.0</v>
+      </c>
       <c r="P14" s="15"/>
       <c r="Q14" s="14"/>
       <c r="R14" s="15"/>
@@ -1503,12 +1546,12 @@
       <c r="Z14" s="18"/>
       <c r="AA14" s="16">
         <f t="shared" si="1"/>
-        <v>244</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="19" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="15">
@@ -1551,7 +1594,7 @@
     </row>
     <row r="16">
       <c r="B16" s="21" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C16" s="18"/>
       <c r="D16" s="15"/>
@@ -1573,7 +1616,9 @@
       <c r="N16" s="15">
         <v>32.0</v>
       </c>
-      <c r="O16" s="14"/>
+      <c r="O16" s="14">
+        <v>26.0</v>
+      </c>
       <c r="P16" s="15"/>
       <c r="Q16" s="14"/>
       <c r="R16" s="15"/>
@@ -1587,12 +1632,12 @@
       <c r="Z16" s="18"/>
       <c r="AA16" s="16">
         <f t="shared" si="1"/>
-        <v>110</v>
+        <v>136</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="21" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C17" s="18">
         <v>23.0</v>
@@ -1622,7 +1667,9 @@
         <v>29.0</v>
       </c>
       <c r="N17" s="16"/>
-      <c r="O17" s="14"/>
+      <c r="O17" s="14">
+        <v>25.0</v>
+      </c>
       <c r="P17" s="15"/>
       <c r="Q17" s="14"/>
       <c r="R17" s="15"/>
@@ -1636,12 +1683,12 @@
       <c r="Z17" s="18"/>
       <c r="AA17" s="16">
         <f t="shared" si="1"/>
-        <v>206</v>
+        <v>231</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="21" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C18" s="18"/>
       <c r="D18" s="15"/>
@@ -1704,41 +1751,43 @@
     </row>
     <row r="20" ht="72.0" customHeight="1">
       <c r="B20" s="24" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C20" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="E20" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="G20" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="H20" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="I20" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="E20" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="F20" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="G20" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="H20" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="I20" s="25" t="s">
-        <v>38</v>
-      </c>
       <c r="J20" s="25" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="K20" s="25"/>
       <c r="L20" s="25"/>
       <c r="M20" s="25" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="N20" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="O20" s="25"/>
+        <v>54</v>
+      </c>
+      <c r="O20" s="25" t="s">
+        <v>42</v>
+      </c>
       <c r="P20" s="25"/>
       <c r="Q20" s="25"/>
       <c r="R20" s="25"/>
@@ -1754,7 +1803,7 @@
     </row>
     <row r="21">
       <c r="B21" s="27" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C21" s="28">
         <v>39.0</v>
@@ -1788,7 +1837,9 @@
       <c r="N21" s="28">
         <v>38.0</v>
       </c>
-      <c r="O21" s="28"/>
+      <c r="O21" s="28">
+        <v>41.0</v>
+      </c>
       <c r="P21" s="28"/>
       <c r="Q21" s="28"/>
       <c r="R21" s="28"/>
@@ -1821,7 +1872,7 @@
   <sheetData>
     <row r="2" ht="24.0" customHeight="1">
       <c r="B2" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
@@ -1834,10 +1885,10 @@
         <v>46360.0</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G3" s="3">
         <v>46086.0</v>
@@ -1846,29 +1897,35 @@
         <v>46300.0</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="L3" s="6">
         <v>46209.0</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="4"/>
+        <v>64</v>
+      </c>
+      <c r="P3" s="6">
+        <v>46149.0</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>46363.0</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="S3" s="5"/>
       <c r="T3" s="4"/>
       <c r="U3" s="5"/>
@@ -1881,87 +1938,87 @@
     </row>
     <row r="4">
       <c r="B4" s="9" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="N4" s="10" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="O4" s="10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="Q4" s="10" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="R4" s="10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="S4" s="10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="T4" s="10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="U4" s="10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="V4" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="W4" s="10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="X4" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Y4" s="10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="Z4" s="10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="AA4" s="12" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="13" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C5" s="14">
         <v>24.0</v>
@@ -1990,7 +2047,9 @@
       <c r="O5" s="14">
         <v>32.0</v>
       </c>
-      <c r="P5" s="15"/>
+      <c r="P5" s="15">
+        <v>33.0</v>
+      </c>
       <c r="Q5" s="14"/>
       <c r="R5" s="15"/>
       <c r="S5" s="14"/>
@@ -2003,12 +2062,12 @@
       <c r="Z5" s="20"/>
       <c r="AA5" s="16">
         <f t="shared" ref="AA5:AA25" si="1">SUM(C5:Z5)</f>
-        <v>205</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C6" s="14">
         <v>28.0</v>
@@ -2037,7 +2096,9 @@
         <v>29.0</v>
       </c>
       <c r="O6" s="14"/>
-      <c r="P6" s="16"/>
+      <c r="P6" s="15">
+        <v>37.0</v>
+      </c>
       <c r="Q6" s="17"/>
       <c r="R6" s="15"/>
       <c r="S6" s="14"/>
@@ -2050,12 +2111,12 @@
       <c r="Z6" s="18"/>
       <c r="AA6" s="16">
         <f t="shared" si="1"/>
-        <v>215</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="19" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C7" s="14">
         <v>24.0</v>
@@ -2094,7 +2155,9 @@
       <c r="O7" s="14">
         <v>36.0</v>
       </c>
-      <c r="P7" s="15"/>
+      <c r="P7" s="15">
+        <v>36.0</v>
+      </c>
       <c r="Q7" s="14"/>
       <c r="R7" s="15"/>
       <c r="S7" s="14"/>
@@ -2107,12 +2170,12 @@
       <c r="Z7" s="18"/>
       <c r="AA7" s="16">
         <f t="shared" si="1"/>
-        <v>385</v>
+        <v>421</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="19" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C8" s="14">
         <v>24.0</v>
@@ -2165,7 +2228,7 @@
     </row>
     <row r="9">
       <c r="B9" s="19" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C9" s="14">
         <v>24.0</v>
@@ -2196,7 +2259,9 @@
       <c r="O9" s="14">
         <v>38.0</v>
       </c>
-      <c r="P9" s="16"/>
+      <c r="P9" s="15">
+        <v>27.0</v>
+      </c>
       <c r="Q9" s="17"/>
       <c r="R9" s="16"/>
       <c r="S9" s="17"/>
@@ -2209,12 +2274,12 @@
       <c r="Z9" s="18"/>
       <c r="AA9" s="16">
         <f t="shared" si="1"/>
-        <v>243</v>
+        <v>270</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="19" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C10" s="17"/>
       <c r="D10" s="15"/>
@@ -2241,7 +2306,9 @@
       <c r="O10" s="14">
         <v>21.0</v>
       </c>
-      <c r="P10" s="16"/>
+      <c r="P10" s="15">
+        <v>32.0</v>
+      </c>
       <c r="Q10" s="14"/>
       <c r="R10" s="15"/>
       <c r="S10" s="17"/>
@@ -2254,12 +2321,12 @@
       <c r="Z10" s="20"/>
       <c r="AA10" s="16">
         <f t="shared" si="1"/>
-        <v>176</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="19" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="15">
@@ -2296,7 +2363,9 @@
       <c r="O11" s="14">
         <v>28.0</v>
       </c>
-      <c r="P11" s="15"/>
+      <c r="P11" s="15">
+        <v>34.0</v>
+      </c>
       <c r="Q11" s="14"/>
       <c r="R11" s="15"/>
       <c r="S11" s="17"/>
@@ -2309,12 +2378,12 @@
       <c r="Z11" s="18"/>
       <c r="AA11" s="16">
         <f t="shared" si="1"/>
-        <v>353</v>
+        <v>387</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="19" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C12" s="14">
         <v>31.0</v>
@@ -2353,7 +2422,7 @@
     </row>
     <row r="13">
       <c r="B13" s="19" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C13" s="14">
         <v>28.0</v>
@@ -2384,7 +2453,9 @@
       <c r="O13" s="14">
         <v>33.0</v>
       </c>
-      <c r="P13" s="15"/>
+      <c r="P13" s="15">
+        <v>35.0</v>
+      </c>
       <c r="Q13" s="14"/>
       <c r="R13" s="15"/>
       <c r="S13" s="17"/>
@@ -2397,12 +2468,12 @@
       <c r="Z13" s="18"/>
       <c r="AA13" s="16">
         <f t="shared" si="1"/>
-        <v>248</v>
+        <v>283</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="19" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C14" s="14">
         <v>23.0</v>
@@ -2435,7 +2506,9 @@
         <v>34.0</v>
       </c>
       <c r="O14" s="17"/>
-      <c r="P14" s="16"/>
+      <c r="P14" s="15">
+        <v>32.0</v>
+      </c>
       <c r="Q14" s="14"/>
       <c r="R14" s="15"/>
       <c r="S14" s="14"/>
@@ -2448,12 +2521,12 @@
       <c r="Z14" s="18"/>
       <c r="AA14" s="16">
         <f t="shared" si="1"/>
-        <v>274</v>
+        <v>306</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="19" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="15">
@@ -2488,7 +2561,9 @@
       <c r="O15" s="14">
         <v>33.0</v>
       </c>
-      <c r="P15" s="15"/>
+      <c r="P15" s="15">
+        <v>30.0</v>
+      </c>
       <c r="Q15" s="14"/>
       <c r="R15" s="15"/>
       <c r="S15" s="14"/>
@@ -2501,12 +2576,12 @@
       <c r="Z15" s="18"/>
       <c r="AA15" s="16">
         <f t="shared" si="1"/>
-        <v>306</v>
+        <v>336</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="19" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C16" s="14">
         <v>20.0</v>
@@ -2543,7 +2618,9 @@
       <c r="O16" s="14">
         <v>31.0</v>
       </c>
-      <c r="P16" s="16"/>
+      <c r="P16" s="15">
+        <v>22.0</v>
+      </c>
       <c r="Q16" s="14"/>
       <c r="R16" s="15"/>
       <c r="S16" s="14"/>
@@ -2556,12 +2633,12 @@
       <c r="Z16" s="18"/>
       <c r="AA16" s="16">
         <f t="shared" si="1"/>
-        <v>262</v>
+        <v>284</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="19" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C17" s="14">
         <v>32.0</v>
@@ -2596,7 +2673,9 @@
       <c r="O17" s="14">
         <v>35.0</v>
       </c>
-      <c r="P17" s="15"/>
+      <c r="P17" s="15">
+        <v>33.0</v>
+      </c>
       <c r="Q17" s="14"/>
       <c r="R17" s="16"/>
       <c r="S17" s="17"/>
@@ -2609,12 +2688,12 @@
       <c r="Z17" s="18"/>
       <c r="AA17" s="16">
         <f t="shared" si="1"/>
-        <v>340</v>
+        <v>373</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="19" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C18" s="14">
         <v>30.0</v>
@@ -2647,7 +2726,9 @@
       <c r="O18" s="14">
         <v>35.0</v>
       </c>
-      <c r="P18" s="16"/>
+      <c r="P18" s="15">
+        <v>36.0</v>
+      </c>
       <c r="Q18" s="14"/>
       <c r="R18" s="15"/>
       <c r="S18" s="14"/>
@@ -2660,12 +2741,12 @@
       <c r="Z18" s="18"/>
       <c r="AA18" s="16">
         <f t="shared" si="1"/>
-        <v>286</v>
+        <v>322</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="19" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C19" s="14">
         <v>28.0</v>
@@ -2716,7 +2797,7 @@
     </row>
     <row r="20">
       <c r="B20" s="19" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C20" s="14"/>
       <c r="D20" s="15"/>
@@ -2757,7 +2838,7 @@
     </row>
     <row r="21">
       <c r="B21" s="19" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C21" s="14">
         <v>20.0</v>
@@ -2798,7 +2879,9 @@
       <c r="O21" s="14">
         <v>31.0</v>
       </c>
-      <c r="P21" s="16"/>
+      <c r="P21" s="15">
+        <v>31.0</v>
+      </c>
       <c r="Q21" s="14"/>
       <c r="R21" s="15"/>
       <c r="S21" s="14"/>
@@ -2811,12 +2894,12 @@
       <c r="Z21" s="18"/>
       <c r="AA21" s="16">
         <f t="shared" si="1"/>
-        <v>386</v>
+        <v>417</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="19" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="15"/>
@@ -2843,7 +2926,9 @@
       <c r="O22" s="14">
         <v>31.0</v>
       </c>
-      <c r="P22" s="16"/>
+      <c r="P22" s="15">
+        <v>33.0</v>
+      </c>
       <c r="Q22" s="14"/>
       <c r="R22" s="15"/>
       <c r="S22" s="14"/>
@@ -2856,12 +2941,12 @@
       <c r="Z22" s="18"/>
       <c r="AA22" s="16">
         <f t="shared" si="1"/>
-        <v>210</v>
+        <v>243</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="19" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C23" s="14"/>
       <c r="D23" s="15">
@@ -2886,7 +2971,9 @@
       <c r="O23" s="14">
         <v>24.0</v>
       </c>
-      <c r="P23" s="16"/>
+      <c r="P23" s="15">
+        <v>22.0</v>
+      </c>
       <c r="Q23" s="14"/>
       <c r="R23" s="15"/>
       <c r="S23" s="14"/>
@@ -2899,12 +2986,12 @@
       <c r="Z23" s="18"/>
       <c r="AA23" s="16">
         <f t="shared" si="1"/>
-        <v>110</v>
+        <v>132</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="19" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C24" s="14">
         <v>35.0</v>
@@ -2955,7 +3042,7 @@
     </row>
     <row r="25">
       <c r="B25" s="19" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C25" s="14">
         <v>19.0</v>
@@ -2990,7 +3077,9 @@
       <c r="O25" s="14">
         <v>42.0</v>
       </c>
-      <c r="P25" s="16"/>
+      <c r="P25" s="15">
+        <v>38.0</v>
+      </c>
       <c r="Q25" s="14"/>
       <c r="R25" s="15"/>
       <c r="S25" s="14"/>
@@ -3003,7 +3092,7 @@
       <c r="Z25" s="18"/>
       <c r="AA25" s="16">
         <f t="shared" si="1"/>
-        <v>317</v>
+        <v>355</v>
       </c>
     </row>
     <row r="26" ht="9.0" customHeight="1">
@@ -3034,48 +3123,50 @@
     </row>
     <row r="27" ht="84.75" customHeight="1">
       <c r="B27" s="24" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E27" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="F27" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="G27" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="H27" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="I27" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="J27" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="F27" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="G27" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="H27" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="I27" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="J27" s="25" t="s">
-        <v>36</v>
-      </c>
       <c r="K27" s="25" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L27" s="25" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="M27" s="25" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="N27" s="25" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="O27" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="P27" s="25"/>
+        <v>77</v>
+      </c>
+      <c r="P27" s="25" t="s">
+        <v>77</v>
+      </c>
       <c r="Q27" s="25"/>
       <c r="R27" s="25"/>
       <c r="S27" s="25"/>
@@ -3090,7 +3181,7 @@
     </row>
     <row r="28">
       <c r="B28" s="27" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C28" s="28">
         <v>35.0</v>
@@ -3131,7 +3222,9 @@
       <c r="O28" s="28">
         <v>42.0</v>
       </c>
-      <c r="P28" s="28"/>
+      <c r="P28" s="28">
+        <v>38.0</v>
+      </c>
       <c r="Q28" s="28"/>
       <c r="R28" s="28"/>
       <c r="S28" s="28"/>
@@ -3163,18 +3256,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="30" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B1" s="31" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C1" s="32" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="33" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B2" s="34">
         <v>20.0</v>
@@ -3185,7 +3278,7 @@
     </row>
     <row r="3">
       <c r="A3" s="19" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B3" s="34">
         <v>14.0</v>
@@ -3196,7 +3289,7 @@
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B4" s="34">
         <v>10.0</v>
@@ -3207,7 +3300,7 @@
     </row>
     <row r="5">
       <c r="A5" s="19" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B5" s="34">
         <v>11.0</v>
@@ -3218,7 +3311,7 @@
     </row>
     <row r="6">
       <c r="A6" s="19" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B6" s="34">
         <v>16.0</v>
@@ -3229,7 +3322,7 @@
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B7" s="34">
         <v>23.0</v>
@@ -3240,7 +3333,7 @@
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B8" s="34">
         <v>32.0</v>
@@ -3251,7 +3344,7 @@
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B9" s="34">
         <v>9.0</v>
@@ -3262,7 +3355,7 @@
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B10" s="34">
         <v>16.0</v>
@@ -3273,7 +3366,7 @@
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B11" s="34">
         <v>23.0</v>
@@ -3284,7 +3377,7 @@
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B12" s="34">
         <v>10.0</v>
@@ -3295,7 +3388,7 @@
     </row>
     <row r="13">
       <c r="A13" s="19" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B13" s="34">
         <v>12.0</v>
@@ -3306,7 +3399,7 @@
     </row>
     <row r="14">
       <c r="A14" s="19" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B14" s="34">
         <v>19.0</v>
@@ -3317,7 +3410,7 @@
     </row>
     <row r="15">
       <c r="A15" s="19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B15" s="34">
         <v>7.0</v>
@@ -3328,7 +3421,7 @@
     </row>
     <row r="16">
       <c r="A16" s="19" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B16" s="34">
         <v>15.0</v>
@@ -3339,7 +3432,7 @@
     </row>
     <row r="17">
       <c r="A17" s="19" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B17" s="34">
         <v>13.0</v>
@@ -3350,7 +3443,7 @@
     </row>
     <row r="18">
       <c r="A18" s="19" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B18" s="34">
         <v>0.0</v>
@@ -3361,7 +3454,7 @@
     </row>
     <row r="19">
       <c r="A19" s="19" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B19" s="34">
         <v>31.0</v>
@@ -3372,7 +3465,7 @@
     </row>
     <row r="20">
       <c r="A20" s="37" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B20" s="34">
         <v>15.0</v>
@@ -3383,7 +3476,7 @@
     </row>
     <row r="21">
       <c r="A21" s="19" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B21" s="34">
         <v>7.0</v>
@@ -3394,7 +3487,7 @@
     </row>
     <row r="22">
       <c r="A22" s="19" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B22" s="34">
         <v>21.0</v>
@@ -3405,7 +3498,7 @@
     </row>
     <row r="23">
       <c r="A23" s="19" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B23" s="34">
         <v>33.0</v>
@@ -3416,7 +3509,7 @@
     </row>
     <row r="24">
       <c r="A24" s="37" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B24" s="34">
         <v>26.0</v>
@@ -3427,7 +3520,7 @@
     </row>
     <row r="25">
       <c r="A25" s="37" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B25" s="34">
         <v>20.0</v>
@@ -3438,7 +3531,7 @@
     </row>
     <row r="26">
       <c r="A26" s="37" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B26" s="15">
         <v>13.0</v>
@@ -3449,7 +3542,7 @@
     </row>
     <row r="27">
       <c r="A27" s="37" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B27" s="15">
         <v>15.0</v>
@@ -3460,7 +3553,7 @@
     </row>
     <row r="28">
       <c r="A28" s="37" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B28" s="15">
         <v>24.0</v>
@@ -3471,7 +3564,7 @@
     </row>
     <row r="29">
       <c r="A29" s="37" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B29" s="15">
         <v>23.0</v>
@@ -3482,7 +3575,7 @@
     </row>
     <row r="30">
       <c r="A30" s="37" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B30" s="15">
         <v>23.0</v>
@@ -3493,7 +3586,7 @@
     </row>
     <row r="31">
       <c r="A31" s="37" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B31" s="15">
         <v>20.0</v>
@@ -3504,7 +3597,7 @@
     </row>
     <row r="32">
       <c r="A32" s="37" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B32" s="15">
         <v>7.0</v>
@@ -7388,13 +7481,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B1" s="38" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C1" s="39" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2">
@@ -7402,10 +7495,10 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="41" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C2" s="42" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -7413,10 +7506,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" s="43" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C3" s="44" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4">
@@ -7424,10 +7517,10 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="43" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5">
@@ -7435,10 +7528,10 @@
         <v>4.0</v>
       </c>
       <c r="B5" s="43" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C5" s="44" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6">
@@ -7446,10 +7539,10 @@
         <v>5.0</v>
       </c>
       <c r="B6" s="43" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C6" s="44" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7">
@@ -7457,10 +7550,10 @@
         <v>6.0</v>
       </c>
       <c r="B7" s="43" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C7" s="44" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8">
@@ -7468,10 +7561,10 @@
         <v>7.0</v>
       </c>
       <c r="B8" s="43" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C8" s="44" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9">
@@ -7479,10 +7572,10 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="43" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C9" s="44" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10">
@@ -7490,10 +7583,10 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="43" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C10" s="44" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="G10" s="16"/>
     </row>
@@ -7502,10 +7595,10 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="43" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C11" s="44" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12">
@@ -7513,10 +7606,10 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="43" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C12" s="44" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13">
@@ -7524,10 +7617,10 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="43" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C13" s="44" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14">
@@ -7535,15 +7628,19 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="43" t="s">
-        <v>96</v>
-      </c>
-      <c r="C14" s="44"/>
+        <v>100</v>
+      </c>
+      <c r="C14" s="44" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="15">
         <v>14.0</v>
       </c>
-      <c r="B15" s="43"/>
+      <c r="B15" s="43" t="s">
+        <v>101</v>
+      </c>
       <c r="C15" s="44"/>
     </row>
     <row r="16">
@@ -12490,19 +12587,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D1" s="45" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2">
@@ -12771,11 +12868,11 @@
       </c>
       <c r="D14" s="47" t="str">
         <f>'THURSDAY SINGLES'!O20</f>
-        <v/>
-      </c>
-      <c r="E14" s="46" t="str">
+        <v>KEN PEEL</v>
+      </c>
+      <c r="E14" s="46">
         <f>'THURSDAY SINGLES'!O21</f>
-        <v/>
+        <v>41</v>
       </c>
     </row>
     <row r="15">
@@ -12784,11 +12881,11 @@
       </c>
       <c r="B15" s="46" t="str">
         <f>'SUNDAY SINGLES'!P27</f>
-        <v/>
-      </c>
-      <c r="C15" s="46" t="str">
+        <v>HELEN RIGG</v>
+      </c>
+      <c r="C15" s="46">
         <f>'SUNDAY SINGLES'!P28</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="D15" s="47" t="str">
         <f>'THURSDAY SINGLES'!P20</f>

</xml_diff>